<commit_message>
added 5 startups and 2 DC from my notes
</commit_message>
<xml_diff>
--- a/Photonic Companies.xlsx
+++ b/Photonic Companies.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11122"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10531"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/blow/Desktop/GitHub/PhotonicCompanies/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C8A6D29-EAA1-4F41-B691-D41504F45002}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{583BC68D-E307-5342-90F3-D241A3B92D3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" xr2:uid="{EBDBD758-277E-6B49-B4C7-31ED6652B0E7}"/>
+    <workbookView xWindow="0" yWindow="620" windowWidth="28800" windowHeight="15660" activeTab="3" xr2:uid="{EBDBD758-277E-6B49-B4C7-31ED6652B0E7}"/>
   </bookViews>
   <sheets>
     <sheet name="Startup" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="625" uniqueCount="566">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="653" uniqueCount="592">
   <si>
     <t>Company Name</t>
   </si>
@@ -1756,6 +1756,85 @@
   </si>
   <si>
     <t xml:space="preserve">Jin Guo (Managing Director) </t>
+  </si>
+  <si>
+    <t>Maxwell Labs, Inc. (MXL Labs)</t>
+  </si>
+  <si>
+    <t>Jacob Balma
+(Co-Founder &amp; CEO), Alejandro Rodriguez (CTO), Mike Karpe (CRO)</t>
+  </si>
+  <si>
+    <t>Saint Paul, Minnesota, USA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Maxwell Labs is developing “photonic cooling” — a laser-/photon-based cooling technology that aims to remove heat from computer chips by converting thermal energy into light (anti-Stokes fluorescence), rather than relying on conventional air or liquid cooling. Data Centers. High Performance Computing, etc. </t>
+  </si>
+  <si>
+    <t>Hartley Ultrafast Ltd</t>
+  </si>
+  <si>
+    <t>Photonic AI inference hardware. using pulses of light plus fast electronics for ultra-low-latency AI inference. Its proof-of-concept photonic neural-network computer is called Babbage, reported to run inference in about 176 ns</t>
+  </si>
+  <si>
+    <t>Josh Silverstone (Founder and CEO)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bristol, United Kingdom </t>
+  </si>
+  <si>
+    <t>Edwatec</t>
+  </si>
+  <si>
+    <t>Erbium-doped photonic integrated circuits for on-chip optical amplification and lasing. erbium ion implantation in silicon-nitride waveguides, aiming for compact, scalable, high-performance optical gain for optical transceivers, data/telecom, AI infrastructure, fiber sensing.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Peter Ils (CEO), Dr. Amir Youssefi (CTO), EPFL Spin-Off </t>
+  </si>
+  <si>
+    <t>Lausanne, Switzerland</t>
+  </si>
+  <si>
+    <t>Photonpath</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dr. Douglas Aguiar (CEO), Emanuele Guglielmi (CTO), Spin-off from Politecnico di Milano </t>
+  </si>
+  <si>
+    <t>Integrated photonics / silicon photonics chipsets and plug-and-play modules for optical communications, AI data centers. Series A stage, with a recent €5.1M raise to scale manufacturing.</t>
+  </si>
+  <si>
+    <t>Temporal Photonics</t>
+  </si>
+  <si>
+    <t>Compact, highly accurate photonic timing / clock systems for resilient timing in GPS/GNSS-denied environments</t>
+  </si>
+  <si>
+    <t>David Marpaung, University of Twente</t>
+  </si>
+  <si>
+    <t>Rotonium</t>
+  </si>
+  <si>
+    <t>Photonic quantum edge processors / photonic quantum computing using single-photon qudits and orbital angular momentum (OAM) of photons</t>
+  </si>
+  <si>
+    <t>Roberto Siagri (CEO), Nicolò Leone (SiPh Lead)</t>
+  </si>
+  <si>
+    <t>Padova, Italy</t>
+  </si>
+  <si>
+    <t>Beacon Photonics Inc.</t>
+  </si>
+  <si>
+    <t>Heterogeneous integrated photonics / optical microsystems for commercial and national-security applications.</t>
+  </si>
+  <si>
+    <t>Gordon Keeler  ( Co-Founder and CEO), John Bowers, John Burke, UCSB</t>
+  </si>
+  <si>
+    <t>Arlington, Virginia, USA</t>
   </si>
 </sst>
 </file>
@@ -2217,7 +2296,8 @@
     <col min="1" max="1" width="10.83203125" style="1"/>
     <col min="2" max="3" width="28" style="3" customWidth="1"/>
     <col min="4" max="4" width="45.1640625" style="1" customWidth="1"/>
-    <col min="5" max="6" width="28" style="1" customWidth="1"/>
+    <col min="5" max="5" width="30.33203125" style="1" customWidth="1"/>
+    <col min="6" max="6" width="28" style="1" customWidth="1"/>
     <col min="7" max="16384" width="10.83203125" style="1"/>
   </cols>
   <sheetData>
@@ -3436,7 +3516,7 @@
       <c r="C73" s="3">
         <v>50</v>
       </c>
-      <c r="D73" s="4" t="s">
+      <c r="D73" s="1" t="s">
         <v>552</v>
       </c>
       <c r="E73" s="1" t="s">
@@ -3467,7 +3547,7 @@
       <c r="B75" s="3" t="s">
         <v>559</v>
       </c>
-      <c r="C75" s="3">
+      <c r="C75" s="1">
         <v>10</v>
       </c>
       <c r="D75" s="1" t="s">
@@ -3480,14 +3560,91 @@
         <v>558</v>
       </c>
     </row>
-    <row r="76" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B76" s="1"/>
-      <c r="C76" s="1"/>
-    </row>
-    <row r="77" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="78" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="79" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="80" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="76" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B76" s="3" t="s">
+        <v>566</v>
+      </c>
+      <c r="C76" s="1">
+        <v>10</v>
+      </c>
+      <c r="D76" s="1" t="s">
+        <v>569</v>
+      </c>
+      <c r="E76" s="1" t="s">
+        <v>567</v>
+      </c>
+      <c r="F76" s="1" t="s">
+        <v>568</v>
+      </c>
+    </row>
+    <row r="77" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B77" s="3" t="s">
+        <v>570</v>
+      </c>
+      <c r="C77" s="3">
+        <v>10</v>
+      </c>
+      <c r="D77" s="1" t="s">
+        <v>571</v>
+      </c>
+      <c r="E77" s="1" t="s">
+        <v>572</v>
+      </c>
+      <c r="F77" s="1" t="s">
+        <v>573</v>
+      </c>
+    </row>
+    <row r="78" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B78" s="3" t="s">
+        <v>574</v>
+      </c>
+      <c r="C78" s="3">
+        <v>15</v>
+      </c>
+      <c r="D78" s="1" t="s">
+        <v>575</v>
+      </c>
+      <c r="E78" s="1" t="s">
+        <v>576</v>
+      </c>
+      <c r="F78" s="1" t="s">
+        <v>577</v>
+      </c>
+    </row>
+    <row r="79" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B79" s="3" t="s">
+        <v>578</v>
+      </c>
+      <c r="C79" s="3">
+        <v>25</v>
+      </c>
+      <c r="D79" s="1" t="s">
+        <v>580</v>
+      </c>
+      <c r="E79" s="1" t="s">
+        <v>579</v>
+      </c>
+      <c r="F79" s="1" t="s">
+        <v>528</v>
+      </c>
+    </row>
+    <row r="80" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B80" s="3" t="s">
+        <v>584</v>
+      </c>
+      <c r="C80" s="3">
+        <v>10</v>
+      </c>
+      <c r="D80" s="1" t="s">
+        <v>585</v>
+      </c>
+      <c r="E80" s="1" t="s">
+        <v>586</v>
+      </c>
+      <c r="F80" s="1" t="s">
+        <v>587</v>
+      </c>
+    </row>
     <row r="81" ht="56.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="82" ht="56.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="83" ht="56.25" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -3521,7 +3678,9 @@
   <cols>
     <col min="1" max="1" width="10.83203125" style="1"/>
     <col min="2" max="3" width="28" style="3" customWidth="1"/>
-    <col min="4" max="7" width="28" style="1" customWidth="1"/>
+    <col min="4" max="4" width="28" style="1" customWidth="1"/>
+    <col min="5" max="5" width="30.5" style="1" customWidth="1"/>
+    <col min="6" max="7" width="28" style="1" customWidth="1"/>
     <col min="8" max="16384" width="10.83203125" style="1"/>
   </cols>
   <sheetData>
@@ -4078,7 +4237,9 @@
   <cols>
     <col min="1" max="1" width="10.83203125" style="1"/>
     <col min="2" max="3" width="28" style="1" customWidth="1"/>
-    <col min="4" max="6" width="28" style="7" customWidth="1"/>
+    <col min="4" max="4" width="28" style="7" customWidth="1"/>
+    <col min="5" max="5" width="30" style="7" customWidth="1"/>
+    <col min="6" max="6" width="28" style="7" customWidth="1"/>
     <col min="7" max="7" width="28" style="1" customWidth="1"/>
     <col min="8" max="16384" width="10.83203125" style="1"/>
   </cols>
@@ -4665,13 +4826,11 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{77D8C265-B588-454D-B906-8DDBB021B0D6}">
   <dimension ref="B1:F25"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="20" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="31" defaultRowHeight="20" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="10.83203125" style="1"/>
-    <col min="2" max="3" width="28" style="3" customWidth="1"/>
-    <col min="4" max="4" width="40" style="1" customWidth="1"/>
-    <col min="5" max="7" width="28" style="1" customWidth="1"/>
-    <col min="8" max="16384" width="10.83203125" style="1"/>
+    <col min="1" max="1" width="31" style="1"/>
+    <col min="2" max="3" width="31" style="3"/>
+    <col min="4" max="16384" width="31" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:6" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -4794,8 +4953,40 @@
         <v>377</v>
       </c>
     </row>
-    <row r="9" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="10" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="9" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B9" s="3" t="s">
+        <v>581</v>
+      </c>
+      <c r="C9" s="3">
+        <v>5</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>582</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>583</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="10" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B10" s="3" t="s">
+        <v>588</v>
+      </c>
+      <c r="C10" s="3">
+        <v>15</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>589</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>590</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>591</v>
+      </c>
+    </row>
     <row r="11" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="12" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="13" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25"/>

</xml_diff>

<commit_message>
added 6 start ups from search
</commit_message>
<xml_diff>
--- a/Photonic Companies.xlsx
+++ b/Photonic Companies.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/blow/Desktop/GitHub/PhotonicCompanies/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{583BC68D-E307-5342-90F3-D241A3B92D3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EBAB5315-1194-A941-9D0A-D36EE3275799}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="620" windowWidth="28800" windowHeight="15660" activeTab="3" xr2:uid="{EBDBD758-277E-6B49-B4C7-31ED6652B0E7}"/>
+    <workbookView xWindow="0" yWindow="620" windowWidth="28800" windowHeight="15660" xr2:uid="{EBDBD758-277E-6B49-B4C7-31ED6652B0E7}"/>
   </bookViews>
   <sheets>
     <sheet name="Startup" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="653" uniqueCount="592">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="677" uniqueCount="615">
   <si>
     <t>Company Name</t>
   </si>
@@ -1835,6 +1835,76 @@
   </si>
   <si>
     <t>Arlington, Virginia, USA</t>
+  </si>
+  <si>
+    <t>Oriole Networks</t>
+  </si>
+  <si>
+    <t>Photonic Routers, Integrated Photonic Switch
+and Transceiver (XTR), Training and inference at the speed of light. developing disruptive technologies for AI/ML and HPC networking that will revolutionize data centers, full photonic AI network fabric</t>
+  </si>
+  <si>
+    <t>Prof. George Zervas, Alessandro Ottino, and Joshua Benjamin, James Regan (CEO), University College London</t>
+  </si>
+  <si>
+    <t>London, United Kingdom</t>
+  </si>
+  <si>
+    <t>LightSolver Ltd.</t>
+  </si>
+  <si>
+    <t>All-optical computing / laser-based high-performance computing accelerator, free-space Photonic NN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ruti Ben-Shlomi, Ph.D (CEO), Dr. Chene Tradonski (CTO),  </t>
+  </si>
+  <si>
+    <t>Tel Aviv, Israel</t>
+  </si>
+  <si>
+    <t>LightOn</t>
+  </si>
+  <si>
+    <t>Free-Space Optical Processing Unit, OPU — a free-space photonic co-processor for large-scale random projections / non-von-Neumann AI/HPC workloads. A 2021 LightOn paper describes it as a photonic AI accelerator reaching 1,500 TeraOPS and usable alongside CPU/GPU systems through Python-based software APIs.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Paris, France </t>
+  </si>
+  <si>
+    <t>Igor Carron, Laurent Daudet, Florent Krzakala, and Sylvain Gigan, École Polytechnique</t>
+  </si>
+  <si>
+    <t>DustPhotonics Ltd.</t>
+  </si>
+  <si>
+    <t>Silicon photonics PICs / optical interconnect for AI and hyperscale data centers SiPho PIC technology for 400G, 800G, 1.6T and beyond, with Credo emphasizing a portfolio across 800G, 1.6T, and 3.2T near-packaged optics and co-packaged optics. DustPhotonics’ site also says the combined Credo/DustPhotonics portfolio spans 800G, 1.6T, and 3.2T NPO/CPO</t>
+  </si>
+  <si>
+    <t>Ronnen Lovinger (CEO), Yoel Shetrit (VP of Photonics)</t>
+  </si>
+  <si>
+    <t>Modiin, Israel</t>
+  </si>
+  <si>
+    <t>LightSpeed Photonics</t>
+  </si>
+  <si>
+    <t>Rohin Kumar Y (CEO) and Ramana V. Pamidighantam (CTO)</t>
+  </si>
+  <si>
+    <t>Singapore and Hyderabad, India</t>
+  </si>
+  <si>
+    <t>NPO, Modular “compute + interconnect” heterogeneous system-in-package / optical interconnect platform. LightSpeed says its approach integrates processors with high-speed optics so data</t>
+  </si>
+  <si>
+    <t>Enlightra</t>
+  </si>
+  <si>
+    <t>Optical interconnects, Extreme-bandwidth, low-power optical interconnects for AI data centers and computing. Chip-scale multiwavelength / multi-color lasers, often described as comb-laser technology, for optical data transmission</t>
+  </si>
+  <si>
+    <t>John Jost (CEO), EPFL</t>
   </si>
 </sst>
 </file>
@@ -3645,22 +3715,118 @@
         <v>587</v>
       </c>
     </row>
-    <row r="81" ht="56.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="82" ht="56.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="83" ht="56.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="84" ht="56.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="85" ht="56.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="86" ht="56.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="87" ht="56.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="88" ht="56.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="89" ht="56.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="90" ht="56.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="91" ht="56.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="92" ht="56.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="93" ht="56.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="94" ht="56.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="95" ht="56.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="96" ht="56.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="81" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B81" s="3" t="s">
+        <v>592</v>
+      </c>
+      <c r="C81" s="3">
+        <v>25</v>
+      </c>
+      <c r="D81" s="1" t="s">
+        <v>593</v>
+      </c>
+      <c r="E81" s="1" t="s">
+        <v>594</v>
+      </c>
+      <c r="F81" s="1" t="s">
+        <v>595</v>
+      </c>
+    </row>
+    <row r="82" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B82" s="3" t="s">
+        <v>596</v>
+      </c>
+      <c r="C82" s="3">
+        <v>30</v>
+      </c>
+      <c r="D82" s="1" t="s">
+        <v>597</v>
+      </c>
+      <c r="E82" s="1" t="s">
+        <v>598</v>
+      </c>
+      <c r="F82" s="1" t="s">
+        <v>599</v>
+      </c>
+    </row>
+    <row r="83" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B83" s="3" t="s">
+        <v>600</v>
+      </c>
+      <c r="C83" s="3">
+        <v>41</v>
+      </c>
+      <c r="D83" s="1" t="s">
+        <v>601</v>
+      </c>
+      <c r="E83" s="1" t="s">
+        <v>603</v>
+      </c>
+      <c r="F83" s="1" t="s">
+        <v>602</v>
+      </c>
+    </row>
+    <row r="84" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B84" s="3" t="s">
+        <v>604</v>
+      </c>
+      <c r="C84" s="3">
+        <v>100</v>
+      </c>
+      <c r="D84" s="1" t="s">
+        <v>605</v>
+      </c>
+      <c r="E84" s="1" t="s">
+        <v>606</v>
+      </c>
+      <c r="F84" s="1" t="s">
+        <v>607</v>
+      </c>
+    </row>
+    <row r="85" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B85" s="3" t="s">
+        <v>608</v>
+      </c>
+      <c r="C85" s="3">
+        <v>28</v>
+      </c>
+      <c r="D85" s="1" t="s">
+        <v>611</v>
+      </c>
+      <c r="E85" s="1" t="s">
+        <v>609</v>
+      </c>
+      <c r="F85" s="1" t="s">
+        <v>610</v>
+      </c>
+    </row>
+    <row r="86" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B86" s="3" t="s">
+        <v>612</v>
+      </c>
+      <c r="C86" s="3">
+        <v>25</v>
+      </c>
+      <c r="D86" s="1" t="s">
+        <v>613</v>
+      </c>
+      <c r="E86" s="4" t="s">
+        <v>614</v>
+      </c>
+      <c r="F86" s="1" t="s">
+        <v>577</v>
+      </c>
+    </row>
+    <row r="87" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="88" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="89" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="90" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="91" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="92" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="93" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="94" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="95" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="96" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="97" ht="56.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="98" ht="56.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="99" ht="56.25" customHeight="1" x14ac:dyDescent="0.25"/>

</xml_diff>

<commit_message>
added to 5 SU, 2 Foundries
</commit_message>
<xml_diff>
--- a/Photonic Companies.xlsx
+++ b/Photonic Companies.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/blow/Desktop/GitHub/PhotonicCompanies/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E039C8F7-D5EA-B342-96BE-BE6631776701}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D71614C-B2B9-0F42-B3A3-128B1EDAF3F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="620" windowWidth="28800" windowHeight="15660" xr2:uid="{EBDBD758-277E-6B49-B4C7-31ED6652B0E7}"/>
+    <workbookView xWindow="0" yWindow="620" windowWidth="28800" windowHeight="15660" activeTab="2" xr2:uid="{EBDBD758-277E-6B49-B4C7-31ED6652B0E7}"/>
   </bookViews>
   <sheets>
     <sheet name="Startup" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="681" uniqueCount="619">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="709" uniqueCount="646">
   <si>
     <t>Company Name</t>
   </si>
@@ -171,9 +171,6 @@
   </si>
   <si>
     <t>Stuttgart, Germany</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3D optical AI computing </t>
   </si>
   <si>
     <t>Oxford, England</t>
@@ -1479,9 +1476,6 @@
   </si>
   <si>
     <t>Marvell Technology</t>
-  </si>
-  <si>
-    <t>3D Silicon Photonics Engine, 1.6T Silicon Photonics Light Engine, 1.6T Silicon Photonics Light Engine</t>
   </si>
   <si>
     <t>CEO: Matt Murphy, CTO Optical Engineering: Dr. Radha Nagarajan</t>
@@ -1728,9 +1722,6 @@
     <t>Neurophos</t>
   </si>
   <si>
-    <t>optical processing units (OPUs) based on metasurface + silicon photonics — using optical modulators built from metamaterials and photonics rather than traditional electronic transistors; claim modulators 10,000x time smaller than SoTA, with 300 TOPS/W</t>
-  </si>
-  <si>
     <t>Patrick Bown (CEO), Hod Finkelstein (CTO)</t>
   </si>
   <si>
@@ -1918,13 +1909,159 @@
   <si>
     <t xml:space="preserve">Integrated photonic sensing using thin-film lithium niobate (TFLN), "Real-world AI starts with real-world data.
 We build integrated photonic sensors to make that possible." </t>
+  </si>
+  <si>
+    <t>3D optical AI computing. Lumai, a developer of optical computing for scalable AI, has launched its Lumai Iris inference server. According to the company, Iris is the first optical computing system to successfully run billion-parameter large language models (LLMs) in real time.</t>
+  </si>
+  <si>
+    <t>OpenLight</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dr. Adam Carter (CEO), </t>
+  </si>
+  <si>
+    <t>Goleta, California and Santa Clara, California</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Custom </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>PASIC</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> — Photonic Application-Specific Integrated Circuit — design and manufacturing using heterogeneous silicon photonics with integrated active/passive components, 50M raise series A</t>
+    </r>
+  </si>
+  <si>
+    <t>optical processing units (OPUs) based on metasurface + silicon photonics — using optical modulators built from metamaterials and photonics rather than traditional electronic transistors; claim modulators 10,000x time smaller than SoTA, with 300 TOPS/W, $110 million series A round</t>
+  </si>
+  <si>
+    <t>3D Silicon Photonics Engine, 1.6T Silicon Photonics Light Engine, 1.6T Silicon Photonics Light Engine, Nvidia invest 2B</t>
+  </si>
+  <si>
+    <t>Vector Photonics Limited</t>
+  </si>
+  <si>
+    <t>Developer of Photonic Crystal Surface-Emitting Lasers — PCSELs, for next-generation datacenters</t>
+  </si>
+  <si>
+    <t>Dr. Richard Taylor, CEO, Spin-out from the University of Glasgow</t>
+  </si>
+  <si>
+    <t>Glasgow, Scotland</t>
+  </si>
+  <si>
+    <t>Mesh Optical Technologies</t>
+  </si>
+  <si>
+    <t>Travis Brashears, Cameron Ramos, and Serena Grown-Haeberli, Ex-SpaceX</t>
+  </si>
+  <si>
+    <t>Los Angeles, California</t>
+  </si>
+  <si>
+    <t>Optical transceivers / optical links for AI and data-center infrastructure, optical engine uses the most reliable distributed feedback (DFB) laser ever developed for an optical transceiver</t>
+  </si>
+  <si>
+    <t>VitreaLab GmbH</t>
+  </si>
+  <si>
+    <t>Develops and manufactures photonic integrated circuit light engines / laser waveguide technology for AR smart-glasses and near-eye display components. The company describes its technology as a Quantum Light Chip for reducing coherent artifacts in AR optical engines</t>
+  </si>
+  <si>
+    <t>Dr. Ronny Timmreck (CEO), Dr. Jonas Zeuner (CTO), Spin-off from the Quantum Group at the University of Vienna</t>
+  </si>
+  <si>
+    <t>Vienna, Austria</t>
+  </si>
+  <si>
+    <t>PicoJool Inc.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Al Yuen (CEO) </t>
+  </si>
+  <si>
+    <r>
+      <t>Optical connectivity for AI and cloud data centers</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">; high-bandwidth </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>VCSELs</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, parallel optical links/modules, and pixel-level photonics aimed at replacing copper interconnects at scale. Raised $12M led by Playground Global</t>
+    </r>
+  </si>
+  <si>
+    <t>Palo Alto, California</t>
+  </si>
+  <si>
+    <t>Quantum Pulse Ventures</t>
+  </si>
+  <si>
+    <t>Ofer Shapiro (CEO), Prof. Yaron Oz, (Chief Scientist), and Prof. Haim Suchowski (Chief Architect)</t>
+  </si>
+  <si>
+    <t>Photonic quantum computing and quantum routing. QPV says its Quantum Pulse 2.0 / QP2.0 platform improves fidelity and robustness for low-loss integrated optical applications, extending beyond photonic quantum-computing components into broader photonic integrated circuits</t>
+  </si>
+  <si>
+    <t>La Luce Cristallina, Inc</t>
+  </si>
+  <si>
+    <t>Manufacturer of Si-integrated high-performance materials for silicon photonics, especially barium titanate / BaTiO₃ wafers and substrates for electro-optic modulators and photonic integrated circuits</t>
+  </si>
+  <si>
+    <t>Alex Demkov, Ph.D. (CEO), Agham Posadas, Ph.D (CTO), University of Texas at Austin</t>
+  </si>
+  <si>
+    <t>Austin, Texas</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -1956,25 +2093,30 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
       <color rgb="FF474747"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
     <font>
       <b/>
-      <sz val="16"/>
-      <color theme="1"/>
-      <name val="Aptos Narrow"/>
+      <sz val="24"/>
+      <color rgb="FF000000"/>
+      <name val="Tahoma"/>
       <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
-      <b/>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
-      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -1998,7 +2140,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -2012,32 +2154,39 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2386,10 +2535,10 @@
   <sheetData>
     <row r="1" spans="2:6" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="2" spans="2:6" s="2" customFormat="1" ht="56.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="6" t="s">
+      <c r="B2" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="C2" s="5" t="s">
         <v>1</v>
       </c>
       <c r="D2" s="2" t="s">
@@ -2399,7 +2548,7 @@
         <v>7</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="3" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -2416,7 +2565,7 @@
         <v>6</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="4" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -2433,7 +2582,7 @@
         <v>9</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="5" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -2512,81 +2661,81 @@
         <v>20</v>
       </c>
       <c r="D9" s="1" t="s">
+        <v>616</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="F9" s="1" t="s">
         <v>44</v>
-      </c>
-      <c r="E9" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="F9" s="1" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="10" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="D10" s="1" t="s">
         <v>47</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="D10" s="1" t="s">
-        <v>48</v>
       </c>
       <c r="E10" s="1" t="s">
         <v>22</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="11" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B11" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="D11" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="C11" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="D11" s="1" t="s">
-        <v>51</v>
-      </c>
       <c r="E11" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="12" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B12" s="3" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D12" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="E12" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="E12" s="1" t="s">
+      <c r="F12" s="1" t="s">
         <v>55</v>
-      </c>
-      <c r="F12" s="1" t="s">
-        <v>56</v>
       </c>
     </row>
     <row r="13" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B13" s="3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C13" s="3">
         <v>10</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="14" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -2594,16 +2743,16 @@
         <v>27</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D14" s="1" t="s">
         <v>33</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="15" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -2611,1247 +2760,1327 @@
         <v>32</v>
       </c>
       <c r="C15" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="E15" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="D15" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="E15" s="1" t="s">
-        <v>75</v>
-      </c>
       <c r="F15" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="16" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B16" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="E16" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="C16" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="D16" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="E16" s="1" t="s">
-        <v>63</v>
-      </c>
       <c r="F16" s="1" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
     </row>
     <row r="17" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B17" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="C17" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="C17" s="3" t="s">
+      <c r="D17" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="D17" s="1" t="s">
+      <c r="E17" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="E17" s="1" t="s">
+      <c r="F17" s="1" t="s">
         <v>68</v>
-      </c>
-      <c r="F17" s="1" t="s">
-        <v>69</v>
       </c>
     </row>
     <row r="18" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B18" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="C18" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="C18" s="3" t="s">
-        <v>82</v>
-      </c>
       <c r="D18" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="F18" s="1" t="s">
         <v>78</v>
-      </c>
-      <c r="E18" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="F18" s="1" t="s">
-        <v>79</v>
       </c>
     </row>
     <row r="19" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B19" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="D19" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="C19" s="3" t="s">
-        <v>86</v>
-      </c>
-      <c r="D19" s="1" t="s">
+      <c r="E19" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="E19" s="1" t="s">
-        <v>85</v>
-      </c>
       <c r="F19" s="1" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
     </row>
     <row r="20" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B20" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="D20" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="C20" s="3" t="s">
-        <v>82</v>
-      </c>
-      <c r="D20" s="1" t="s">
+      <c r="E20" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="F20" s="1" t="s">
         <v>88</v>
-      </c>
-      <c r="E20" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="F20" s="1" t="s">
-        <v>89</v>
       </c>
     </row>
     <row r="21" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B21" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="C21" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="E21" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="C21" s="3" t="s">
-        <v>82</v>
-      </c>
-      <c r="D21" s="1" t="s">
+      <c r="F21" s="1" t="s">
         <v>93</v>
-      </c>
-      <c r="E21" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="F21" s="1" t="s">
-        <v>94</v>
       </c>
     </row>
     <row r="22" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B22" s="3" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C22" s="3">
         <v>50</v>
       </c>
       <c r="D22" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="E22" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="F22" s="1" t="s">
         <v>99</v>
-      </c>
-      <c r="E22" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="F22" s="1" t="s">
-        <v>100</v>
       </c>
     </row>
     <row r="23" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B23" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="C23" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="D23" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="E23" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="F23" s="1" t="s">
         <v>103</v>
-      </c>
-      <c r="C23" s="3" t="s">
-        <v>105</v>
-      </c>
-      <c r="D23" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="E23" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="F23" s="1" t="s">
-        <v>104</v>
       </c>
     </row>
     <row r="24" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B24" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="C24" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="D24" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="C24" s="3" t="s">
+      <c r="E24" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="D24" s="1" t="s">
-        <v>107</v>
-      </c>
-      <c r="E24" s="1" t="s">
-        <v>109</v>
-      </c>
       <c r="F24" s="1" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="25" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B25" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="C25" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="D25" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="C25" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="D25" s="1" t="s">
+      <c r="E25" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="E25" s="1" t="s">
-        <v>112</v>
-      </c>
       <c r="F25" s="1" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="26" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B26" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="C26" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="D26" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="E26" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="F26" s="1" t="s">
         <v>113</v>
-      </c>
-      <c r="C26" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="D26" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="E26" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="F26" s="1" t="s">
-        <v>114</v>
       </c>
     </row>
     <row r="27" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B27" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="C27" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="D27" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="E27" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="C27" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="D27" s="1" t="s">
-        <v>118</v>
-      </c>
-      <c r="E27" s="1" t="s">
-        <v>117</v>
-      </c>
       <c r="F27" s="1" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="28" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B28" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="C28" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="D28" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="E28" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="F28" s="1" t="s">
         <v>120</v>
-      </c>
-      <c r="C28" s="3" t="s">
-        <v>82</v>
-      </c>
-      <c r="D28" s="1" t="s">
-        <v>119</v>
-      </c>
-      <c r="E28" s="1" t="s">
-        <v>122</v>
-      </c>
-      <c r="F28" s="1" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="29" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B29" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="C29" s="3" t="s">
         <v>124</v>
       </c>
-      <c r="C29" s="3" t="s">
+      <c r="D29" s="1" t="s">
         <v>125</v>
       </c>
-      <c r="D29" s="1" t="s">
+      <c r="E29" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="F29" s="1" t="s">
         <v>126</v>
-      </c>
-      <c r="E29" s="1" t="s">
-        <v>129</v>
-      </c>
-      <c r="F29" s="1" t="s">
-        <v>127</v>
       </c>
     </row>
     <row r="30" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B30" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="C30" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="D30" s="1" t="s">
         <v>131</v>
       </c>
-      <c r="C30" s="3" t="s">
-        <v>82</v>
-      </c>
-      <c r="D30" s="1" t="s">
+      <c r="E30" s="1" t="s">
         <v>132</v>
       </c>
-      <c r="E30" s="1" t="s">
-        <v>133</v>
-      </c>
       <c r="F30" s="1" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="31" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B31" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="C31" s="3" t="s">
         <v>134</v>
       </c>
-      <c r="C31" s="3" t="s">
+      <c r="D31" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="D31" s="1" t="s">
-        <v>136</v>
-      </c>
       <c r="E31" s="1" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="F31" s="1" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
     <row r="32" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B32" s="3" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="F32" s="1" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="33" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B33" s="3" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="C33" s="3">
         <v>10</v>
       </c>
       <c r="D33" s="1" t="s">
+        <v>243</v>
+      </c>
+      <c r="E33" s="1" t="s">
+        <v>245</v>
+      </c>
+      <c r="F33" s="1" t="s">
         <v>244</v>
-      </c>
-      <c r="E33" s="1" t="s">
-        <v>246</v>
-      </c>
-      <c r="F33" s="1" t="s">
-        <v>245</v>
       </c>
     </row>
     <row r="34" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B34" s="3" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="C34" s="3">
         <v>190</v>
       </c>
       <c r="D34" s="1" t="s">
+        <v>290</v>
+      </c>
+      <c r="E34" s="1" t="s">
+        <v>296</v>
+      </c>
+      <c r="F34" s="1" t="s">
         <v>291</v>
-      </c>
-      <c r="E34" s="1" t="s">
-        <v>297</v>
-      </c>
-      <c r="F34" s="1" t="s">
-        <v>292</v>
       </c>
     </row>
     <row r="35" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B35" s="3" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="C35" s="3">
         <v>30</v>
       </c>
       <c r="D35" s="1" t="s">
+        <v>293</v>
+      </c>
+      <c r="E35" s="1" t="s">
         <v>294</v>
       </c>
-      <c r="E35" s="1" t="s">
+      <c r="F35" s="1" t="s">
         <v>295</v>
-      </c>
-      <c r="F35" s="1" t="s">
-        <v>296</v>
       </c>
     </row>
     <row r="36" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B36" s="3" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="C36" s="3">
         <v>15</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>533</v>
+        <v>531</v>
       </c>
       <c r="E36" s="1" t="s">
-        <v>532</v>
+        <v>530</v>
       </c>
       <c r="F36" s="1" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
     </row>
     <row r="37" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B37" s="3" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="C37" s="3">
         <v>40</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="E37" s="1" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="F37" s="1" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
     </row>
     <row r="38" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B38" s="3" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="C38" s="3">
         <v>30</v>
       </c>
       <c r="D38" s="1" t="s">
+        <v>312</v>
+      </c>
+      <c r="E38" s="1" t="s">
         <v>313</v>
       </c>
-      <c r="E38" s="1" t="s">
+      <c r="F38" s="1" t="s">
         <v>314</v>
       </c>
-      <c r="F38" s="1" t="s">
-        <v>315</v>
-      </c>
-    </row>
-    <row r="39" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B39" s="11" t="s">
-        <v>333</v>
-      </c>
-      <c r="C39" s="11">
+    </row>
+    <row r="39" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B39" s="3" t="s">
+        <v>332</v>
+      </c>
+      <c r="C39" s="3">
         <v>50</v>
       </c>
-      <c r="D39" s="7" t="s">
+      <c r="D39" s="1" t="s">
+        <v>330</v>
+      </c>
+      <c r="E39" s="1" t="s">
         <v>331</v>
       </c>
-      <c r="E39" s="7" t="s">
-        <v>332</v>
-      </c>
-      <c r="F39" s="7" t="s">
-        <v>335</v>
+      <c r="F39" s="1" t="s">
+        <v>334</v>
       </c>
     </row>
     <row r="40" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B40" s="3" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="C40" s="3">
         <v>20</v>
       </c>
       <c r="D40" s="1" t="s">
+        <v>345</v>
+      </c>
+      <c r="E40" s="1" t="s">
         <v>346</v>
       </c>
-      <c r="E40" s="1" t="s">
-        <v>347</v>
-      </c>
       <c r="F40" s="1" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
     </row>
     <row r="41" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B41" s="3" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="C41" s="3">
         <v>81</v>
       </c>
       <c r="D41" s="1" t="s">
+        <v>348</v>
+      </c>
+      <c r="E41" s="1" t="s">
+        <v>350</v>
+      </c>
+      <c r="F41" s="1" t="s">
         <v>349</v>
-      </c>
-      <c r="E41" s="1" t="s">
-        <v>351</v>
-      </c>
-      <c r="F41" s="1" t="s">
-        <v>350</v>
       </c>
     </row>
     <row r="42" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B42" s="3" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="C42" s="3">
         <v>120</v>
       </c>
       <c r="D42" s="1" t="s">
+        <v>352</v>
+      </c>
+      <c r="E42" s="1" t="s">
+        <v>354</v>
+      </c>
+      <c r="F42" s="1" t="s">
         <v>353</v>
-      </c>
-      <c r="E42" s="1" t="s">
-        <v>355</v>
-      </c>
-      <c r="F42" s="1" t="s">
-        <v>354</v>
       </c>
     </row>
     <row r="43" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B43" s="3" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="C43" s="3">
         <v>20</v>
       </c>
       <c r="D43" s="1" t="s">
+        <v>356</v>
+      </c>
+      <c r="E43" s="1" t="s">
         <v>357</v>
       </c>
-      <c r="E43" s="1" t="s">
+      <c r="F43" s="1" t="s">
         <v>358</v>
-      </c>
-      <c r="F43" s="1" t="s">
-        <v>359</v>
       </c>
     </row>
     <row r="44" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B44" s="3" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="C44" s="3">
         <v>50</v>
       </c>
       <c r="D44" s="1" t="s">
+        <v>360</v>
+      </c>
+      <c r="E44" s="1" t="s">
         <v>361</v>
       </c>
-      <c r="E44" s="1" t="s">
+      <c r="F44" s="1" t="s">
         <v>362</v>
-      </c>
-      <c r="F44" s="1" t="s">
-        <v>363</v>
       </c>
     </row>
     <row r="45" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B45" s="3" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="C45" s="3">
         <v>20</v>
       </c>
       <c r="D45" s="1" t="s">
+        <v>368</v>
+      </c>
+      <c r="E45" s="1" t="s">
+        <v>367</v>
+      </c>
+      <c r="F45" s="1" t="s">
         <v>369</v>
-      </c>
-      <c r="E45" s="1" t="s">
-        <v>368</v>
-      </c>
-      <c r="F45" s="1" t="s">
-        <v>370</v>
       </c>
     </row>
     <row r="46" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B46" s="3" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="C46" s="3">
         <v>50</v>
       </c>
       <c r="D46" s="1" t="s">
+        <v>371</v>
+      </c>
+      <c r="E46" s="1" t="s">
         <v>372</v>
       </c>
-      <c r="E46" s="1" t="s">
+      <c r="F46" s="1" t="s">
         <v>373</v>
-      </c>
-      <c r="F46" s="1" t="s">
-        <v>374</v>
       </c>
     </row>
     <row r="47" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B47" s="3" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="C47" s="3">
         <v>150</v>
       </c>
       <c r="D47" s="1" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="E47" s="1" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="F47" s="1" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
     </row>
     <row r="48" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B48" s="3" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="C48" s="3">
         <v>3</v>
       </c>
       <c r="D48" s="1" t="s">
+        <v>389</v>
+      </c>
+      <c r="E48" s="1" t="s">
         <v>390</v>
       </c>
-      <c r="E48" s="1" t="s">
-        <v>391</v>
-      </c>
       <c r="F48" s="1" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
     </row>
     <row r="49" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B49" s="3" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="C49" s="3">
         <v>104</v>
       </c>
       <c r="D49" s="1" t="s">
+        <v>435</v>
+      </c>
+      <c r="E49" s="1" t="s">
         <v>436</v>
       </c>
-      <c r="E49" s="1" t="s">
-        <v>437</v>
-      </c>
       <c r="F49" s="1" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="50" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B50" s="3" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="C50" s="3">
         <v>50</v>
       </c>
       <c r="D50" s="1" t="s">
+        <v>438</v>
+      </c>
+      <c r="E50" s="1" t="s">
         <v>439</v>
       </c>
-      <c r="E50" s="1" t="s">
-        <v>440</v>
-      </c>
       <c r="F50" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="51" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B51" s="3" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="C51" s="3">
         <v>26</v>
       </c>
       <c r="D51" s="1" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="E51" s="1" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="F51" s="1" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
     </row>
     <row r="52" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B52" s="3" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="C52" s="3">
         <v>21</v>
       </c>
       <c r="D52" s="1" t="s">
+        <v>451</v>
+      </c>
+      <c r="E52" s="1" t="s">
         <v>452</v>
       </c>
-      <c r="E52" s="1" t="s">
-        <v>453</v>
-      </c>
       <c r="F52" s="1" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
     </row>
     <row r="53" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B53" s="3" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
       <c r="C53" s="3">
         <v>5</v>
       </c>
       <c r="D53" s="1" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="E53" s="1" t="s">
+        <v>454</v>
+      </c>
+      <c r="F53" s="1" t="s">
         <v>455</v>
-      </c>
-      <c r="F53" s="1" t="s">
-        <v>456</v>
       </c>
     </row>
     <row r="54" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B54" s="3" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="C54" s="3">
         <v>207</v>
       </c>
       <c r="D54" s="1" t="s">
+        <v>462</v>
+      </c>
+      <c r="E54" s="1" t="s">
         <v>463</v>
       </c>
-      <c r="E54" s="1" t="s">
-        <v>464</v>
-      </c>
       <c r="F54" s="1" t="s">
-        <v>485</v>
+        <v>483</v>
       </c>
     </row>
     <row r="55" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B55" s="3" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="C55" s="3">
         <v>10</v>
       </c>
       <c r="D55" s="1" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="E55" s="1" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="F55" s="1" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
     </row>
     <row r="56" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B56" s="3" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="C56" s="3">
         <v>13</v>
       </c>
       <c r="D56" s="1" t="s">
+        <v>469</v>
+      </c>
+      <c r="E56" s="1" t="s">
+        <v>471</v>
+      </c>
+      <c r="F56" s="1" t="s">
         <v>470</v>
-      </c>
-      <c r="E56" s="1" t="s">
-        <v>472</v>
-      </c>
-      <c r="F56" s="1" t="s">
-        <v>471</v>
       </c>
     </row>
     <row r="57" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B57" s="3" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="C57" s="3">
         <v>5</v>
       </c>
       <c r="D57" s="1" t="s">
+        <v>473</v>
+      </c>
+      <c r="E57" s="1" t="s">
         <v>474</v>
       </c>
-      <c r="E57" s="1" t="s">
+      <c r="F57" s="1" t="s">
         <v>475</v>
-      </c>
-      <c r="F57" s="1" t="s">
-        <v>476</v>
       </c>
     </row>
     <row r="58" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B58" s="3" t="s">
-        <v>481</v>
+        <v>479</v>
       </c>
       <c r="C58" s="3">
         <v>50</v>
       </c>
       <c r="D58" s="1" t="s">
+        <v>480</v>
+      </c>
+      <c r="E58" s="1" t="s">
+        <v>481</v>
+      </c>
+      <c r="F58" s="1" t="s">
         <v>482</v>
-      </c>
-      <c r="E58" s="1" t="s">
-        <v>483</v>
-      </c>
-      <c r="F58" s="1" t="s">
-        <v>484</v>
       </c>
     </row>
     <row r="59" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B59" s="3" t="s">
+        <v>484</v>
+      </c>
+      <c r="C59" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="D59" s="1" t="s">
+        <v>485</v>
+      </c>
+      <c r="E59" s="1" t="s">
         <v>486</v>
       </c>
-      <c r="C59" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="D59" s="1" t="s">
+      <c r="F59" s="1" t="s">
         <v>487</v>
-      </c>
-      <c r="E59" s="1" t="s">
-        <v>488</v>
-      </c>
-      <c r="F59" s="1" t="s">
-        <v>489</v>
       </c>
     </row>
     <row r="60" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B60" s="3" t="s">
-        <v>493</v>
+        <v>491</v>
       </c>
       <c r="C60" s="3" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D60" s="1" t="s">
+        <v>488</v>
+      </c>
+      <c r="E60" s="1" t="s">
+        <v>489</v>
+      </c>
+      <c r="F60" s="1" t="s">
         <v>490</v>
-      </c>
-      <c r="E60" s="1" t="s">
-        <v>491</v>
-      </c>
-      <c r="F60" s="1" t="s">
-        <v>492</v>
       </c>
     </row>
     <row r="61" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B61" s="3" t="s">
-        <v>494</v>
+        <v>492</v>
       </c>
       <c r="C61" s="3">
         <v>50</v>
       </c>
       <c r="D61" s="1" t="s">
+        <v>493</v>
+      </c>
+      <c r="E61" s="1" t="s">
+        <v>494</v>
+      </c>
+      <c r="F61" s="1" t="s">
         <v>495</v>
-      </c>
-      <c r="E61" s="1" t="s">
-        <v>496</v>
-      </c>
-      <c r="F61" s="1" t="s">
-        <v>497</v>
       </c>
     </row>
     <row r="62" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B62" s="3" t="s">
+        <v>496</v>
+      </c>
+      <c r="C62" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="D62" s="1" t="s">
+        <v>497</v>
+      </c>
+      <c r="E62" s="1" t="s">
         <v>498</v>
       </c>
-      <c r="C62" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="D62" s="1" t="s">
-        <v>499</v>
-      </c>
-      <c r="E62" s="1" t="s">
-        <v>500</v>
-      </c>
       <c r="F62" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="63" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B63" s="3" t="s">
-        <v>503</v>
+        <v>501</v>
       </c>
       <c r="C63" s="3" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D63" s="1" t="s">
-        <v>501</v>
+        <v>499</v>
       </c>
       <c r="E63" s="1" t="s">
-        <v>502</v>
+        <v>500</v>
       </c>
       <c r="F63" s="1" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
     </row>
     <row r="64" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B64" s="3" t="s">
-        <v>514</v>
+        <v>512</v>
       </c>
       <c r="C64" s="3">
         <v>30</v>
       </c>
       <c r="D64" s="1" t="s">
-        <v>515</v>
+        <v>513</v>
       </c>
       <c r="E64" s="1" t="s">
-        <v>512</v>
+        <v>510</v>
       </c>
       <c r="F64" s="1" t="s">
-        <v>513</v>
+        <v>511</v>
       </c>
     </row>
     <row r="65" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B65" s="3" t="s">
+        <v>515</v>
+      </c>
+      <c r="C65" s="3" t="s">
         <v>517</v>
       </c>
-      <c r="C65" s="3" t="s">
-        <v>519</v>
-      </c>
       <c r="D65" s="1" t="s">
+        <v>516</v>
+      </c>
+      <c r="E65" s="1" t="s">
         <v>518</v>
       </c>
-      <c r="E65" s="1" t="s">
-        <v>520</v>
-      </c>
       <c r="F65" s="1" t="s">
-        <v>516</v>
+        <v>514</v>
       </c>
     </row>
     <row r="66" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B66" s="3" t="s">
+        <v>519</v>
+      </c>
+      <c r="C66" s="3" t="s">
+        <v>517</v>
+      </c>
+      <c r="D66" s="1" t="s">
+        <v>522</v>
+      </c>
+      <c r="E66" s="1" t="s">
+        <v>520</v>
+      </c>
+      <c r="F66" s="1" t="s">
         <v>521</v>
-      </c>
-      <c r="C66" s="3" t="s">
-        <v>519</v>
-      </c>
-      <c r="D66" s="1" t="s">
-        <v>524</v>
-      </c>
-      <c r="E66" s="1" t="s">
-        <v>522</v>
-      </c>
-      <c r="F66" s="1" t="s">
-        <v>523</v>
       </c>
     </row>
     <row r="67" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B67" s="3" t="s">
+        <v>523</v>
+      </c>
+      <c r="C67" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="D67" s="1" t="s">
+        <v>540</v>
+      </c>
+      <c r="E67" s="1" t="s">
+        <v>524</v>
+      </c>
+      <c r="F67" s="1" t="s">
         <v>525</v>
-      </c>
-      <c r="C67" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="D67" s="1" t="s">
-        <v>542</v>
-      </c>
-      <c r="E67" s="1" t="s">
-        <v>526</v>
-      </c>
-      <c r="F67" s="1" t="s">
-        <v>527</v>
       </c>
     </row>
     <row r="68" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B68" s="3" t="s">
-        <v>531</v>
+        <v>529</v>
       </c>
       <c r="C68" s="3">
         <v>18</v>
       </c>
       <c r="D68" s="1" t="s">
-        <v>530</v>
+        <v>528</v>
       </c>
       <c r="E68" s="1" t="s">
-        <v>529</v>
+        <v>527</v>
       </c>
       <c r="F68" s="1" t="s">
-        <v>528</v>
+        <v>526</v>
       </c>
     </row>
     <row r="69" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B69" s="3" t="s">
-        <v>537</v>
+        <v>535</v>
       </c>
       <c r="C69" s="3" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D69" s="1" t="s">
-        <v>536</v>
+        <v>534</v>
       </c>
       <c r="E69" s="1" t="s">
-        <v>534</v>
+        <v>532</v>
       </c>
       <c r="F69" s="1" t="s">
-        <v>535</v>
+        <v>533</v>
       </c>
     </row>
     <row r="70" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B70" s="3" t="s">
+        <v>536</v>
+      </c>
+      <c r="C70" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="D70" s="1" t="s">
+        <v>539</v>
+      </c>
+      <c r="E70" s="1" t="s">
+        <v>537</v>
+      </c>
+      <c r="F70" s="1" t="s">
         <v>538</v>
-      </c>
-      <c r="C70" s="3" t="s">
-        <v>144</v>
-      </c>
-      <c r="D70" s="1" t="s">
-        <v>541</v>
-      </c>
-      <c r="E70" s="1" t="s">
-        <v>539</v>
-      </c>
-      <c r="F70" s="1" t="s">
-        <v>540</v>
       </c>
     </row>
     <row r="71" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B71" s="3" t="s">
-        <v>543</v>
+        <v>541</v>
       </c>
       <c r="C71" s="3">
         <v>10</v>
       </c>
       <c r="D71" s="1" t="s">
-        <v>544</v>
+        <v>542</v>
       </c>
       <c r="E71" s="1" t="s">
-        <v>545</v>
+        <v>543</v>
       </c>
       <c r="F71" s="1" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="72" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B72" s="3" t="s">
-        <v>546</v>
+        <v>544</v>
       </c>
       <c r="C72" s="3">
         <v>20</v>
       </c>
       <c r="D72" s="1" t="s">
+        <v>545</v>
+      </c>
+      <c r="E72" s="1" t="s">
         <v>547</v>
       </c>
-      <c r="E72" s="1" t="s">
-        <v>549</v>
-      </c>
       <c r="F72" s="1" t="s">
-        <v>548</v>
+        <v>546</v>
       </c>
     </row>
     <row r="73" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B73" s="3" t="s">
-        <v>550</v>
+        <v>548</v>
       </c>
       <c r="C73" s="3">
         <v>50</v>
       </c>
       <c r="D73" s="1" t="s">
-        <v>552</v>
+        <v>550</v>
       </c>
       <c r="E73" s="1" t="s">
-        <v>553</v>
+        <v>551</v>
       </c>
       <c r="F73" s="1" t="s">
-        <v>551</v>
+        <v>549</v>
       </c>
     </row>
     <row r="74" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B74" s="3" t="s">
-        <v>555</v>
+        <v>553</v>
       </c>
       <c r="C74" s="3">
         <v>22</v>
       </c>
       <c r="D74" s="1" t="s">
-        <v>556</v>
+        <v>621</v>
       </c>
       <c r="E74" s="1" t="s">
-        <v>557</v>
+        <v>554</v>
       </c>
       <c r="F74" s="1" t="s">
-        <v>554</v>
+        <v>552</v>
       </c>
     </row>
     <row r="75" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B75" s="3" t="s">
-        <v>559</v>
+        <v>556</v>
       </c>
       <c r="C75" s="1">
         <v>10</v>
       </c>
       <c r="D75" s="1" t="s">
-        <v>561</v>
+        <v>558</v>
       </c>
       <c r="E75" s="1" t="s">
-        <v>560</v>
+        <v>557</v>
       </c>
       <c r="F75" s="1" t="s">
-        <v>558</v>
+        <v>555</v>
       </c>
     </row>
     <row r="76" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B76" s="3" t="s">
-        <v>566</v>
+        <v>563</v>
       </c>
       <c r="C76" s="1">
         <v>10</v>
       </c>
       <c r="D76" s="1" t="s">
-        <v>569</v>
+        <v>566</v>
       </c>
       <c r="E76" s="1" t="s">
-        <v>567</v>
+        <v>564</v>
       </c>
       <c r="F76" s="1" t="s">
-        <v>568</v>
+        <v>565</v>
       </c>
     </row>
     <row r="77" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B77" s="3" t="s">
-        <v>570</v>
+        <v>567</v>
       </c>
       <c r="C77" s="3">
         <v>10</v>
       </c>
       <c r="D77" s="1" t="s">
-        <v>571</v>
+        <v>568</v>
       </c>
       <c r="E77" s="1" t="s">
-        <v>572</v>
+        <v>569</v>
       </c>
       <c r="F77" s="1" t="s">
-        <v>573</v>
+        <v>570</v>
       </c>
     </row>
     <row r="78" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B78" s="3" t="s">
-        <v>574</v>
+        <v>571</v>
       </c>
       <c r="C78" s="3">
         <v>15</v>
       </c>
       <c r="D78" s="1" t="s">
-        <v>575</v>
+        <v>572</v>
       </c>
       <c r="E78" s="1" t="s">
-        <v>576</v>
+        <v>573</v>
       </c>
       <c r="F78" s="1" t="s">
-        <v>577</v>
+        <v>574</v>
       </c>
     </row>
     <row r="79" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B79" s="3" t="s">
-        <v>578</v>
+        <v>575</v>
       </c>
       <c r="C79" s="3">
         <v>25</v>
       </c>
       <c r="D79" s="1" t="s">
-        <v>580</v>
+        <v>577</v>
       </c>
       <c r="E79" s="1" t="s">
-        <v>579</v>
+        <v>576</v>
       </c>
       <c r="F79" s="1" t="s">
-        <v>528</v>
+        <v>526</v>
       </c>
     </row>
     <row r="80" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B80" s="3" t="s">
-        <v>584</v>
+        <v>581</v>
       </c>
       <c r="C80" s="3">
         <v>10</v>
       </c>
       <c r="D80" s="1" t="s">
-        <v>585</v>
+        <v>582</v>
       </c>
       <c r="E80" s="1" t="s">
-        <v>586</v>
+        <v>583</v>
       </c>
       <c r="F80" s="1" t="s">
-        <v>587</v>
+        <v>584</v>
       </c>
     </row>
     <row r="81" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B81" s="3" t="s">
-        <v>592</v>
+        <v>589</v>
       </c>
       <c r="C81" s="3">
         <v>25</v>
       </c>
       <c r="D81" s="1" t="s">
-        <v>593</v>
+        <v>590</v>
       </c>
       <c r="E81" s="1" t="s">
-        <v>594</v>
+        <v>591</v>
       </c>
       <c r="F81" s="1" t="s">
-        <v>595</v>
+        <v>592</v>
       </c>
     </row>
     <row r="82" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B82" s="3" t="s">
-        <v>596</v>
+        <v>593</v>
       </c>
       <c r="C82" s="3">
         <v>30</v>
       </c>
       <c r="D82" s="1" t="s">
-        <v>597</v>
+        <v>594</v>
       </c>
       <c r="E82" s="1" t="s">
-        <v>598</v>
+        <v>595</v>
       </c>
       <c r="F82" s="1" t="s">
-        <v>599</v>
+        <v>596</v>
       </c>
     </row>
     <row r="83" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B83" s="3" t="s">
-        <v>600</v>
+        <v>597</v>
       </c>
       <c r="C83" s="3">
         <v>41</v>
       </c>
       <c r="D83" s="1" t="s">
-        <v>601</v>
+        <v>598</v>
       </c>
       <c r="E83" s="1" t="s">
-        <v>603</v>
+        <v>600</v>
       </c>
       <c r="F83" s="1" t="s">
-        <v>602</v>
+        <v>599</v>
       </c>
     </row>
     <row r="84" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B84" s="3" t="s">
-        <v>604</v>
+        <v>601</v>
       </c>
       <c r="C84" s="3">
         <v>100</v>
       </c>
       <c r="D84" s="1" t="s">
-        <v>605</v>
+        <v>602</v>
       </c>
       <c r="E84" s="1" t="s">
-        <v>606</v>
+        <v>603</v>
       </c>
       <c r="F84" s="1" t="s">
-        <v>607</v>
+        <v>604</v>
       </c>
     </row>
     <row r="85" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B85" s="3" t="s">
-        <v>608</v>
+        <v>605</v>
       </c>
       <c r="C85" s="3">
         <v>28</v>
       </c>
       <c r="D85" s="1" t="s">
-        <v>611</v>
+        <v>608</v>
       </c>
       <c r="E85" s="1" t="s">
-        <v>609</v>
+        <v>606</v>
       </c>
       <c r="F85" s="1" t="s">
-        <v>610</v>
+        <v>607</v>
       </c>
     </row>
     <row r="86" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B86" s="3" t="s">
-        <v>612</v>
+        <v>609</v>
       </c>
       <c r="C86" s="3">
         <v>25</v>
       </c>
       <c r="D86" s="1" t="s">
-        <v>613</v>
-      </c>
-      <c r="E86" s="4" t="s">
-        <v>614</v>
+        <v>610</v>
+      </c>
+      <c r="E86" s="1" t="s">
+        <v>611</v>
       </c>
       <c r="F86" s="1" t="s">
-        <v>577</v>
+        <v>574</v>
       </c>
     </row>
     <row r="87" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B87" s="3" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
       <c r="C87" s="3">
         <v>10</v>
       </c>
       <c r="D87" s="1" t="s">
-        <v>618</v>
+        <v>615</v>
       </c>
       <c r="E87" s="1" t="s">
-        <v>617</v>
+        <v>614</v>
       </c>
       <c r="F87" s="1" t="s">
-        <v>616</v>
-      </c>
-    </row>
-    <row r="88" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="89" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="90" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="91" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="92" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25"/>
+        <v>613</v>
+      </c>
+    </row>
+    <row r="88" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B88" s="3" t="s">
+        <v>623</v>
+      </c>
+      <c r="C88" s="3">
+        <v>20</v>
+      </c>
+      <c r="D88" s="1" t="s">
+        <v>624</v>
+      </c>
+      <c r="E88" s="1" t="s">
+        <v>625</v>
+      </c>
+      <c r="F88" s="1" t="s">
+        <v>626</v>
+      </c>
+    </row>
+    <row r="89" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B89" s="3" t="s">
+        <v>627</v>
+      </c>
+      <c r="C89" s="3">
+        <v>20</v>
+      </c>
+      <c r="D89" s="1" t="s">
+        <v>630</v>
+      </c>
+      <c r="E89" s="1" t="s">
+        <v>628</v>
+      </c>
+      <c r="F89" s="1" t="s">
+        <v>629</v>
+      </c>
+    </row>
+    <row r="90" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B90" s="3" t="s">
+        <v>631</v>
+      </c>
+      <c r="C90" s="3">
+        <v>20</v>
+      </c>
+      <c r="D90" s="1" t="s">
+        <v>632</v>
+      </c>
+      <c r="E90" s="1" t="s">
+        <v>633</v>
+      </c>
+      <c r="F90" s="1" t="s">
+        <v>634</v>
+      </c>
+    </row>
+    <row r="91" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B91" s="3" t="s">
+        <v>635</v>
+      </c>
+      <c r="C91" s="3">
+        <v>10</v>
+      </c>
+      <c r="D91" s="9" t="s">
+        <v>637</v>
+      </c>
+      <c r="E91" s="1" t="s">
+        <v>636</v>
+      </c>
+      <c r="F91" s="1" t="s">
+        <v>638</v>
+      </c>
+    </row>
+    <row r="92" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B92" s="3" t="s">
+        <v>639</v>
+      </c>
+      <c r="C92" s="3">
+        <v>10</v>
+      </c>
+      <c r="D92" s="1" t="s">
+        <v>641</v>
+      </c>
+      <c r="E92" s="1" t="s">
+        <v>640</v>
+      </c>
+      <c r="F92" s="1" t="s">
+        <v>596</v>
+      </c>
+    </row>
     <row r="93" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="94" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="95" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -3894,24 +4123,24 @@
         <v>7</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="3" spans="2:6" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B3" s="3" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="C3" s="3" t="s">
         <v>11</v>
       </c>
       <c r="D3" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="E3" s="1" t="s">
         <v>159</v>
       </c>
-      <c r="E3" s="1" t="s">
-        <v>160</v>
-      </c>
       <c r="F3" s="1" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
     </row>
     <row r="4" spans="2:6" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -3919,33 +4148,33 @@
         <v>19</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="D4" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="E4" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="E4" s="1" t="s">
-        <v>165</v>
-      </c>
       <c r="F4" s="4" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="5" spans="2:6" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="3" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="C5" s="3">
         <v>500</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
     </row>
     <row r="6" spans="2:6" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -3956,13 +4185,13 @@
         <v>700</v>
       </c>
       <c r="D6" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="F6" s="1" t="s">
         <v>168</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>170</v>
-      </c>
-      <c r="F6" s="1" t="s">
-        <v>169</v>
       </c>
     </row>
     <row r="7" spans="2:6" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -3973,438 +4202,438 @@
         <v>470</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="8" spans="2:6" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B8" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="C8" s="13">
+      <c r="C8" s="7">
         <v>1500</v>
       </c>
       <c r="D8" s="1" t="s">
+        <v>225</v>
+      </c>
+      <c r="E8" s="1" t="s">
         <v>226</v>
       </c>
-      <c r="E8" s="1" t="s">
+      <c r="F8" s="1" t="s">
         <v>227</v>
-      </c>
-      <c r="F8" s="1" t="s">
-        <v>228</v>
       </c>
     </row>
     <row r="9" spans="2:6" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B9" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="C9" s="13">
+      <c r="C9" s="7">
         <v>30000</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
     </row>
     <row r="10" spans="2:6" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="C10" s="13">
+      <c r="C10" s="7">
         <v>5000</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="11" spans="2:6" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B11" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="C11" s="13">
+        <v>69</v>
+      </c>
+      <c r="C11" s="7">
         <v>8000</v>
       </c>
       <c r="D11" s="1" t="s">
+        <v>269</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>271</v>
+      </c>
+      <c r="F11" s="1" t="s">
         <v>270</v>
-      </c>
-      <c r="E11" s="1" t="s">
-        <v>272</v>
-      </c>
-      <c r="F11" s="1" t="s">
-        <v>271</v>
       </c>
     </row>
     <row r="12" spans="2:6" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B12" s="3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C12" s="3">
         <v>150</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="E12" s="1" t="s">
+        <v>272</v>
+      </c>
+      <c r="F12" s="1" t="s">
         <v>273</v>
-      </c>
-      <c r="F12" s="1" t="s">
-        <v>274</v>
       </c>
     </row>
     <row r="13" spans="2:6" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B13" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="C13" s="13">
+        <v>71</v>
+      </c>
+      <c r="C13" s="7">
         <v>700</v>
       </c>
       <c r="D13" s="1" t="s">
+        <v>275</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>277</v>
+      </c>
+      <c r="F13" s="1" t="s">
         <v>276</v>
-      </c>
-      <c r="E13" s="1" t="s">
-        <v>278</v>
-      </c>
-      <c r="F13" s="1" t="s">
-        <v>277</v>
       </c>
     </row>
     <row r="14" spans="2:6" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B14" s="3" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="C14" s="3">
         <v>800</v>
       </c>
       <c r="D14" s="1" t="s">
+        <v>279</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>281</v>
+      </c>
+      <c r="F14" s="1" t="s">
         <v>280</v>
-      </c>
-      <c r="E14" s="1" t="s">
-        <v>282</v>
-      </c>
-      <c r="F14" s="1" t="s">
-        <v>281</v>
       </c>
     </row>
     <row r="15" spans="2:6" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B15" s="3" t="s">
+        <v>283</v>
+      </c>
+      <c r="C15" s="7">
+        <v>1400</v>
+      </c>
+      <c r="D15" s="1" t="s">
         <v>284</v>
       </c>
-      <c r="C15" s="13">
-        <v>1400</v>
-      </c>
-      <c r="D15" s="1" t="s">
+      <c r="E15" s="1" t="s">
+        <v>282</v>
+      </c>
+      <c r="F15" s="1" t="s">
         <v>285</v>
-      </c>
-      <c r="E15" s="1" t="s">
-        <v>283</v>
-      </c>
-      <c r="F15" s="1" t="s">
-        <v>286</v>
       </c>
     </row>
     <row r="16" spans="2:6" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B16" s="3" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="C16" s="3">
         <v>500</v>
       </c>
       <c r="D16" s="1" t="s">
+        <v>265</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>268</v>
+      </c>
+      <c r="F16" s="1" t="s">
         <v>266</v>
-      </c>
-      <c r="E16" s="1" t="s">
-        <v>269</v>
-      </c>
-      <c r="F16" s="1" t="s">
-        <v>267</v>
       </c>
     </row>
     <row r="17" spans="2:6" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B17" s="3" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C17" s="3">
         <v>100</v>
       </c>
       <c r="D17" s="1" t="s">
+        <v>263</v>
+      </c>
+      <c r="E17" s="1" t="s">
         <v>264</v>
       </c>
-      <c r="E17" s="1" t="s">
-        <v>265</v>
-      </c>
       <c r="F17" s="1" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
     </row>
     <row r="18" spans="2:6" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B18" s="3" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C18" s="3">
         <v>30</v>
       </c>
       <c r="D18" s="1" t="s">
+        <v>260</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>259</v>
+      </c>
+      <c r="F18" s="1" t="s">
         <v>261</v>
-      </c>
-      <c r="E18" s="1" t="s">
-        <v>260</v>
-      </c>
-      <c r="F18" s="1" t="s">
-        <v>262</v>
       </c>
     </row>
     <row r="19" spans="2:6" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B19" s="3" t="s">
-        <v>128</v>
-      </c>
-      <c r="C19" s="13">
+        <v>127</v>
+      </c>
+      <c r="C19" s="7">
         <v>15000</v>
       </c>
       <c r="D19" s="1" t="s">
+        <v>257</v>
+      </c>
+      <c r="E19" s="1" t="s">
         <v>258</v>
       </c>
-      <c r="E19" s="1" t="s">
-        <v>259</v>
-      </c>
       <c r="F19" s="1" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
     </row>
     <row r="20" spans="2:6" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B20" s="3" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C20" s="3">
         <v>14000</v>
       </c>
       <c r="D20" s="1" t="s">
+        <v>251</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>253</v>
+      </c>
+      <c r="F20" s="1" t="s">
         <v>252</v>
-      </c>
-      <c r="E20" s="1" t="s">
-        <v>254</v>
-      </c>
-      <c r="F20" s="1" t="s">
-        <v>253</v>
       </c>
     </row>
     <row r="21" spans="2:6" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B21" s="3" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="C21" s="3">
         <v>300</v>
       </c>
       <c r="D21" s="1" t="s">
+        <v>233</v>
+      </c>
+      <c r="E21" s="1" t="s">
         <v>234</v>
       </c>
-      <c r="E21" s="1" t="s">
-        <v>235</v>
-      </c>
       <c r="F21" s="1" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="22" spans="2:6" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B22" s="3" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="C22" s="3">
         <v>500</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
     </row>
     <row r="23" spans="2:6" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B23" s="3" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="C23" s="3">
         <v>100</v>
       </c>
       <c r="D23" s="1" t="s">
+        <v>316</v>
+      </c>
+      <c r="E23" s="1" t="s">
         <v>317</v>
       </c>
-      <c r="E23" s="1" t="s">
+      <c r="F23" s="1" t="s">
         <v>318</v>
-      </c>
-      <c r="F23" s="1" t="s">
-        <v>319</v>
       </c>
     </row>
     <row r="24" spans="2:6" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B24" s="3" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="C24" s="3">
         <v>500</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
     </row>
     <row r="25" spans="2:6" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B25" s="3" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="C25" s="3">
         <v>200</v>
       </c>
       <c r="D25" s="1" t="s">
+        <v>323</v>
+      </c>
+      <c r="E25" s="1" t="s">
         <v>324</v>
       </c>
-      <c r="E25" s="1" t="s">
+      <c r="F25" s="1" t="s">
         <v>325</v>
-      </c>
-      <c r="F25" s="1" t="s">
-        <v>326</v>
       </c>
     </row>
     <row r="26" spans="2:6" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B26" s="3" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="C26" s="3">
         <v>400</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
     </row>
     <row r="27" spans="2:6" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B27" s="3" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="C27" s="3">
         <v>500</v>
       </c>
       <c r="D27" s="1" t="s">
+        <v>384</v>
+      </c>
+      <c r="E27" s="1" t="s">
         <v>385</v>
       </c>
-      <c r="E27" s="1" t="s">
-        <v>386</v>
-      </c>
       <c r="F27" s="1" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
     </row>
     <row r="28" spans="2:6" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B28" s="3" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="C28" s="3">
         <v>2000</v>
       </c>
       <c r="D28" s="1" t="s">
+        <v>442</v>
+      </c>
+      <c r="E28" s="1" t="s">
         <v>443</v>
       </c>
-      <c r="E28" s="1" t="s">
+      <c r="F28" s="1" t="s">
         <v>444</v>
-      </c>
-      <c r="F28" s="1" t="s">
-        <v>445</v>
       </c>
     </row>
     <row r="29" spans="2:6" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B29" s="3" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="C29" s="3">
         <v>2300</v>
       </c>
       <c r="D29" s="1" t="s">
+        <v>458</v>
+      </c>
+      <c r="E29" s="1" t="s">
         <v>459</v>
       </c>
-      <c r="E29" s="1" t="s">
+      <c r="F29" s="1" t="s">
         <v>460</v>
-      </c>
-      <c r="F29" s="1" t="s">
-        <v>461</v>
       </c>
     </row>
     <row r="30" spans="2:6" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B30" s="3" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="C30" s="3">
         <v>5000</v>
       </c>
       <c r="D30" s="1" t="s">
+        <v>622</v>
+      </c>
+      <c r="E30" s="1" t="s">
+        <v>477</v>
+      </c>
+      <c r="F30" s="1" t="s">
         <v>478</v>
-      </c>
-      <c r="E30" s="1" t="s">
-        <v>479</v>
-      </c>
-      <c r="F30" s="1" t="s">
-        <v>480</v>
       </c>
     </row>
     <row r="31" spans="2:6" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B31" s="3" t="s">
+        <v>502</v>
+      </c>
+      <c r="C31" s="7">
+        <v>1294</v>
+      </c>
+      <c r="D31" s="1" t="s">
+        <v>503</v>
+      </c>
+      <c r="E31" s="1" t="s">
         <v>504</v>
       </c>
-      <c r="C31" s="13">
-        <v>1294</v>
-      </c>
-      <c r="D31" s="1" t="s">
+      <c r="F31" s="1" t="s">
         <v>505</v>
-      </c>
-      <c r="E31" s="1" t="s">
-        <v>506</v>
-      </c>
-      <c r="F31" s="1" t="s">
-        <v>507</v>
       </c>
     </row>
     <row r="32" spans="2:6" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B32" s="3" t="s">
+        <v>506</v>
+      </c>
+      <c r="C32" s="7">
+        <v>1933</v>
+      </c>
+      <c r="D32" s="1" t="s">
+        <v>507</v>
+      </c>
+      <c r="E32" s="1" t="s">
         <v>508</v>
       </c>
-      <c r="C32" s="13">
-        <v>1933</v>
-      </c>
-      <c r="D32" s="1" t="s">
+      <c r="F32" s="4" t="s">
         <v>509</v>
-      </c>
-      <c r="E32" s="1" t="s">
-        <v>510</v>
-      </c>
-      <c r="F32" s="4" t="s">
-        <v>511</v>
       </c>
     </row>
     <row r="33" ht="59.25" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -4427,20 +4656,18 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{78C3E1C2-3C44-2549-B6BE-21FD6EE1DD33}">
-  <dimension ref="B1:F45"/>
+  <dimension ref="B1:G45"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="10.83203125" style="1"/>
-    <col min="2" max="3" width="28" style="1" customWidth="1"/>
-    <col min="4" max="4" width="28" style="7" customWidth="1"/>
-    <col min="5" max="5" width="30" style="7" customWidth="1"/>
-    <col min="6" max="6" width="28" style="7" customWidth="1"/>
-    <col min="7" max="7" width="28" style="1" customWidth="1"/>
-    <col min="8" max="16384" width="10.83203125" style="1"/>
+    <col min="1" max="1" width="10.83203125" style="8"/>
+    <col min="2" max="4" width="28" style="8" customWidth="1"/>
+    <col min="5" max="5" width="30" style="8" customWidth="1"/>
+    <col min="6" max="7" width="28" style="8" customWidth="1"/>
+    <col min="8" max="16384" width="10.83203125" style="8"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:6" ht="22" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="2" spans="2:6" s="12" customFormat="1" ht="58" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:6" s="12" customFormat="1" ht="58" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B2" s="12" t="s">
         <v>0</v>
       </c>
@@ -4454,564 +4681,597 @@
         <v>7</v>
       </c>
       <c r="F2" s="12" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="3" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B3" s="1" t="s">
+      <c r="B3" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="C3" s="5">
+      <c r="C3" s="13">
         <v>13000</v>
       </c>
-      <c r="D3" s="7" t="s">
+      <c r="D3" s="8" t="s">
+        <v>178</v>
+      </c>
+      <c r="E3" s="8" t="s">
         <v>179</v>
       </c>
-      <c r="E3" s="7" t="s">
+      <c r="F3" s="8" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="4" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B4" s="8" t="s">
+        <v>181</v>
+      </c>
+      <c r="C4" s="8">
+        <v>500</v>
+      </c>
+      <c r="D4" s="8" t="s">
+        <v>182</v>
+      </c>
+      <c r="E4" s="8" t="s">
+        <v>186</v>
+      </c>
+      <c r="F4" s="8" t="s">
         <v>180</v>
       </c>
-      <c r="F3" s="7" t="s">
-        <v>224</v>
-      </c>
-    </row>
-    <row r="4" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B4" s="1" t="s">
-        <v>182</v>
-      </c>
-      <c r="C4" s="1">
-        <v>500</v>
-      </c>
-      <c r="D4" s="7" t="s">
+    </row>
+    <row r="5" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B5" s="8" t="s">
+        <v>184</v>
+      </c>
+      <c r="C5" s="8">
+        <v>130</v>
+      </c>
+      <c r="D5" s="8" t="s">
+        <v>185</v>
+      </c>
+      <c r="E5" s="8" t="s">
+        <v>187</v>
+      </c>
+      <c r="F5" s="8" t="s">
         <v>183</v>
       </c>
-      <c r="E4" s="7" t="s">
-        <v>187</v>
-      </c>
-      <c r="F4" s="7" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="5" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B5" s="1" t="s">
-        <v>185</v>
-      </c>
-      <c r="C5" s="1">
-        <v>130</v>
-      </c>
-      <c r="D5" s="7" t="s">
-        <v>186</v>
-      </c>
-      <c r="E5" s="7" t="s">
+    </row>
+    <row r="6" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B6" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="C6" s="8" t="s">
+        <v>191</v>
+      </c>
+      <c r="D6" s="8" t="s">
+        <v>189</v>
+      </c>
+      <c r="E6" s="8" t="s">
         <v>188</v>
       </c>
-      <c r="F5" s="7" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="6" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B6" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="C6" s="1" t="s">
+      <c r="F6" s="8" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="7" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B7" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="C7" s="8" t="s">
+        <v>195</v>
+      </c>
+      <c r="D7" s="8" t="s">
+        <v>193</v>
+      </c>
+      <c r="E7" s="8" t="s">
+        <v>194</v>
+      </c>
+      <c r="F7" s="8" t="s">
         <v>192</v>
       </c>
-      <c r="D6" s="7" t="s">
-        <v>190</v>
-      </c>
-      <c r="E6" s="7" t="s">
-        <v>189</v>
-      </c>
-      <c r="F6" s="7" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="7" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B7" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="C7" s="1" t="s">
+    </row>
+    <row r="8" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B8" s="8" t="s">
+        <v>198</v>
+      </c>
+      <c r="C8" s="8">
+        <v>70</v>
+      </c>
+      <c r="D8" s="8" t="s">
         <v>196</v>
       </c>
-      <c r="D7" s="7" t="s">
-        <v>194</v>
-      </c>
-      <c r="E7" s="7" t="s">
-        <v>195</v>
-      </c>
-      <c r="F7" s="7" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="8" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B8" s="1" t="s">
+      <c r="E8" s="8" t="s">
+        <v>197</v>
+      </c>
+      <c r="F8" s="8" t="s">
         <v>199</v>
       </c>
-      <c r="C8" s="1">
-        <v>70</v>
-      </c>
-      <c r="D8" s="7" t="s">
-        <v>197</v>
-      </c>
-      <c r="E8" s="7" t="s">
-        <v>198</v>
-      </c>
-      <c r="F8" s="7" t="s">
+    </row>
+    <row r="9" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B9" s="8" t="s">
         <v>200</v>
       </c>
-    </row>
-    <row r="9" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B9" s="1" t="s">
+      <c r="C9" s="13">
+        <v>10000</v>
+      </c>
+      <c r="D9" s="8" t="s">
         <v>201</v>
       </c>
-      <c r="C9" s="5">
-        <v>10000</v>
-      </c>
-      <c r="D9" s="7" t="s">
+      <c r="E9" s="8" t="s">
         <v>202</v>
       </c>
-      <c r="E9" s="7" t="s">
+      <c r="F9" s="8" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="10" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B10" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="C10" s="8">
+        <v>100</v>
+      </c>
+      <c r="D10" s="8" t="s">
+        <v>205</v>
+      </c>
+      <c r="E10" s="8" t="s">
+        <v>95</v>
+      </c>
+      <c r="F10" s="8" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="11" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B11" s="8" t="s">
+        <v>76</v>
+      </c>
+      <c r="C11" s="8" t="s">
+        <v>210</v>
+      </c>
+      <c r="D11" s="8" t="s">
+        <v>207</v>
+      </c>
+      <c r="E11" s="8" t="s">
+        <v>208</v>
+      </c>
+      <c r="F11" s="8" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="12" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B12" s="8" t="s">
+        <v>122</v>
+      </c>
+      <c r="C12" s="13">
+        <v>5500</v>
+      </c>
+      <c r="D12" s="8" t="s">
+        <v>211</v>
+      </c>
+      <c r="E12" s="8" t="s">
+        <v>212</v>
+      </c>
+      <c r="F12" s="8" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="13" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B13" s="8" t="s">
         <v>203</v>
       </c>
-      <c r="F9" s="7" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="10" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B10" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="C10" s="1">
+      <c r="C13" s="8" t="s">
+        <v>215</v>
+      </c>
+      <c r="D13" s="8" t="s">
+        <v>213</v>
+      </c>
+      <c r="E13" s="8" t="s">
+        <v>204</v>
+      </c>
+      <c r="F13" s="8" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="14" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B14" s="8" t="s">
+        <v>206</v>
+      </c>
+      <c r="C14" s="13">
+        <v>4500</v>
+      </c>
+      <c r="D14" s="8" t="s">
+        <v>217</v>
+      </c>
+      <c r="E14" s="8" t="s">
+        <v>218</v>
+      </c>
+      <c r="F14" s="8" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="15" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B15" s="8" t="s">
+        <v>214</v>
+      </c>
+      <c r="C15" s="8">
+        <v>20</v>
+      </c>
+      <c r="D15" s="8" t="s">
+        <v>219</v>
+      </c>
+      <c r="E15" s="8" t="s">
+        <v>220</v>
+      </c>
+      <c r="F15" s="8" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="16" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B16" s="8" t="s">
+        <v>238</v>
+      </c>
+      <c r="C16" s="8">
+        <v>20</v>
+      </c>
+      <c r="D16" s="8" t="s">
+        <v>236</v>
+      </c>
+      <c r="E16" s="8" t="s">
+        <v>239</v>
+      </c>
+      <c r="F16" s="8" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="17" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B17" s="8" t="s">
+        <v>246</v>
+      </c>
+      <c r="C17" s="8">
+        <v>150</v>
+      </c>
+      <c r="D17" s="8" t="s">
+        <v>247</v>
+      </c>
+      <c r="E17" s="8" t="s">
+        <v>248</v>
+      </c>
+      <c r="F17" s="8" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="18" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B18" s="8" t="s">
+        <v>307</v>
+      </c>
+      <c r="C18" s="8">
+        <v>1000</v>
+      </c>
+      <c r="D18" s="8" t="s">
+        <v>309</v>
+      </c>
+      <c r="E18" s="8" t="s">
+        <v>308</v>
+      </c>
+      <c r="F18" s="10" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="19" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B19" s="8" t="s">
+        <v>327</v>
+      </c>
+      <c r="C19" s="8">
+        <v>20</v>
+      </c>
+      <c r="D19" s="8" t="s">
+        <v>328</v>
+      </c>
+      <c r="E19" s="10" t="s">
+        <v>329</v>
+      </c>
+      <c r="F19" s="11" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="20" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B20" s="8" t="s">
+        <v>332</v>
+      </c>
+      <c r="C20" s="8">
+        <v>50</v>
+      </c>
+      <c r="D20" s="8" t="s">
+        <v>330</v>
+      </c>
+      <c r="E20" s="8" t="s">
+        <v>331</v>
+      </c>
+      <c r="F20" s="8" t="s">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="21" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B21" s="8" t="s">
+        <v>392</v>
+      </c>
+      <c r="C21" s="8">
+        <v>50</v>
+      </c>
+      <c r="D21" s="8" t="s">
+        <v>391</v>
+      </c>
+      <c r="E21" s="8" t="s">
+        <v>394</v>
+      </c>
+      <c r="F21" s="8" t="s">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="22" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B22" s="8" t="s">
+        <v>395</v>
+      </c>
+      <c r="C22" s="8" t="s">
+        <v>387</v>
+      </c>
+      <c r="D22" s="8" t="s">
+        <v>396</v>
+      </c>
+      <c r="E22" s="8" t="s">
+        <v>397</v>
+      </c>
+      <c r="F22" s="8" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="23" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B23" s="8" t="s">
+        <v>399</v>
+      </c>
+      <c r="C23" s="8">
         <v>100</v>
       </c>
-      <c r="D10" s="7" t="s">
-        <v>206</v>
-      </c>
-      <c r="E10" s="7" t="s">
-        <v>96</v>
-      </c>
-      <c r="F10" s="7" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="11" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B11" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="C11" s="1" t="s">
-        <v>211</v>
-      </c>
-      <c r="D11" s="7" t="s">
-        <v>208</v>
-      </c>
-      <c r="E11" s="7" t="s">
-        <v>209</v>
-      </c>
-      <c r="F11" s="7" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="12" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B12" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="C12" s="5">
-        <v>5500</v>
-      </c>
-      <c r="D12" s="7" t="s">
-        <v>212</v>
-      </c>
-      <c r="E12" s="7" t="s">
-        <v>213</v>
-      </c>
-      <c r="F12" s="7" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="13" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B13" s="1" t="s">
-        <v>204</v>
-      </c>
-      <c r="C13" s="1" t="s">
-        <v>216</v>
-      </c>
-      <c r="D13" s="7" t="s">
-        <v>214</v>
-      </c>
-      <c r="E13" s="7" t="s">
-        <v>205</v>
-      </c>
-      <c r="F13" s="7" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="14" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B14" s="1" t="s">
-        <v>207</v>
-      </c>
-      <c r="C14" s="5">
-        <v>4500</v>
-      </c>
-      <c r="D14" s="7" t="s">
-        <v>218</v>
-      </c>
-      <c r="E14" s="7" t="s">
-        <v>219</v>
-      </c>
-      <c r="F14" s="7" t="s">
-        <v>288</v>
-      </c>
-    </row>
-    <row r="15" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B15" s="1" t="s">
-        <v>215</v>
-      </c>
-      <c r="C15" s="1">
+      <c r="D23" s="8" t="s">
+        <v>400</v>
+      </c>
+      <c r="E23" s="8" t="s">
+        <v>398</v>
+      </c>
+      <c r="F23" s="8" t="s">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="24" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B24" s="8" t="s">
+        <v>363</v>
+      </c>
+      <c r="C24" s="8">
+        <v>10</v>
+      </c>
+      <c r="D24" s="8" t="s">
+        <v>364</v>
+      </c>
+      <c r="E24" s="8" t="s">
+        <v>365</v>
+      </c>
+      <c r="F24" s="8" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="25" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B25" s="8" t="s">
+        <v>402</v>
+      </c>
+      <c r="C25" s="8">
         <v>20</v>
       </c>
-      <c r="D15" s="7" t="s">
-        <v>220</v>
-      </c>
-      <c r="E15" s="7" t="s">
-        <v>221</v>
-      </c>
-      <c r="F15" s="7" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="16" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B16" s="1" t="s">
-        <v>239</v>
-      </c>
-      <c r="C16" s="1">
+      <c r="D25" s="8" t="s">
+        <v>403</v>
+      </c>
+      <c r="E25" s="8" t="s">
+        <v>405</v>
+      </c>
+      <c r="F25" s="8" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="26" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B26" s="8" t="s">
+        <v>406</v>
+      </c>
+      <c r="C26" s="8">
+        <v>1000</v>
+      </c>
+      <c r="D26" s="8" t="s">
+        <v>407</v>
+      </c>
+      <c r="E26" s="8" t="s">
+        <v>409</v>
+      </c>
+      <c r="F26" s="8" t="s">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="27" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B27" s="8" t="s">
+        <v>411</v>
+      </c>
+      <c r="C27" s="8">
+        <v>200</v>
+      </c>
+      <c r="D27" s="8" t="s">
+        <v>410</v>
+      </c>
+      <c r="E27" s="8" t="s">
+        <v>412</v>
+      </c>
+      <c r="F27" s="8" t="s">
+        <v>414</v>
+      </c>
+    </row>
+    <row r="28" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B28" s="8" t="s">
+        <v>413</v>
+      </c>
+      <c r="C28" s="8">
+        <v>10</v>
+      </c>
+      <c r="D28" s="8" t="s">
+        <v>415</v>
+      </c>
+      <c r="E28" s="8" t="s">
+        <v>416</v>
+      </c>
+      <c r="F28" s="8" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="29" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B29" s="8" t="s">
+        <v>417</v>
+      </c>
+      <c r="C29" s="8">
+        <v>35</v>
+      </c>
+      <c r="D29" s="8" t="s">
+        <v>420</v>
+      </c>
+      <c r="E29" s="8" t="s">
+        <v>422</v>
+      </c>
+      <c r="F29" s="8" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="30" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B30" s="8" t="s">
+        <v>426</v>
+      </c>
+      <c r="C30" s="8">
+        <v>80</v>
+      </c>
+      <c r="D30" s="8" t="s">
+        <v>423</v>
+      </c>
+      <c r="E30" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="F30" s="8" t="s">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="31" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B31" s="8" t="s">
+        <v>418</v>
+      </c>
+      <c r="C31" s="8">
         <v>20</v>
       </c>
-      <c r="D16" s="7" t="s">
-        <v>237</v>
-      </c>
-      <c r="E16" s="7" t="s">
-        <v>240</v>
-      </c>
-      <c r="F16" s="7" t="s">
-        <v>238</v>
-      </c>
-    </row>
-    <row r="17" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B17" s="1" t="s">
-        <v>247</v>
-      </c>
-      <c r="C17" s="1">
-        <v>150</v>
-      </c>
-      <c r="D17" s="7" t="s">
-        <v>248</v>
-      </c>
-      <c r="E17" s="7" t="s">
-        <v>249</v>
-      </c>
-      <c r="F17" s="7" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="18" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B18" s="1" t="s">
-        <v>308</v>
-      </c>
-      <c r="C18" s="1">
-        <v>1000</v>
-      </c>
-      <c r="D18" s="7" t="s">
-        <v>310</v>
-      </c>
-      <c r="E18" s="7" t="s">
-        <v>309</v>
-      </c>
-      <c r="F18" s="8" t="s">
-        <v>311</v>
-      </c>
-    </row>
-    <row r="19" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B19" s="1" t="s">
-        <v>328</v>
-      </c>
-      <c r="C19" s="1">
-        <v>20</v>
-      </c>
-      <c r="D19" s="7" t="s">
-        <v>329</v>
-      </c>
-      <c r="E19" s="10" t="s">
-        <v>330</v>
-      </c>
-      <c r="F19" s="9" t="s">
+      <c r="D31" s="8" t="s">
+        <v>427</v>
+      </c>
+      <c r="E31" s="8" t="s">
+        <v>428</v>
+      </c>
+      <c r="F31" s="8" t="s">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="32" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B32" s="8" t="s">
+        <v>419</v>
+      </c>
+      <c r="C32" s="8">
+        <v>40</v>
+      </c>
+      <c r="D32" s="8" t="s">
+        <v>431</v>
+      </c>
+      <c r="E32" s="8" t="s">
+        <v>432</v>
+      </c>
+      <c r="F32" s="8" t="s">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="33" spans="2:7" ht="58" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B33" s="8" t="s">
+        <v>434</v>
+      </c>
+      <c r="C33" s="8">
+        <v>104</v>
+      </c>
+      <c r="D33" s="8" t="s">
+        <v>437</v>
+      </c>
+      <c r="E33" s="8" t="s">
+        <v>436</v>
+      </c>
+      <c r="F33" s="8" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="34" spans="2:7" ht="58" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B34" s="8" t="s">
+        <v>560</v>
+      </c>
+      <c r="C34" s="8">
         <v>200</v>
       </c>
-    </row>
-    <row r="20" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B20" s="1" t="s">
-        <v>333</v>
-      </c>
-      <c r="C20" s="1">
+      <c r="D34" s="8" t="s">
+        <v>561</v>
+      </c>
+      <c r="E34" s="8" t="s">
+        <v>562</v>
+      </c>
+      <c r="F34" s="8" t="s">
+        <v>559</v>
+      </c>
+    </row>
+    <row r="35" spans="2:7" ht="58" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B35" s="8" t="s">
+        <v>617</v>
+      </c>
+      <c r="C35" s="8">
         <v>50</v>
       </c>
-      <c r="D20" s="7" t="s">
-        <v>331</v>
-      </c>
-      <c r="E20" s="7" t="s">
-        <v>332</v>
-      </c>
-      <c r="F20" s="7" t="s">
-        <v>334</v>
-      </c>
-    </row>
-    <row r="21" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B21" s="1" t="s">
-        <v>393</v>
-      </c>
-      <c r="C21" s="1">
-        <v>50</v>
-      </c>
-      <c r="D21" s="7" t="s">
-        <v>392</v>
-      </c>
-      <c r="E21" s="7" t="s">
-        <v>395</v>
-      </c>
-      <c r="F21" s="7" t="s">
-        <v>394</v>
-      </c>
-    </row>
-    <row r="22" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B22" s="1" t="s">
-        <v>396</v>
-      </c>
-      <c r="C22" s="1" t="s">
-        <v>388</v>
-      </c>
-      <c r="D22" s="7" t="s">
-        <v>397</v>
-      </c>
-      <c r="E22" s="7" t="s">
-        <v>398</v>
-      </c>
-      <c r="F22" s="7" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="23" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B23" s="1" t="s">
-        <v>400</v>
-      </c>
-      <c r="C23" s="1">
-        <v>100</v>
-      </c>
-      <c r="D23" s="7" t="s">
-        <v>401</v>
-      </c>
-      <c r="E23" s="7" t="s">
-        <v>399</v>
-      </c>
-      <c r="F23" s="7" t="s">
-        <v>402</v>
-      </c>
-    </row>
-    <row r="24" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B24" s="1" t="s">
-        <v>364</v>
-      </c>
-      <c r="C24" s="1">
+      <c r="D35" s="6" t="s">
+        <v>620</v>
+      </c>
+      <c r="E35" s="8" t="s">
+        <v>618</v>
+      </c>
+      <c r="F35" s="8" t="s">
+        <v>619</v>
+      </c>
+    </row>
+    <row r="36" spans="2:7" ht="58" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B36" s="15" t="s">
+        <v>642</v>
+      </c>
+      <c r="C36" s="8">
         <v>10</v>
       </c>
-      <c r="D24" s="1" t="s">
-        <v>365</v>
-      </c>
-      <c r="E24" s="1" t="s">
-        <v>366</v>
-      </c>
-      <c r="F24" s="1" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="25" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B25" s="1" t="s">
-        <v>403</v>
-      </c>
-      <c r="C25" s="1">
-        <v>20</v>
-      </c>
-      <c r="D25" s="1" t="s">
-        <v>404</v>
-      </c>
-      <c r="E25" s="7" t="s">
-        <v>406</v>
-      </c>
-      <c r="F25" s="7" t="s">
-        <v>405</v>
-      </c>
-    </row>
-    <row r="26" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B26" s="1" t="s">
-        <v>407</v>
-      </c>
-      <c r="C26" s="1">
-        <v>1000</v>
-      </c>
-      <c r="D26" s="7" t="s">
-        <v>408</v>
-      </c>
-      <c r="E26" s="7" t="s">
-        <v>410</v>
-      </c>
-      <c r="F26" s="7" t="s">
-        <v>409</v>
-      </c>
-    </row>
-    <row r="27" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B27" s="1" t="s">
-        <v>412</v>
-      </c>
-      <c r="C27" s="1">
-        <v>200</v>
-      </c>
-      <c r="D27" s="7" t="s">
-        <v>411</v>
-      </c>
-      <c r="E27" s="7" t="s">
-        <v>413</v>
-      </c>
-      <c r="F27" s="7" t="s">
-        <v>415</v>
-      </c>
-    </row>
-    <row r="28" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B28" s="1" t="s">
-        <v>414</v>
-      </c>
-      <c r="C28" s="1">
-        <v>10</v>
-      </c>
-      <c r="D28" s="7" t="s">
-        <v>416</v>
-      </c>
-      <c r="E28" s="7" t="s">
-        <v>417</v>
-      </c>
-      <c r="F28" s="7" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="29" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B29" s="1" t="s">
-        <v>418</v>
-      </c>
-      <c r="C29" s="1">
-        <v>35</v>
-      </c>
-      <c r="D29" s="7" t="s">
-        <v>421</v>
-      </c>
-      <c r="E29" s="7" t="s">
-        <v>423</v>
-      </c>
-      <c r="F29" s="7" t="s">
-        <v>422</v>
-      </c>
-    </row>
-    <row r="30" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B30" s="1" t="s">
-        <v>427</v>
-      </c>
-      <c r="C30" s="1">
-        <v>80</v>
-      </c>
-      <c r="D30" s="7" t="s">
-        <v>424</v>
-      </c>
-      <c r="E30" s="7" t="s">
-        <v>425</v>
-      </c>
-      <c r="F30" s="7" t="s">
-        <v>426</v>
-      </c>
-    </row>
-    <row r="31" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B31" s="1" t="s">
-        <v>419</v>
-      </c>
-      <c r="C31" s="1">
-        <v>20</v>
-      </c>
-      <c r="D31" s="7" t="s">
-        <v>428</v>
-      </c>
-      <c r="E31" s="7" t="s">
-        <v>429</v>
-      </c>
-      <c r="F31" s="7" t="s">
-        <v>430</v>
-      </c>
-    </row>
-    <row r="32" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B32" s="1" t="s">
-        <v>420</v>
-      </c>
-      <c r="C32" s="1">
-        <v>40</v>
-      </c>
-      <c r="D32" s="7" t="s">
-        <v>432</v>
-      </c>
-      <c r="E32" s="7" t="s">
-        <v>433</v>
-      </c>
-      <c r="F32" s="7" t="s">
-        <v>431</v>
-      </c>
-    </row>
-    <row r="33" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B33" s="3" t="s">
-        <v>435</v>
-      </c>
-      <c r="C33" s="3">
-        <v>104</v>
-      </c>
-      <c r="D33" s="1" t="s">
-        <v>438</v>
-      </c>
-      <c r="E33" s="1" t="s">
-        <v>437</v>
-      </c>
-      <c r="F33" s="1" t="s">
-        <v>434</v>
-      </c>
-    </row>
-    <row r="34" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B34" s="3" t="s">
-        <v>563</v>
-      </c>
-      <c r="C34" s="3">
-        <v>200</v>
-      </c>
-      <c r="D34" s="1" t="s">
-        <v>564</v>
-      </c>
-      <c r="E34" s="1" t="s">
-        <v>565</v>
-      </c>
-      <c r="F34" s="1" t="s">
-        <v>562</v>
-      </c>
-    </row>
-    <row r="35" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="36" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="37" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="38" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="39" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="40" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="41" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="42" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="43" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="44" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="45" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2"/>
+      <c r="D36" s="16" t="s">
+        <v>643</v>
+      </c>
+      <c r="E36" s="8" t="s">
+        <v>644</v>
+      </c>
+      <c r="F36" s="6" t="s">
+        <v>645</v>
+      </c>
+      <c r="G36" s="14"/>
+    </row>
+    <row r="37" spans="2:7" ht="58" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="38" spans="2:7" ht="58" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="39" spans="2:7" ht="58" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="40" spans="2:7" ht="58" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="41" spans="2:7" ht="58" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="42" spans="2:7" ht="58" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="43" spans="2:7" ht="58" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="44" spans="2:7" ht="58" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="45" spans="2:7" ht="58" customHeight="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -5043,7 +5303,7 @@
         <v>7</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="3" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -5051,16 +5311,16 @@
         <v>16</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>18</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="4" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -5068,118 +5328,118 @@
         <v>17</v>
       </c>
       <c r="C4" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="D4" s="1" t="s">
         <v>144</v>
       </c>
-      <c r="D4" s="1" t="s">
-        <v>145</v>
-      </c>
       <c r="E4" s="1" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="5" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="C5" s="3" t="s">
         <v>143</v>
       </c>
-      <c r="C5" s="3" t="s">
-        <v>144</v>
-      </c>
       <c r="D5" s="1" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="6" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="3" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="C6" s="3">
         <v>40</v>
       </c>
       <c r="D6" s="1" t="s">
+        <v>300</v>
+      </c>
+      <c r="E6" s="1" t="s">
         <v>301</v>
       </c>
-      <c r="E6" s="1" t="s">
+      <c r="F6" s="1" t="s">
         <v>302</v>
-      </c>
-      <c r="F6" s="1" t="s">
-        <v>303</v>
       </c>
     </row>
     <row r="7" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B7" s="3" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="C7" s="3">
         <v>50</v>
       </c>
       <c r="D7" s="1" t="s">
+        <v>340</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>342</v>
+      </c>
+      <c r="F7" s="1" t="s">
         <v>341</v>
-      </c>
-      <c r="E7" s="1" t="s">
-        <v>343</v>
-      </c>
-      <c r="F7" s="1" t="s">
-        <v>342</v>
       </c>
     </row>
     <row r="8" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B8" s="3" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="C8" s="3">
         <v>300</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="E8" s="1" t="s">
+        <v>375</v>
+      </c>
+      <c r="F8" s="1" t="s">
         <v>376</v>
-      </c>
-      <c r="F8" s="1" t="s">
-        <v>377</v>
       </c>
     </row>
     <row r="9" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B9" s="3" t="s">
-        <v>581</v>
+        <v>578</v>
       </c>
       <c r="C9" s="3">
         <v>5</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>582</v>
+        <v>579</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>583</v>
+        <v>580</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="10" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="3" t="s">
-        <v>588</v>
+        <v>585</v>
       </c>
       <c r="C10" s="3">
         <v>15</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>589</v>
+        <v>586</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>590</v>
+        <v>587</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>591</v>
+        <v>588</v>
       </c>
     </row>
     <row r="11" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25"/>

</xml_diff>

<commit_message>
added 1 SU 1 LC
</commit_message>
<xml_diff>
--- a/Photonic Companies.xlsx
+++ b/Photonic Companies.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/blow/Desktop/GitHub/PhotonicCompanies/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D71614C-B2B9-0F42-B3A3-128B1EDAF3F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{629F32E4-6996-9847-A81C-F00E30FB6745}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="620" windowWidth="28800" windowHeight="15660" activeTab="2" xr2:uid="{EBDBD758-277E-6B49-B4C7-31ED6652B0E7}"/>
+    <workbookView xWindow="0" yWindow="620" windowWidth="28800" windowHeight="15660" xr2:uid="{EBDBD758-277E-6B49-B4C7-31ED6652B0E7}"/>
   </bookViews>
   <sheets>
     <sheet name="Startup" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="709" uniqueCount="646">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="717" uniqueCount="654">
   <si>
     <t>Company Name</t>
   </si>
@@ -742,9 +742,6 @@
   </si>
   <si>
     <t>photonics chipset developer/supplier for high-volume sensor and communication products.</t>
-  </si>
-  <si>
-    <t>CEO: Richard Meier</t>
   </si>
   <si>
     <t>hown an interest in photonic technologies and the benefits of ultra-fast data communication</t>
@@ -2055,6 +2052,33 @@
   </si>
   <si>
     <t>Austin, Texas</t>
+  </si>
+  <si>
+    <t>CEO: Richard Meier, files for bankruptcy</t>
+  </si>
+  <si>
+    <t>Astera Labs</t>
+  </si>
+  <si>
+    <t>Rack-scale AI and cloud infrastructure connectivity, Scorpio smart fabric switches, and COSMOS</t>
+  </si>
+  <si>
+    <t>CEO/co-founder Jitendra Mohan; President &amp; COO/co-founder Sanjay Gajendra</t>
+  </si>
+  <si>
+    <t xml:space="preserve">San Jose, California and Austin, Texas and  Aachen, Germany and Ahmedabad, India and Bengaluru, India and Haifa, Israel and Ho Chi Minh City, Vietnam and Hyderabad, India and Irvine, California and Seattle, United States and Shanghai, China and Singapore, Singapore and Taipei, Taiwan and Tel Aviv, Israel and Toronto, Canada and Vancouver, Canada </t>
+  </si>
+  <si>
+    <t>Lumilens</t>
+  </si>
+  <si>
+    <t>$133.4M raised, Photonic interconnects for AI data centers and HPC: scale-up and scale-out optical interconnects, high-density pluggables, near-package optics, co-packaged optics, GPU-to-GPU connectivity, and automated/robotics-driven photonics manufacturing</t>
+  </si>
+  <si>
+    <t>Ankur Singla, CEO, Ying Huang, VP Silicon Photonics</t>
+  </si>
+  <si>
+    <t>San Jose, California and Singapore and Thailand and Bengaluru, India</t>
   </si>
 </sst>
 </file>
@@ -2140,7 +2164,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -2163,13 +2187,10 @@
     <xf numFmtId="3" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -2178,7 +2199,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -2661,7 +2682,7 @@
         <v>20</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
       <c r="E9" s="1" t="s">
         <v>45</v>
@@ -3063,305 +3084,305 @@
     </row>
     <row r="33" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B33" s="3" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="C33" s="3">
         <v>10</v>
       </c>
       <c r="D33" s="1" t="s">
+        <v>242</v>
+      </c>
+      <c r="E33" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="F33" s="1" t="s">
         <v>243</v>
-      </c>
-      <c r="E33" s="1" t="s">
-        <v>245</v>
-      </c>
-      <c r="F33" s="1" t="s">
-        <v>244</v>
       </c>
     </row>
     <row r="34" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B34" s="3" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="C34" s="3">
         <v>190</v>
       </c>
       <c r="D34" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="E34" s="1" t="s">
+        <v>295</v>
+      </c>
+      <c r="F34" s="1" t="s">
         <v>290</v>
-      </c>
-      <c r="E34" s="1" t="s">
-        <v>296</v>
-      </c>
-      <c r="F34" s="1" t="s">
-        <v>291</v>
       </c>
     </row>
     <row r="35" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B35" s="3" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="C35" s="3">
         <v>30</v>
       </c>
       <c r="D35" s="1" t="s">
+        <v>292</v>
+      </c>
+      <c r="E35" s="1" t="s">
         <v>293</v>
       </c>
-      <c r="E35" s="1" t="s">
+      <c r="F35" s="1" t="s">
         <v>294</v>
-      </c>
-      <c r="F35" s="1" t="s">
-        <v>295</v>
       </c>
     </row>
     <row r="36" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B36" s="3" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C36" s="3">
         <v>15</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="E36" s="1" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="F36" s="1" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
     </row>
     <row r="37" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B37" s="3" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="C37" s="3">
         <v>40</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="E37" s="1" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="F37" s="1" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
     </row>
     <row r="38" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B38" s="3" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="C38" s="3">
         <v>30</v>
       </c>
       <c r="D38" s="1" t="s">
+        <v>311</v>
+      </c>
+      <c r="E38" s="1" t="s">
         <v>312</v>
       </c>
-      <c r="E38" s="1" t="s">
+      <c r="F38" s="1" t="s">
         <v>313</v>
-      </c>
-      <c r="F38" s="1" t="s">
-        <v>314</v>
       </c>
     </row>
     <row r="39" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B39" s="3" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="C39" s="3">
         <v>50</v>
       </c>
       <c r="D39" s="1" t="s">
+        <v>329</v>
+      </c>
+      <c r="E39" s="1" t="s">
         <v>330</v>
       </c>
-      <c r="E39" s="1" t="s">
-        <v>331</v>
-      </c>
       <c r="F39" s="1" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
     </row>
     <row r="40" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B40" s="3" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="C40" s="3">
         <v>20</v>
       </c>
       <c r="D40" s="1" t="s">
+        <v>344</v>
+      </c>
+      <c r="E40" s="1" t="s">
         <v>345</v>
       </c>
-      <c r="E40" s="1" t="s">
-        <v>346</v>
-      </c>
       <c r="F40" s="1" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
     </row>
     <row r="41" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B41" s="3" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="C41" s="3">
         <v>81</v>
       </c>
       <c r="D41" s="1" t="s">
+        <v>347</v>
+      </c>
+      <c r="E41" s="1" t="s">
+        <v>349</v>
+      </c>
+      <c r="F41" s="1" t="s">
         <v>348</v>
-      </c>
-      <c r="E41" s="1" t="s">
-        <v>350</v>
-      </c>
-      <c r="F41" s="1" t="s">
-        <v>349</v>
       </c>
     </row>
     <row r="42" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B42" s="3" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="C42" s="3">
         <v>120</v>
       </c>
       <c r="D42" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="E42" s="1" t="s">
+        <v>353</v>
+      </c>
+      <c r="F42" s="1" t="s">
         <v>352</v>
-      </c>
-      <c r="E42" s="1" t="s">
-        <v>354</v>
-      </c>
-      <c r="F42" s="1" t="s">
-        <v>353</v>
       </c>
     </row>
     <row r="43" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B43" s="3" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="C43" s="3">
         <v>20</v>
       </c>
       <c r="D43" s="1" t="s">
+        <v>355</v>
+      </c>
+      <c r="E43" s="1" t="s">
         <v>356</v>
       </c>
-      <c r="E43" s="1" t="s">
+      <c r="F43" s="1" t="s">
         <v>357</v>
-      </c>
-      <c r="F43" s="1" t="s">
-        <v>358</v>
       </c>
     </row>
     <row r="44" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B44" s="3" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="C44" s="3">
         <v>50</v>
       </c>
       <c r="D44" s="1" t="s">
+        <v>359</v>
+      </c>
+      <c r="E44" s="1" t="s">
         <v>360</v>
       </c>
-      <c r="E44" s="1" t="s">
+      <c r="F44" s="1" t="s">
         <v>361</v>
-      </c>
-      <c r="F44" s="1" t="s">
-        <v>362</v>
       </c>
     </row>
     <row r="45" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B45" s="3" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="C45" s="3">
         <v>20</v>
       </c>
       <c r="D45" s="1" t="s">
+        <v>367</v>
+      </c>
+      <c r="E45" s="1" t="s">
+        <v>366</v>
+      </c>
+      <c r="F45" s="1" t="s">
         <v>368</v>
-      </c>
-      <c r="E45" s="1" t="s">
-        <v>367</v>
-      </c>
-      <c r="F45" s="1" t="s">
-        <v>369</v>
       </c>
     </row>
     <row r="46" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B46" s="3" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="C46" s="3">
         <v>50</v>
       </c>
       <c r="D46" s="1" t="s">
+        <v>370</v>
+      </c>
+      <c r="E46" s="1" t="s">
         <v>371</v>
       </c>
-      <c r="E46" s="1" t="s">
+      <c r="F46" s="1" t="s">
         <v>372</v>
-      </c>
-      <c r="F46" s="1" t="s">
-        <v>373</v>
       </c>
     </row>
     <row r="47" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B47" s="3" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="C47" s="3">
         <v>150</v>
       </c>
       <c r="D47" s="1" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="E47" s="1" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="F47" s="1" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
     </row>
     <row r="48" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B48" s="3" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="C48" s="3">
         <v>3</v>
       </c>
       <c r="D48" s="1" t="s">
+        <v>388</v>
+      </c>
+      <c r="E48" s="1" t="s">
         <v>389</v>
       </c>
-      <c r="E48" s="1" t="s">
-        <v>390</v>
-      </c>
       <c r="F48" s="1" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
     </row>
     <row r="49" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B49" s="3" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="C49" s="3">
         <v>104</v>
       </c>
       <c r="D49" s="1" t="s">
+        <v>434</v>
+      </c>
+      <c r="E49" s="1" t="s">
         <v>435</v>
       </c>
-      <c r="E49" s="1" t="s">
-        <v>436</v>
-      </c>
       <c r="F49" s="1" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
     </row>
     <row r="50" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B50" s="3" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="C50" s="3">
         <v>50</v>
       </c>
       <c r="D50" s="1" t="s">
+        <v>437</v>
+      </c>
+      <c r="E50" s="1" t="s">
         <v>438</v>
-      </c>
-      <c r="E50" s="1" t="s">
-        <v>439</v>
       </c>
       <c r="F50" s="1" t="s">
         <v>59</v>
@@ -3369,203 +3390,203 @@
     </row>
     <row r="51" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B51" s="3" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="C51" s="3">
         <v>26</v>
       </c>
       <c r="D51" s="1" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="E51" s="1" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="F51" s="1" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
     </row>
     <row r="52" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B52" s="3" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
       <c r="C52" s="3">
         <v>21</v>
       </c>
       <c r="D52" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="E52" s="1" t="s">
         <v>451</v>
       </c>
-      <c r="E52" s="1" t="s">
-        <v>452</v>
-      </c>
       <c r="F52" s="1" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
     </row>
     <row r="53" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B53" s="3" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C53" s="3">
         <v>5</v>
       </c>
       <c r="D53" s="1" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
       <c r="E53" s="1" t="s">
+        <v>453</v>
+      </c>
+      <c r="F53" s="1" t="s">
         <v>454</v>
-      </c>
-      <c r="F53" s="1" t="s">
-        <v>455</v>
       </c>
     </row>
     <row r="54" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B54" s="3" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="C54" s="3">
         <v>207</v>
       </c>
       <c r="D54" s="1" t="s">
+        <v>461</v>
+      </c>
+      <c r="E54" s="1" t="s">
         <v>462</v>
       </c>
-      <c r="E54" s="1" t="s">
-        <v>463</v>
-      </c>
       <c r="F54" s="1" t="s">
-        <v>483</v>
+        <v>482</v>
       </c>
     </row>
     <row r="55" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B55" s="3" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="C55" s="3">
         <v>10</v>
       </c>
       <c r="D55" s="1" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="E55" s="1" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="F55" s="1" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
     </row>
     <row r="56" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B56" s="3" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="C56" s="3">
         <v>13</v>
       </c>
       <c r="D56" s="1" t="s">
+        <v>468</v>
+      </c>
+      <c r="E56" s="1" t="s">
+        <v>470</v>
+      </c>
+      <c r="F56" s="1" t="s">
         <v>469</v>
-      </c>
-      <c r="E56" s="1" t="s">
-        <v>471</v>
-      </c>
-      <c r="F56" s="1" t="s">
-        <v>470</v>
       </c>
     </row>
     <row r="57" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B57" s="3" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="C57" s="3">
         <v>5</v>
       </c>
       <c r="D57" s="1" t="s">
+        <v>472</v>
+      </c>
+      <c r="E57" s="1" t="s">
         <v>473</v>
       </c>
-      <c r="E57" s="1" t="s">
+      <c r="F57" s="1" t="s">
         <v>474</v>
-      </c>
-      <c r="F57" s="1" t="s">
-        <v>475</v>
       </c>
     </row>
     <row r="58" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B58" s="3" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="C58" s="3">
         <v>50</v>
       </c>
       <c r="D58" s="1" t="s">
+        <v>479</v>
+      </c>
+      <c r="E58" s="1" t="s">
         <v>480</v>
       </c>
-      <c r="E58" s="1" t="s">
+      <c r="F58" s="1" t="s">
         <v>481</v>
-      </c>
-      <c r="F58" s="1" t="s">
-        <v>482</v>
       </c>
     </row>
     <row r="59" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B59" s="3" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
       <c r="C59" s="3" t="s">
         <v>63</v>
       </c>
       <c r="D59" s="1" t="s">
+        <v>484</v>
+      </c>
+      <c r="E59" s="1" t="s">
         <v>485</v>
       </c>
-      <c r="E59" s="1" t="s">
+      <c r="F59" s="1" t="s">
         <v>486</v>
-      </c>
-      <c r="F59" s="1" t="s">
-        <v>487</v>
       </c>
     </row>
     <row r="60" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B60" s="3" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="C60" s="3" t="s">
         <v>81</v>
       </c>
       <c r="D60" s="1" t="s">
+        <v>487</v>
+      </c>
+      <c r="E60" s="1" t="s">
         <v>488</v>
       </c>
-      <c r="E60" s="1" t="s">
+      <c r="F60" s="1" t="s">
         <v>489</v>
-      </c>
-      <c r="F60" s="1" t="s">
-        <v>490</v>
       </c>
     </row>
     <row r="61" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B61" s="3" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="C61" s="3">
         <v>50</v>
       </c>
       <c r="D61" s="1" t="s">
+        <v>492</v>
+      </c>
+      <c r="E61" s="1" t="s">
         <v>493</v>
       </c>
-      <c r="E61" s="1" t="s">
+      <c r="F61" s="1" t="s">
         <v>494</v>
-      </c>
-      <c r="F61" s="1" t="s">
-        <v>495</v>
       </c>
     </row>
     <row r="62" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B62" s="3" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="C62" s="3" t="s">
         <v>73</v>
       </c>
       <c r="D62" s="1" t="s">
+        <v>496</v>
+      </c>
+      <c r="E62" s="1" t="s">
         <v>497</v>
-      </c>
-      <c r="E62" s="1" t="s">
-        <v>498</v>
       </c>
       <c r="F62" s="1" t="s">
         <v>59</v>
@@ -3573,152 +3594,152 @@
     </row>
     <row r="63" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B63" s="3" t="s">
-        <v>501</v>
+        <v>500</v>
       </c>
       <c r="C63" s="3" t="s">
         <v>63</v>
       </c>
       <c r="D63" s="1" t="s">
+        <v>498</v>
+      </c>
+      <c r="E63" s="1" t="s">
         <v>499</v>
       </c>
-      <c r="E63" s="1" t="s">
-        <v>500</v>
-      </c>
       <c r="F63" s="1" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
     </row>
     <row r="64" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B64" s="3" t="s">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="C64" s="3">
         <v>30</v>
       </c>
       <c r="D64" s="1" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="E64" s="1" t="s">
+        <v>509</v>
+      </c>
+      <c r="F64" s="1" t="s">
         <v>510</v>
-      </c>
-      <c r="F64" s="1" t="s">
-        <v>511</v>
       </c>
     </row>
     <row r="65" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B65" s="3" t="s">
+        <v>514</v>
+      </c>
+      <c r="C65" s="3" t="s">
+        <v>516</v>
+      </c>
+      <c r="D65" s="1" t="s">
         <v>515</v>
       </c>
-      <c r="C65" s="3" t="s">
+      <c r="E65" s="1" t="s">
         <v>517</v>
       </c>
-      <c r="D65" s="1" t="s">
-        <v>516</v>
-      </c>
-      <c r="E65" s="1" t="s">
-        <v>518</v>
-      </c>
       <c r="F65" s="1" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
     </row>
     <row r="66" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B66" s="3" t="s">
+        <v>518</v>
+      </c>
+      <c r="C66" s="3" t="s">
+        <v>516</v>
+      </c>
+      <c r="D66" s="1" t="s">
+        <v>521</v>
+      </c>
+      <c r="E66" s="1" t="s">
         <v>519</v>
       </c>
-      <c r="C66" s="3" t="s">
-        <v>517</v>
-      </c>
-      <c r="D66" s="1" t="s">
-        <v>522</v>
-      </c>
-      <c r="E66" s="1" t="s">
+      <c r="F66" s="1" t="s">
         <v>520</v>
-      </c>
-      <c r="F66" s="1" t="s">
-        <v>521</v>
       </c>
     </row>
     <row r="67" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B67" s="3" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="C67" s="3" t="s">
         <v>63</v>
       </c>
       <c r="D67" s="1" t="s">
-        <v>540</v>
+        <v>539</v>
       </c>
       <c r="E67" s="1" t="s">
+        <v>523</v>
+      </c>
+      <c r="F67" s="1" t="s">
         <v>524</v>
-      </c>
-      <c r="F67" s="1" t="s">
-        <v>525</v>
       </c>
     </row>
     <row r="68" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B68" s="3" t="s">
-        <v>529</v>
+        <v>528</v>
       </c>
       <c r="C68" s="3">
         <v>18</v>
       </c>
       <c r="D68" s="1" t="s">
-        <v>528</v>
+        <v>527</v>
       </c>
       <c r="E68" s="1" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="F68" s="1" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
     </row>
     <row r="69" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B69" s="3" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="C69" s="3" t="s">
         <v>85</v>
       </c>
       <c r="D69" s="1" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="E69" s="1" t="s">
+        <v>531</v>
+      </c>
+      <c r="F69" s="1" t="s">
         <v>532</v>
-      </c>
-      <c r="F69" s="1" t="s">
-        <v>533</v>
       </c>
     </row>
     <row r="70" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B70" s="3" t="s">
-        <v>536</v>
+        <v>535</v>
       </c>
       <c r="C70" s="3" t="s">
         <v>143</v>
       </c>
       <c r="D70" s="1" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
       <c r="E70" s="1" t="s">
+        <v>536</v>
+      </c>
+      <c r="F70" s="1" t="s">
         <v>537</v>
-      </c>
-      <c r="F70" s="1" t="s">
-        <v>538</v>
       </c>
     </row>
     <row r="71" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B71" s="3" t="s">
-        <v>541</v>
+        <v>540</v>
       </c>
       <c r="C71" s="3">
         <v>10</v>
       </c>
       <c r="D71" s="1" t="s">
+        <v>541</v>
+      </c>
+      <c r="E71" s="1" t="s">
         <v>542</v>
-      </c>
-      <c r="E71" s="1" t="s">
-        <v>543</v>
       </c>
       <c r="F71" s="1" t="s">
         <v>199</v>
@@ -3726,362 +3747,378 @@
     </row>
     <row r="72" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B72" s="3" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
       <c r="C72" s="3">
         <v>20</v>
       </c>
       <c r="D72" s="1" t="s">
+        <v>544</v>
+      </c>
+      <c r="E72" s="1" t="s">
+        <v>546</v>
+      </c>
+      <c r="F72" s="1" t="s">
         <v>545</v>
-      </c>
-      <c r="E72" s="1" t="s">
-        <v>547</v>
-      </c>
-      <c r="F72" s="1" t="s">
-        <v>546</v>
       </c>
     </row>
     <row r="73" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B73" s="3" t="s">
-        <v>548</v>
+        <v>547</v>
       </c>
       <c r="C73" s="3">
         <v>50</v>
       </c>
       <c r="D73" s="1" t="s">
+        <v>549</v>
+      </c>
+      <c r="E73" s="1" t="s">
         <v>550</v>
       </c>
-      <c r="E73" s="1" t="s">
-        <v>551</v>
-      </c>
       <c r="F73" s="1" t="s">
-        <v>549</v>
+        <v>548</v>
       </c>
     </row>
     <row r="74" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B74" s="3" t="s">
-        <v>553</v>
+        <v>552</v>
       </c>
       <c r="C74" s="3">
         <v>22</v>
       </c>
       <c r="D74" s="1" t="s">
-        <v>621</v>
+        <v>620</v>
       </c>
       <c r="E74" s="1" t="s">
-        <v>554</v>
+        <v>553</v>
       </c>
       <c r="F74" s="1" t="s">
-        <v>552</v>
+        <v>551</v>
       </c>
     </row>
     <row r="75" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B75" s="3" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="C75" s="1">
         <v>10</v>
       </c>
       <c r="D75" s="1" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
       <c r="E75" s="1" t="s">
-        <v>557</v>
+        <v>556</v>
       </c>
       <c r="F75" s="1" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
     </row>
     <row r="76" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B76" s="3" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
       <c r="C76" s="1">
         <v>10</v>
       </c>
       <c r="D76" s="1" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
       <c r="E76" s="1" t="s">
+        <v>563</v>
+      </c>
+      <c r="F76" s="1" t="s">
         <v>564</v>
-      </c>
-      <c r="F76" s="1" t="s">
-        <v>565</v>
       </c>
     </row>
     <row r="77" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B77" s="3" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
       <c r="C77" s="3">
         <v>10</v>
       </c>
       <c r="D77" s="1" t="s">
+        <v>567</v>
+      </c>
+      <c r="E77" s="1" t="s">
         <v>568</v>
       </c>
-      <c r="E77" s="1" t="s">
+      <c r="F77" s="1" t="s">
         <v>569</v>
-      </c>
-      <c r="F77" s="1" t="s">
-        <v>570</v>
       </c>
     </row>
     <row r="78" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B78" s="3" t="s">
-        <v>571</v>
+        <v>570</v>
       </c>
       <c r="C78" s="3">
         <v>15</v>
       </c>
       <c r="D78" s="1" t="s">
+        <v>571</v>
+      </c>
+      <c r="E78" s="1" t="s">
         <v>572</v>
       </c>
-      <c r="E78" s="1" t="s">
+      <c r="F78" s="1" t="s">
         <v>573</v>
-      </c>
-      <c r="F78" s="1" t="s">
-        <v>574</v>
       </c>
     </row>
     <row r="79" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B79" s="3" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="C79" s="3">
         <v>25</v>
       </c>
       <c r="D79" s="1" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="E79" s="1" t="s">
-        <v>576</v>
+        <v>575</v>
       </c>
       <c r="F79" s="1" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
     </row>
     <row r="80" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B80" s="3" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="C80" s="3">
         <v>10</v>
       </c>
       <c r="D80" s="1" t="s">
+        <v>581</v>
+      </c>
+      <c r="E80" s="1" t="s">
         <v>582</v>
       </c>
-      <c r="E80" s="1" t="s">
+      <c r="F80" s="1" t="s">
         <v>583</v>
-      </c>
-      <c r="F80" s="1" t="s">
-        <v>584</v>
       </c>
     </row>
     <row r="81" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B81" s="3" t="s">
-        <v>589</v>
+        <v>588</v>
       </c>
       <c r="C81" s="3">
         <v>25</v>
       </c>
       <c r="D81" s="1" t="s">
+        <v>589</v>
+      </c>
+      <c r="E81" s="1" t="s">
         <v>590</v>
       </c>
-      <c r="E81" s="1" t="s">
+      <c r="F81" s="1" t="s">
         <v>591</v>
-      </c>
-      <c r="F81" s="1" t="s">
-        <v>592</v>
       </c>
     </row>
     <row r="82" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B82" s="3" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="C82" s="3">
         <v>30</v>
       </c>
       <c r="D82" s="1" t="s">
+        <v>593</v>
+      </c>
+      <c r="E82" s="1" t="s">
         <v>594</v>
       </c>
-      <c r="E82" s="1" t="s">
+      <c r="F82" s="1" t="s">
         <v>595</v>
-      </c>
-      <c r="F82" s="1" t="s">
-        <v>596</v>
       </c>
     </row>
     <row r="83" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B83" s="3" t="s">
-        <v>597</v>
+        <v>596</v>
       </c>
       <c r="C83" s="3">
         <v>41</v>
       </c>
       <c r="D83" s="1" t="s">
+        <v>597</v>
+      </c>
+      <c r="E83" s="1" t="s">
+        <v>599</v>
+      </c>
+      <c r="F83" s="1" t="s">
         <v>598</v>
-      </c>
-      <c r="E83" s="1" t="s">
-        <v>600</v>
-      </c>
-      <c r="F83" s="1" t="s">
-        <v>599</v>
       </c>
     </row>
     <row r="84" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B84" s="3" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="C84" s="3">
         <v>100</v>
       </c>
       <c r="D84" s="1" t="s">
+        <v>601</v>
+      </c>
+      <c r="E84" s="1" t="s">
         <v>602</v>
       </c>
-      <c r="E84" s="1" t="s">
+      <c r="F84" s="1" t="s">
         <v>603</v>
-      </c>
-      <c r="F84" s="1" t="s">
-        <v>604</v>
       </c>
     </row>
     <row r="85" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B85" s="3" t="s">
-        <v>605</v>
+        <v>604</v>
       </c>
       <c r="C85" s="3">
         <v>28</v>
       </c>
       <c r="D85" s="1" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="E85" s="1" t="s">
+        <v>605</v>
+      </c>
+      <c r="F85" s="1" t="s">
         <v>606</v>
-      </c>
-      <c r="F85" s="1" t="s">
-        <v>607</v>
       </c>
     </row>
     <row r="86" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B86" s="3" t="s">
-        <v>609</v>
+        <v>608</v>
       </c>
       <c r="C86" s="3">
         <v>25</v>
       </c>
       <c r="D86" s="1" t="s">
+        <v>609</v>
+      </c>
+      <c r="E86" s="1" t="s">
         <v>610</v>
       </c>
-      <c r="E86" s="1" t="s">
-        <v>611</v>
-      </c>
       <c r="F86" s="1" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
     </row>
     <row r="87" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B87" s="3" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
       <c r="C87" s="3">
         <v>10</v>
       </c>
       <c r="D87" s="1" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
       <c r="E87" s="1" t="s">
-        <v>614</v>
+        <v>613</v>
       </c>
       <c r="F87" s="1" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
     </row>
     <row r="88" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B88" s="3" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="C88" s="3">
         <v>20</v>
       </c>
       <c r="D88" s="1" t="s">
+        <v>623</v>
+      </c>
+      <c r="E88" s="1" t="s">
         <v>624</v>
       </c>
-      <c r="E88" s="1" t="s">
+      <c r="F88" s="1" t="s">
         <v>625</v>
-      </c>
-      <c r="F88" s="1" t="s">
-        <v>626</v>
       </c>
     </row>
     <row r="89" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B89" s="3" t="s">
-        <v>627</v>
+        <v>626</v>
       </c>
       <c r="C89" s="3">
         <v>20</v>
       </c>
       <c r="D89" s="1" t="s">
-        <v>630</v>
+        <v>629</v>
       </c>
       <c r="E89" s="1" t="s">
+        <v>627</v>
+      </c>
+      <c r="F89" s="1" t="s">
         <v>628</v>
-      </c>
-      <c r="F89" s="1" t="s">
-        <v>629</v>
       </c>
     </row>
     <row r="90" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B90" s="3" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="C90" s="3">
         <v>20</v>
       </c>
       <c r="D90" s="1" t="s">
+        <v>631</v>
+      </c>
+      <c r="E90" s="1" t="s">
         <v>632</v>
       </c>
-      <c r="E90" s="1" t="s">
+      <c r="F90" s="1" t="s">
         <v>633</v>
-      </c>
-      <c r="F90" s="1" t="s">
-        <v>634</v>
       </c>
     </row>
     <row r="91" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B91" s="3" t="s">
-        <v>635</v>
+        <v>634</v>
       </c>
       <c r="C91" s="3">
         <v>10</v>
       </c>
-      <c r="D91" s="9" t="s">
+      <c r="D91" s="8" t="s">
+        <v>636</v>
+      </c>
+      <c r="E91" s="1" t="s">
+        <v>635</v>
+      </c>
+      <c r="F91" s="1" t="s">
         <v>637</v>
-      </c>
-      <c r="E91" s="1" t="s">
-        <v>636</v>
-      </c>
-      <c r="F91" s="1" t="s">
-        <v>638</v>
       </c>
     </row>
     <row r="92" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B92" s="3" t="s">
-        <v>639</v>
+        <v>638</v>
       </c>
       <c r="C92" s="3">
         <v>10</v>
       </c>
       <c r="D92" s="1" t="s">
-        <v>641</v>
+        <v>640</v>
       </c>
       <c r="E92" s="1" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
       <c r="F92" s="1" t="s">
-        <v>596</v>
-      </c>
-    </row>
-    <row r="93" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25"/>
+        <v>595</v>
+      </c>
+    </row>
+    <row r="93" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B93" s="3" t="s">
+        <v>650</v>
+      </c>
+      <c r="C93" s="3">
+        <v>43</v>
+      </c>
+      <c r="D93" s="1" t="s">
+        <v>651</v>
+      </c>
+      <c r="E93" s="1" t="s">
+        <v>652</v>
+      </c>
+      <c r="F93" s="1" t="s">
+        <v>653</v>
+      </c>
+    </row>
     <row r="94" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="95" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="96" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -4162,7 +4199,7 @@
     </row>
     <row r="5" spans="2:6" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="3" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="C5" s="3">
         <v>500</v>
@@ -4174,7 +4211,7 @@
         <v>171</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="6" spans="2:6" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -4253,13 +4290,13 @@
         <v>5000</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="11" spans="2:6" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -4270,13 +4307,13 @@
         <v>8000</v>
       </c>
       <c r="D11" s="1" t="s">
+        <v>268</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>270</v>
+      </c>
+      <c r="F11" s="1" t="s">
         <v>269</v>
-      </c>
-      <c r="E11" s="1" t="s">
-        <v>271</v>
-      </c>
-      <c r="F11" s="1" t="s">
-        <v>270</v>
       </c>
     </row>
     <row r="12" spans="2:6" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -4287,13 +4324,13 @@
         <v>150</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="E12" s="1" t="s">
+        <v>271</v>
+      </c>
+      <c r="F12" s="1" t="s">
         <v>272</v>
-      </c>
-      <c r="F12" s="1" t="s">
-        <v>273</v>
       </c>
     </row>
     <row r="13" spans="2:6" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -4304,64 +4341,64 @@
         <v>700</v>
       </c>
       <c r="D13" s="1" t="s">
+        <v>274</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>276</v>
+      </c>
+      <c r="F13" s="1" t="s">
         <v>275</v>
-      </c>
-      <c r="E13" s="1" t="s">
-        <v>277</v>
-      </c>
-      <c r="F13" s="1" t="s">
-        <v>276</v>
       </c>
     </row>
     <row r="14" spans="2:6" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B14" s="3" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="C14" s="3">
         <v>800</v>
       </c>
       <c r="D14" s="1" t="s">
+        <v>278</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>280</v>
+      </c>
+      <c r="F14" s="1" t="s">
         <v>279</v>
-      </c>
-      <c r="E14" s="1" t="s">
-        <v>281</v>
-      </c>
-      <c r="F14" s="1" t="s">
-        <v>280</v>
       </c>
     </row>
     <row r="15" spans="2:6" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B15" s="3" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="C15" s="7">
         <v>1400</v>
       </c>
       <c r="D15" s="1" t="s">
+        <v>283</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>281</v>
+      </c>
+      <c r="F15" s="1" t="s">
         <v>284</v>
-      </c>
-      <c r="E15" s="1" t="s">
-        <v>282</v>
-      </c>
-      <c r="F15" s="1" t="s">
-        <v>285</v>
       </c>
     </row>
     <row r="16" spans="2:6" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B16" s="3" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="C16" s="3">
         <v>500</v>
       </c>
       <c r="D16" s="1" t="s">
+        <v>264</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>267</v>
+      </c>
+      <c r="F16" s="1" t="s">
         <v>265</v>
-      </c>
-      <c r="E16" s="1" t="s">
-        <v>268</v>
-      </c>
-      <c r="F16" s="1" t="s">
-        <v>266</v>
       </c>
     </row>
     <row r="17" spans="2:6" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -4372,10 +4409,10 @@
         <v>100</v>
       </c>
       <c r="D17" s="1" t="s">
+        <v>262</v>
+      </c>
+      <c r="E17" s="1" t="s">
         <v>263</v>
-      </c>
-      <c r="E17" s="1" t="s">
-        <v>264</v>
       </c>
       <c r="F17" s="1" t="s">
         <v>146</v>
@@ -4389,13 +4426,13 @@
         <v>30</v>
       </c>
       <c r="D18" s="1" t="s">
+        <v>259</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>258</v>
+      </c>
+      <c r="F18" s="1" t="s">
         <v>260</v>
-      </c>
-      <c r="E18" s="1" t="s">
-        <v>259</v>
-      </c>
-      <c r="F18" s="1" t="s">
-        <v>261</v>
       </c>
     </row>
     <row r="19" spans="2:6" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -4406,13 +4443,13 @@
         <v>15000</v>
       </c>
       <c r="D19" s="1" t="s">
+        <v>256</v>
+      </c>
+      <c r="E19" s="1" t="s">
         <v>257</v>
       </c>
-      <c r="E19" s="1" t="s">
-        <v>258</v>
-      </c>
       <c r="F19" s="1" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
     </row>
     <row r="20" spans="2:6" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -4423,13 +4460,13 @@
         <v>14000</v>
       </c>
       <c r="D20" s="1" t="s">
+        <v>250</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>252</v>
+      </c>
+      <c r="F20" s="1" t="s">
         <v>251</v>
-      </c>
-      <c r="E20" s="1" t="s">
-        <v>253</v>
-      </c>
-      <c r="F20" s="1" t="s">
-        <v>252</v>
       </c>
     </row>
     <row r="21" spans="2:6" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -4443,7 +4480,7 @@
         <v>233</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>234</v>
+        <v>645</v>
       </c>
       <c r="F21" s="1" t="s">
         <v>232</v>
@@ -4451,50 +4488,50 @@
     </row>
     <row r="22" spans="2:6" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B22" s="3" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="C22" s="3">
         <v>500</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
     </row>
     <row r="23" spans="2:6" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B23" s="3" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="C23" s="3">
         <v>100</v>
       </c>
       <c r="D23" s="1" t="s">
+        <v>315</v>
+      </c>
+      <c r="E23" s="1" t="s">
         <v>316</v>
       </c>
-      <c r="E23" s="1" t="s">
+      <c r="F23" s="1" t="s">
         <v>317</v>
-      </c>
-      <c r="F23" s="1" t="s">
-        <v>318</v>
       </c>
     </row>
     <row r="24" spans="2:6" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B24" s="3" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="C24" s="3">
         <v>500</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="F24" s="1" t="s">
         <v>176</v>
@@ -4502,153 +4539,169 @@
     </row>
     <row r="25" spans="2:6" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B25" s="3" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="C25" s="3">
         <v>200</v>
       </c>
       <c r="D25" s="1" t="s">
+        <v>322</v>
+      </c>
+      <c r="E25" s="1" t="s">
         <v>323</v>
       </c>
-      <c r="E25" s="1" t="s">
+      <c r="F25" s="1" t="s">
         <v>324</v>
-      </c>
-      <c r="F25" s="1" t="s">
-        <v>325</v>
       </c>
     </row>
     <row r="26" spans="2:6" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B26" s="3" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="C26" s="3">
         <v>400</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
     </row>
     <row r="27" spans="2:6" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B27" s="3" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="C27" s="3">
         <v>500</v>
       </c>
       <c r="D27" s="1" t="s">
+        <v>383</v>
+      </c>
+      <c r="E27" s="1" t="s">
         <v>384</v>
       </c>
-      <c r="E27" s="1" t="s">
-        <v>385</v>
-      </c>
       <c r="F27" s="1" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
     </row>
     <row r="28" spans="2:6" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B28" s="3" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="C28" s="3">
         <v>2000</v>
       </c>
       <c r="D28" s="1" t="s">
+        <v>441</v>
+      </c>
+      <c r="E28" s="1" t="s">
         <v>442</v>
       </c>
-      <c r="E28" s="1" t="s">
+      <c r="F28" s="1" t="s">
         <v>443</v>
-      </c>
-      <c r="F28" s="1" t="s">
-        <v>444</v>
       </c>
     </row>
     <row r="29" spans="2:6" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B29" s="3" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="C29" s="3">
         <v>2300</v>
       </c>
       <c r="D29" s="1" t="s">
+        <v>457</v>
+      </c>
+      <c r="E29" s="1" t="s">
         <v>458</v>
       </c>
-      <c r="E29" s="1" t="s">
+      <c r="F29" s="1" t="s">
         <v>459</v>
-      </c>
-      <c r="F29" s="1" t="s">
-        <v>460</v>
       </c>
     </row>
     <row r="30" spans="2:6" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B30" s="3" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="C30" s="3">
         <v>5000</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>622</v>
+        <v>621</v>
       </c>
       <c r="E30" s="1" t="s">
+        <v>476</v>
+      </c>
+      <c r="F30" s="1" t="s">
         <v>477</v>
-      </c>
-      <c r="F30" s="1" t="s">
-        <v>478</v>
       </c>
     </row>
     <row r="31" spans="2:6" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B31" s="3" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="C31" s="7">
         <v>1294</v>
       </c>
       <c r="D31" s="1" t="s">
+        <v>502</v>
+      </c>
+      <c r="E31" s="1" t="s">
         <v>503</v>
       </c>
-      <c r="E31" s="1" t="s">
+      <c r="F31" s="1" t="s">
         <v>504</v>
-      </c>
-      <c r="F31" s="1" t="s">
-        <v>505</v>
       </c>
     </row>
     <row r="32" spans="2:6" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B32" s="3" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="C32" s="7">
         <v>1933</v>
       </c>
       <c r="D32" s="1" t="s">
+        <v>506</v>
+      </c>
+      <c r="E32" s="1" t="s">
         <v>507</v>
       </c>
-      <c r="E32" s="1" t="s">
+      <c r="F32" s="4" t="s">
         <v>508</v>
       </c>
-      <c r="F32" s="4" t="s">
-        <v>509</v>
-      </c>
-    </row>
-    <row r="33" ht="59.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="34" ht="59.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="35" ht="59.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="36" ht="59.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="37" ht="59.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="38" ht="59.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="39" ht="59.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="40" ht="59.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="41" ht="59.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="42" ht="59.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="43" ht="59.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="44" ht="59.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="45" ht="59.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    </row>
+    <row r="33" spans="2:6" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B33" s="3" t="s">
+        <v>646</v>
+      </c>
+      <c r="C33" s="3">
+        <v>756</v>
+      </c>
+      <c r="D33" s="1" t="s">
+        <v>647</v>
+      </c>
+      <c r="E33" s="1" t="s">
+        <v>648</v>
+      </c>
+      <c r="F33" s="1" t="s">
+        <v>649</v>
+      </c>
+    </row>
+    <row r="34" spans="2:6" ht="59.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="35" spans="2:6" ht="59.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="36" spans="2:6" ht="59.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="37" spans="2:6" ht="59.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="38" spans="2:6" ht="59.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="39" spans="2:6" ht="59.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="40" spans="2:6" ht="59.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="41" spans="2:6" ht="59.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="42" spans="2:6" ht="59.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="43" spans="2:6" ht="59.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="44" spans="2:6" ht="59.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="45" spans="2:6" ht="59.25" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -4659,609 +4712,609 @@
   <dimension ref="B1:G45"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="10.83203125" style="8"/>
-    <col min="2" max="4" width="28" style="8" customWidth="1"/>
-    <col min="5" max="5" width="30" style="8" customWidth="1"/>
-    <col min="6" max="7" width="28" style="8" customWidth="1"/>
-    <col min="8" max="16384" width="10.83203125" style="8"/>
+    <col min="1" max="1" width="10.83203125" style="6"/>
+    <col min="2" max="4" width="28" style="6" customWidth="1"/>
+    <col min="5" max="5" width="30" style="6" customWidth="1"/>
+    <col min="6" max="7" width="28" style="6" customWidth="1"/>
+    <col min="8" max="16384" width="10.83203125" style="6"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:6" ht="22" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="2" spans="2:6" s="12" customFormat="1" ht="58" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B2" s="12" t="s">
+    <row r="2" spans="2:6" s="11" customFormat="1" ht="58" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B2" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="12" t="s">
+      <c r="C2" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="12" t="s">
+      <c r="D2" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="E2" s="12" t="s">
+      <c r="E2" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="F2" s="12" t="s">
+      <c r="F2" s="11" t="s">
         <v>148</v>
       </c>
     </row>
     <row r="3" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B3" s="8" t="s">
+      <c r="B3" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="C3" s="13">
+      <c r="C3" s="12">
         <v>13000</v>
       </c>
-      <c r="D3" s="8" t="s">
+      <c r="D3" s="6" t="s">
         <v>178</v>
       </c>
-      <c r="E3" s="8" t="s">
+      <c r="E3" s="6" t="s">
         <v>179</v>
       </c>
-      <c r="F3" s="8" t="s">
+      <c r="F3" s="6" t="s">
         <v>223</v>
       </c>
     </row>
     <row r="4" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B4" s="8" t="s">
+      <c r="B4" s="6" t="s">
         <v>181</v>
       </c>
-      <c r="C4" s="8">
+      <c r="C4" s="6">
         <v>500</v>
       </c>
-      <c r="D4" s="8" t="s">
+      <c r="D4" s="6" t="s">
         <v>182</v>
       </c>
-      <c r="E4" s="8" t="s">
+      <c r="E4" s="6" t="s">
         <v>186</v>
       </c>
-      <c r="F4" s="8" t="s">
+      <c r="F4" s="6" t="s">
         <v>180</v>
       </c>
     </row>
     <row r="5" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B5" s="8" t="s">
+      <c r="B5" s="6" t="s">
         <v>184</v>
       </c>
-      <c r="C5" s="8">
+      <c r="C5" s="6">
         <v>130</v>
       </c>
-      <c r="D5" s="8" t="s">
+      <c r="D5" s="6" t="s">
         <v>185</v>
       </c>
-      <c r="E5" s="8" t="s">
+      <c r="E5" s="6" t="s">
         <v>187</v>
       </c>
-      <c r="F5" s="8" t="s">
+      <c r="F5" s="6" t="s">
         <v>183</v>
       </c>
     </row>
     <row r="6" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B6" s="8" t="s">
+      <c r="B6" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="C6" s="8" t="s">
+      <c r="C6" s="6" t="s">
         <v>191</v>
       </c>
-      <c r="D6" s="8" t="s">
+      <c r="D6" s="6" t="s">
         <v>189</v>
       </c>
-      <c r="E6" s="8" t="s">
+      <c r="E6" s="6" t="s">
         <v>188</v>
       </c>
-      <c r="F6" s="8" t="s">
+      <c r="F6" s="6" t="s">
         <v>190</v>
       </c>
     </row>
     <row r="7" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B7" s="8" t="s">
+      <c r="B7" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="C7" s="8" t="s">
+      <c r="C7" s="6" t="s">
         <v>195</v>
       </c>
-      <c r="D7" s="8" t="s">
+      <c r="D7" s="6" t="s">
         <v>193</v>
       </c>
-      <c r="E7" s="8" t="s">
+      <c r="E7" s="6" t="s">
         <v>194</v>
       </c>
-      <c r="F7" s="8" t="s">
+      <c r="F7" s="6" t="s">
         <v>192</v>
       </c>
     </row>
     <row r="8" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B8" s="8" t="s">
+      <c r="B8" s="6" t="s">
         <v>198</v>
       </c>
-      <c r="C8" s="8">
+      <c r="C8" s="6">
         <v>70</v>
       </c>
-      <c r="D8" s="8" t="s">
+      <c r="D8" s="6" t="s">
         <v>196</v>
       </c>
-      <c r="E8" s="8" t="s">
+      <c r="E8" s="6" t="s">
         <v>197</v>
       </c>
-      <c r="F8" s="8" t="s">
+      <c r="F8" s="6" t="s">
         <v>199</v>
       </c>
     </row>
     <row r="9" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B9" s="8" t="s">
+      <c r="B9" s="6" t="s">
         <v>200</v>
       </c>
-      <c r="C9" s="13">
+      <c r="C9" s="12">
         <v>10000</v>
       </c>
-      <c r="D9" s="8" t="s">
+      <c r="D9" s="6" t="s">
         <v>201</v>
       </c>
-      <c r="E9" s="8" t="s">
+      <c r="E9" s="6" t="s">
         <v>202</v>
       </c>
-      <c r="F9" s="8" t="s">
+      <c r="F9" s="6" t="s">
         <v>222</v>
       </c>
     </row>
     <row r="10" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B10" s="8" t="s">
+      <c r="B10" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="C10" s="8">
+      <c r="C10" s="6">
         <v>100</v>
       </c>
-      <c r="D10" s="8" t="s">
+      <c r="D10" s="6" t="s">
         <v>205</v>
       </c>
-      <c r="E10" s="8" t="s">
+      <c r="E10" s="6" t="s">
         <v>95</v>
       </c>
-      <c r="F10" s="8" t="s">
+      <c r="F10" s="6" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="11" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B11" s="8" t="s">
+      <c r="B11" s="6" t="s">
         <v>76</v>
       </c>
-      <c r="C11" s="8" t="s">
+      <c r="C11" s="6" t="s">
         <v>210</v>
       </c>
-      <c r="D11" s="8" t="s">
+      <c r="D11" s="6" t="s">
         <v>207</v>
       </c>
-      <c r="E11" s="8" t="s">
+      <c r="E11" s="6" t="s">
         <v>208</v>
       </c>
-      <c r="F11" s="8" t="s">
+      <c r="F11" s="6" t="s">
         <v>209</v>
       </c>
     </row>
     <row r="12" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B12" s="8" t="s">
+      <c r="B12" s="6" t="s">
         <v>122</v>
       </c>
-      <c r="C12" s="13">
+      <c r="C12" s="12">
         <v>5500</v>
       </c>
-      <c r="D12" s="8" t="s">
+      <c r="D12" s="6" t="s">
         <v>211</v>
       </c>
-      <c r="E12" s="8" t="s">
+      <c r="E12" s="6" t="s">
         <v>212</v>
       </c>
-      <c r="F12" s="8" t="s">
-        <v>288</v>
+      <c r="F12" s="6" t="s">
+        <v>287</v>
       </c>
     </row>
     <row r="13" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B13" s="8" t="s">
+      <c r="B13" s="6" t="s">
         <v>203</v>
       </c>
-      <c r="C13" s="8" t="s">
+      <c r="C13" s="6" t="s">
         <v>215</v>
       </c>
-      <c r="D13" s="8" t="s">
+      <c r="D13" s="6" t="s">
         <v>213</v>
       </c>
-      <c r="E13" s="8" t="s">
+      <c r="E13" s="6" t="s">
         <v>204</v>
       </c>
-      <c r="F13" s="8" t="s">
+      <c r="F13" s="6" t="s">
         <v>216</v>
       </c>
     </row>
     <row r="14" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B14" s="8" t="s">
+      <c r="B14" s="6" t="s">
         <v>206</v>
       </c>
-      <c r="C14" s="13">
+      <c r="C14" s="12">
         <v>4500</v>
       </c>
-      <c r="D14" s="8" t="s">
+      <c r="D14" s="6" t="s">
         <v>217</v>
       </c>
-      <c r="E14" s="8" t="s">
+      <c r="E14" s="6" t="s">
         <v>218</v>
       </c>
-      <c r="F14" s="8" t="s">
-        <v>287</v>
+      <c r="F14" s="6" t="s">
+        <v>286</v>
       </c>
     </row>
     <row r="15" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B15" s="8" t="s">
+      <c r="B15" s="6" t="s">
         <v>214</v>
       </c>
-      <c r="C15" s="8">
+      <c r="C15" s="6">
         <v>20</v>
       </c>
-      <c r="D15" s="8" t="s">
+      <c r="D15" s="6" t="s">
         <v>219</v>
       </c>
-      <c r="E15" s="8" t="s">
+      <c r="E15" s="6" t="s">
         <v>220</v>
       </c>
-      <c r="F15" s="8" t="s">
+      <c r="F15" s="6" t="s">
         <v>221</v>
       </c>
     </row>
     <row r="16" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B16" s="8" t="s">
+      <c r="B16" s="6" t="s">
+        <v>237</v>
+      </c>
+      <c r="C16" s="6">
+        <v>20</v>
+      </c>
+      <c r="D16" s="6" t="s">
+        <v>235</v>
+      </c>
+      <c r="E16" s="6" t="s">
         <v>238</v>
       </c>
-      <c r="C16" s="8">
+      <c r="F16" s="6" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="17" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B17" s="6" t="s">
+        <v>245</v>
+      </c>
+      <c r="C17" s="6">
+        <v>150</v>
+      </c>
+      <c r="D17" s="6" t="s">
+        <v>246</v>
+      </c>
+      <c r="E17" s="6" t="s">
+        <v>247</v>
+      </c>
+      <c r="F17" s="6" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="18" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B18" s="6" t="s">
+        <v>306</v>
+      </c>
+      <c r="C18" s="6">
+        <v>1000</v>
+      </c>
+      <c r="D18" s="6" t="s">
+        <v>308</v>
+      </c>
+      <c r="E18" s="6" t="s">
+        <v>307</v>
+      </c>
+      <c r="F18" s="9" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="19" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B19" s="6" t="s">
+        <v>326</v>
+      </c>
+      <c r="C19" s="6">
         <v>20</v>
       </c>
-      <c r="D16" s="8" t="s">
-        <v>236</v>
-      </c>
-      <c r="E16" s="8" t="s">
-        <v>239</v>
-      </c>
-      <c r="F16" s="8" t="s">
-        <v>237</v>
-      </c>
-    </row>
-    <row r="17" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B17" s="8" t="s">
-        <v>246</v>
-      </c>
-      <c r="C17" s="8">
-        <v>150</v>
-      </c>
-      <c r="D17" s="8" t="s">
-        <v>247</v>
-      </c>
-      <c r="E17" s="8" t="s">
-        <v>248</v>
-      </c>
-      <c r="F17" s="8" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="18" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B18" s="8" t="s">
-        <v>307</v>
-      </c>
-      <c r="C18" s="8">
+      <c r="D19" s="6" t="s">
+        <v>327</v>
+      </c>
+      <c r="E19" s="9" t="s">
+        <v>328</v>
+      </c>
+      <c r="F19" s="10" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="20" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B20" s="6" t="s">
+        <v>331</v>
+      </c>
+      <c r="C20" s="6">
+        <v>50</v>
+      </c>
+      <c r="D20" s="6" t="s">
+        <v>329</v>
+      </c>
+      <c r="E20" s="6" t="s">
+        <v>330</v>
+      </c>
+      <c r="F20" s="6" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="21" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B21" s="6" t="s">
+        <v>391</v>
+      </c>
+      <c r="C21" s="6">
+        <v>50</v>
+      </c>
+      <c r="D21" s="6" t="s">
+        <v>390</v>
+      </c>
+      <c r="E21" s="6" t="s">
+        <v>393</v>
+      </c>
+      <c r="F21" s="6" t="s">
+        <v>392</v>
+      </c>
+    </row>
+    <row r="22" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B22" s="6" t="s">
+        <v>394</v>
+      </c>
+      <c r="C22" s="6" t="s">
+        <v>386</v>
+      </c>
+      <c r="D22" s="6" t="s">
+        <v>395</v>
+      </c>
+      <c r="E22" s="6" t="s">
+        <v>396</v>
+      </c>
+      <c r="F22" s="6" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="23" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B23" s="6" t="s">
+        <v>398</v>
+      </c>
+      <c r="C23" s="6">
+        <v>100</v>
+      </c>
+      <c r="D23" s="6" t="s">
+        <v>399</v>
+      </c>
+      <c r="E23" s="6" t="s">
+        <v>397</v>
+      </c>
+      <c r="F23" s="6" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="24" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B24" s="6" t="s">
+        <v>362</v>
+      </c>
+      <c r="C24" s="6">
+        <v>10</v>
+      </c>
+      <c r="D24" s="6" t="s">
+        <v>363</v>
+      </c>
+      <c r="E24" s="6" t="s">
+        <v>364</v>
+      </c>
+      <c r="F24" s="6" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="25" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B25" s="6" t="s">
+        <v>401</v>
+      </c>
+      <c r="C25" s="6">
+        <v>20</v>
+      </c>
+      <c r="D25" s="6" t="s">
+        <v>402</v>
+      </c>
+      <c r="E25" s="6" t="s">
+        <v>404</v>
+      </c>
+      <c r="F25" s="6" t="s">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="26" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B26" s="6" t="s">
+        <v>405</v>
+      </c>
+      <c r="C26" s="6">
         <v>1000</v>
       </c>
-      <c r="D18" s="8" t="s">
-        <v>309</v>
-      </c>
-      <c r="E18" s="8" t="s">
-        <v>308</v>
-      </c>
-      <c r="F18" s="10" t="s">
-        <v>310</v>
-      </c>
-    </row>
-    <row r="19" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B19" s="8" t="s">
-        <v>327</v>
-      </c>
-      <c r="C19" s="8">
+      <c r="D26" s="6" t="s">
+        <v>406</v>
+      </c>
+      <c r="E26" s="6" t="s">
+        <v>408</v>
+      </c>
+      <c r="F26" s="6" t="s">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="27" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B27" s="6" t="s">
+        <v>410</v>
+      </c>
+      <c r="C27" s="6">
+        <v>200</v>
+      </c>
+      <c r="D27" s="6" t="s">
+        <v>409</v>
+      </c>
+      <c r="E27" s="6" t="s">
+        <v>411</v>
+      </c>
+      <c r="F27" s="6" t="s">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="28" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B28" s="6" t="s">
+        <v>412</v>
+      </c>
+      <c r="C28" s="6">
+        <v>10</v>
+      </c>
+      <c r="D28" s="6" t="s">
+        <v>414</v>
+      </c>
+      <c r="E28" s="6" t="s">
+        <v>415</v>
+      </c>
+      <c r="F28" s="6" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="29" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B29" s="6" t="s">
+        <v>416</v>
+      </c>
+      <c r="C29" s="6">
+        <v>35</v>
+      </c>
+      <c r="D29" s="6" t="s">
+        <v>419</v>
+      </c>
+      <c r="E29" s="6" t="s">
+        <v>421</v>
+      </c>
+      <c r="F29" s="6" t="s">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="30" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B30" s="6" t="s">
+        <v>425</v>
+      </c>
+      <c r="C30" s="6">
+        <v>80</v>
+      </c>
+      <c r="D30" s="6" t="s">
+        <v>422</v>
+      </c>
+      <c r="E30" s="6" t="s">
+        <v>423</v>
+      </c>
+      <c r="F30" s="6" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="31" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B31" s="6" t="s">
+        <v>417</v>
+      </c>
+      <c r="C31" s="6">
         <v>20</v>
       </c>
-      <c r="D19" s="8" t="s">
-        <v>328</v>
-      </c>
-      <c r="E19" s="10" t="s">
-        <v>329</v>
-      </c>
-      <c r="F19" s="11" t="s">
-        <v>199</v>
-      </c>
-    </row>
-    <row r="20" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B20" s="8" t="s">
-        <v>332</v>
-      </c>
-      <c r="C20" s="8">
+      <c r="D31" s="6" t="s">
+        <v>426</v>
+      </c>
+      <c r="E31" s="6" t="s">
+        <v>427</v>
+      </c>
+      <c r="F31" s="6" t="s">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="32" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B32" s="6" t="s">
+        <v>418</v>
+      </c>
+      <c r="C32" s="6">
+        <v>40</v>
+      </c>
+      <c r="D32" s="6" t="s">
+        <v>430</v>
+      </c>
+      <c r="E32" s="6" t="s">
+        <v>431</v>
+      </c>
+      <c r="F32" s="6" t="s">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="33" spans="2:7" ht="58" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B33" s="6" t="s">
+        <v>433</v>
+      </c>
+      <c r="C33" s="6">
+        <v>104</v>
+      </c>
+      <c r="D33" s="6" t="s">
+        <v>436</v>
+      </c>
+      <c r="E33" s="6" t="s">
+        <v>435</v>
+      </c>
+      <c r="F33" s="6" t="s">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="34" spans="2:7" ht="58" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B34" s="6" t="s">
+        <v>559</v>
+      </c>
+      <c r="C34" s="6">
+        <v>200</v>
+      </c>
+      <c r="D34" s="6" t="s">
+        <v>560</v>
+      </c>
+      <c r="E34" s="6" t="s">
+        <v>561</v>
+      </c>
+      <c r="F34" s="6" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="35" spans="2:7" ht="58" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B35" s="6" t="s">
+        <v>616</v>
+      </c>
+      <c r="C35" s="6">
         <v>50</v>
       </c>
-      <c r="D20" s="8" t="s">
-        <v>330</v>
-      </c>
-      <c r="E20" s="8" t="s">
-        <v>331</v>
-      </c>
-      <c r="F20" s="8" t="s">
-        <v>333</v>
-      </c>
-    </row>
-    <row r="21" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B21" s="8" t="s">
-        <v>392</v>
-      </c>
-      <c r="C21" s="8">
-        <v>50</v>
-      </c>
-      <c r="D21" s="8" t="s">
-        <v>391</v>
-      </c>
-      <c r="E21" s="8" t="s">
-        <v>394</v>
-      </c>
-      <c r="F21" s="8" t="s">
-        <v>393</v>
-      </c>
-    </row>
-    <row r="22" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B22" s="8" t="s">
-        <v>395</v>
-      </c>
-      <c r="C22" s="8" t="s">
-        <v>387</v>
-      </c>
-      <c r="D22" s="8" t="s">
-        <v>396</v>
-      </c>
-      <c r="E22" s="8" t="s">
-        <v>397</v>
-      </c>
-      <c r="F22" s="8" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="23" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B23" s="8" t="s">
-        <v>399</v>
-      </c>
-      <c r="C23" s="8">
-        <v>100</v>
-      </c>
-      <c r="D23" s="8" t="s">
-        <v>400</v>
-      </c>
-      <c r="E23" s="8" t="s">
-        <v>398</v>
-      </c>
-      <c r="F23" s="8" t="s">
-        <v>401</v>
-      </c>
-    </row>
-    <row r="24" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B24" s="8" t="s">
-        <v>363</v>
-      </c>
-      <c r="C24" s="8">
+      <c r="D35" s="6" t="s">
+        <v>619</v>
+      </c>
+      <c r="E35" s="6" t="s">
+        <v>617</v>
+      </c>
+      <c r="F35" s="6" t="s">
+        <v>618</v>
+      </c>
+    </row>
+    <row r="36" spans="2:7" ht="58" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B36" s="14" t="s">
+        <v>641</v>
+      </c>
+      <c r="C36" s="6">
         <v>10</v>
       </c>
-      <c r="D24" s="8" t="s">
-        <v>364</v>
-      </c>
-      <c r="E24" s="8" t="s">
-        <v>365</v>
-      </c>
-      <c r="F24" s="8" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="25" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B25" s="8" t="s">
-        <v>402</v>
-      </c>
-      <c r="C25" s="8">
-        <v>20</v>
-      </c>
-      <c r="D25" s="8" t="s">
-        <v>403</v>
-      </c>
-      <c r="E25" s="8" t="s">
-        <v>405</v>
-      </c>
-      <c r="F25" s="8" t="s">
-        <v>404</v>
-      </c>
-    </row>
-    <row r="26" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B26" s="8" t="s">
-        <v>406</v>
-      </c>
-      <c r="C26" s="8">
-        <v>1000</v>
-      </c>
-      <c r="D26" s="8" t="s">
-        <v>407</v>
-      </c>
-      <c r="E26" s="8" t="s">
-        <v>409</v>
-      </c>
-      <c r="F26" s="8" t="s">
-        <v>408</v>
-      </c>
-    </row>
-    <row r="27" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B27" s="8" t="s">
-        <v>411</v>
-      </c>
-      <c r="C27" s="8">
-        <v>200</v>
-      </c>
-      <c r="D27" s="8" t="s">
-        <v>410</v>
-      </c>
-      <c r="E27" s="8" t="s">
-        <v>412</v>
-      </c>
-      <c r="F27" s="8" t="s">
-        <v>414</v>
-      </c>
-    </row>
-    <row r="28" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B28" s="8" t="s">
-        <v>413</v>
-      </c>
-      <c r="C28" s="8">
-        <v>10</v>
-      </c>
-      <c r="D28" s="8" t="s">
-        <v>415</v>
-      </c>
-      <c r="E28" s="8" t="s">
-        <v>416</v>
-      </c>
-      <c r="F28" s="8" t="s">
-        <v>199</v>
-      </c>
-    </row>
-    <row r="29" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B29" s="8" t="s">
-        <v>417</v>
-      </c>
-      <c r="C29" s="8">
-        <v>35</v>
-      </c>
-      <c r="D29" s="8" t="s">
-        <v>420</v>
-      </c>
-      <c r="E29" s="8" t="s">
-        <v>422</v>
-      </c>
-      <c r="F29" s="8" t="s">
-        <v>421</v>
-      </c>
-    </row>
-    <row r="30" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B30" s="8" t="s">
-        <v>426</v>
-      </c>
-      <c r="C30" s="8">
-        <v>80</v>
-      </c>
-      <c r="D30" s="8" t="s">
-        <v>423</v>
-      </c>
-      <c r="E30" s="8" t="s">
-        <v>424</v>
-      </c>
-      <c r="F30" s="8" t="s">
-        <v>425</v>
-      </c>
-    </row>
-    <row r="31" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B31" s="8" t="s">
-        <v>418</v>
-      </c>
-      <c r="C31" s="8">
-        <v>20</v>
-      </c>
-      <c r="D31" s="8" t="s">
-        <v>427</v>
-      </c>
-      <c r="E31" s="8" t="s">
-        <v>428</v>
-      </c>
-      <c r="F31" s="8" t="s">
-        <v>429</v>
-      </c>
-    </row>
-    <row r="32" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B32" s="8" t="s">
-        <v>419</v>
-      </c>
-      <c r="C32" s="8">
-        <v>40</v>
-      </c>
-      <c r="D32" s="8" t="s">
-        <v>431</v>
-      </c>
-      <c r="E32" s="8" t="s">
-        <v>432</v>
-      </c>
-      <c r="F32" s="8" t="s">
-        <v>430</v>
-      </c>
-    </row>
-    <row r="33" spans="2:7" ht="58" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B33" s="8" t="s">
-        <v>434</v>
-      </c>
-      <c r="C33" s="8">
-        <v>104</v>
-      </c>
-      <c r="D33" s="8" t="s">
-        <v>437</v>
-      </c>
-      <c r="E33" s="8" t="s">
-        <v>436</v>
-      </c>
-      <c r="F33" s="8" t="s">
-        <v>433</v>
-      </c>
-    </row>
-    <row r="34" spans="2:7" ht="58" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B34" s="8" t="s">
-        <v>560</v>
-      </c>
-      <c r="C34" s="8">
-        <v>200</v>
-      </c>
-      <c r="D34" s="8" t="s">
-        <v>561</v>
-      </c>
-      <c r="E34" s="8" t="s">
-        <v>562</v>
-      </c>
-      <c r="F34" s="8" t="s">
-        <v>559</v>
-      </c>
-    </row>
-    <row r="35" spans="2:7" ht="58" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B35" s="8" t="s">
-        <v>617</v>
-      </c>
-      <c r="C35" s="8">
-        <v>50</v>
-      </c>
-      <c r="D35" s="6" t="s">
-        <v>620</v>
-      </c>
-      <c r="E35" s="8" t="s">
-        <v>618</v>
-      </c>
-      <c r="F35" s="8" t="s">
-        <v>619</v>
-      </c>
-    </row>
-    <row r="36" spans="2:7" ht="58" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B36" s="15" t="s">
+      <c r="D36" s="15" t="s">
         <v>642</v>
       </c>
-      <c r="C36" s="8">
-        <v>10</v>
-      </c>
-      <c r="D36" s="16" t="s">
+      <c r="E36" s="6" t="s">
         <v>643</v>
       </c>
-      <c r="E36" s="8" t="s">
+      <c r="F36" s="6" t="s">
         <v>644</v>
       </c>
-      <c r="F36" s="6" t="s">
-        <v>645</v>
-      </c>
-      <c r="G36" s="14"/>
+      <c r="G36" s="13"/>
     </row>
     <row r="37" spans="2:7" ht="58" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="38" spans="2:7" ht="58" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -5359,67 +5412,67 @@
     </row>
     <row r="6" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="3" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="C6" s="3">
         <v>40</v>
       </c>
       <c r="D6" s="1" t="s">
+        <v>299</v>
+      </c>
+      <c r="E6" s="1" t="s">
         <v>300</v>
       </c>
-      <c r="E6" s="1" t="s">
+      <c r="F6" s="1" t="s">
         <v>301</v>
-      </c>
-      <c r="F6" s="1" t="s">
-        <v>302</v>
       </c>
     </row>
     <row r="7" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B7" s="3" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="C7" s="3">
         <v>50</v>
       </c>
       <c r="D7" s="1" t="s">
+        <v>339</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>341</v>
+      </c>
+      <c r="F7" s="1" t="s">
         <v>340</v>
-      </c>
-      <c r="E7" s="1" t="s">
-        <v>342</v>
-      </c>
-      <c r="F7" s="1" t="s">
-        <v>341</v>
       </c>
     </row>
     <row r="8" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B8" s="3" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="C8" s="3">
         <v>300</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="E8" s="1" t="s">
+        <v>374</v>
+      </c>
+      <c r="F8" s="1" t="s">
         <v>375</v>
-      </c>
-      <c r="F8" s="1" t="s">
-        <v>376</v>
       </c>
     </row>
     <row r="9" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B9" s="3" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="C9" s="3">
         <v>5</v>
       </c>
       <c r="D9" s="1" t="s">
+        <v>578</v>
+      </c>
+      <c r="E9" s="1" t="s">
         <v>579</v>
-      </c>
-      <c r="E9" s="1" t="s">
-        <v>580</v>
       </c>
       <c r="F9" s="1" t="s">
         <v>199</v>
@@ -5427,19 +5480,19 @@
     </row>
     <row r="10" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="3" t="s">
-        <v>585</v>
+        <v>584</v>
       </c>
       <c r="C10" s="3">
         <v>15</v>
       </c>
       <c r="D10" s="1" t="s">
+        <v>585</v>
+      </c>
+      <c r="E10" s="1" t="s">
         <v>586</v>
       </c>
-      <c r="E10" s="1" t="s">
+      <c r="F10" s="1" t="s">
         <v>587</v>
-      </c>
-      <c r="F10" s="1" t="s">
-        <v>588</v>
       </c>
     </row>
     <row r="11" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25"/>

</xml_diff>

<commit_message>
added a seperate notebook to allow for location-based list filter
</commit_message>
<xml_diff>
--- a/Photonic Companies.xlsx
+++ b/Photonic Companies.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/blow/Desktop/GitHub/PhotonicCompanies/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{629F32E4-6996-9847-A81C-F00E30FB6745}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC9E5797-1404-874E-B6FC-A64D185F187D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="620" windowWidth="28800" windowHeight="15660" xr2:uid="{EBDBD758-277E-6B49-B4C7-31ED6652B0E7}"/>
+    <workbookView xWindow="0" yWindow="620" windowWidth="28800" windowHeight="15660" activeTab="3" xr2:uid="{EBDBD758-277E-6B49-B4C7-31ED6652B0E7}"/>
   </bookViews>
   <sheets>
     <sheet name="Startup" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="717" uniqueCount="654">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="684" uniqueCount="643">
   <si>
     <t>Company Name</t>
   </si>
@@ -74,9 +74,6 @@
     <t>Ayar Labs</t>
   </si>
   <si>
-    <t>200+</t>
-  </si>
-  <si>
     <t xml:space="preserve">Optical I/O for AI, Interconnection </t>
   </si>
   <si>
@@ -230,15 +227,9 @@
     <t>Vivek Raghunathan, Michal Lipson, Keren Bergman, Columbia</t>
   </si>
   <si>
-    <t>&lt; 50</t>
-  </si>
-  <si>
     <t>Optelligence</t>
   </si>
   <si>
-    <t>&lt; 3</t>
-  </si>
-  <si>
     <t xml:space="preserve">Photonic AI </t>
   </si>
   <si>
@@ -260,9 +251,6 @@
     <t>Santa Clara, CA, USA</t>
   </si>
   <si>
-    <t>&lt; 200</t>
-  </si>
-  <si>
     <t>David Lazovsky</t>
   </si>
   <si>
@@ -284,9 +272,6 @@
     <t>Nubis Communications</t>
   </si>
   <si>
-    <t xml:space="preserve">&lt; 50 </t>
-  </si>
-  <si>
     <t>Voyant Photonics</t>
   </si>
   <si>
@@ -296,9 +281,6 @@
     <t>Steven Miller, Michel Lipson</t>
   </si>
   <si>
-    <t>&lt; 30</t>
-  </si>
-  <si>
     <t>Aegiq</t>
   </si>
   <si>
@@ -362,9 +344,6 @@
     <t>error-corrected photonic quantum computers</t>
   </si>
   <si>
-    <t>~100</t>
-  </si>
-  <si>
     <t>Professor Ian Walmsley, Josh Nunn, Richard Murray, University of Oxford</t>
   </si>
   <si>
@@ -413,9 +392,6 @@
     <t>Lumiphase</t>
   </si>
   <si>
-    <t xml:space="preserve">&lt; 100 </t>
-  </si>
-  <si>
     <t>Optical interconnects and computing using Si Ph and BTO</t>
   </si>
   <si>
@@ -441,9 +417,6 @@
   </si>
   <si>
     <t>Nexus Photonics</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt; 20 </t>
   </si>
   <si>
     <t>Advanced heterogeneous integration, SiN, GaAs, GaN, InP</t>
@@ -537,9 +510,6 @@
     <t xml:space="preserve">Quantum: Hartmut Neven, Taara: Mahesh Krishnaswamy </t>
   </si>
   <si>
-    <t>300+</t>
-  </si>
-  <si>
     <t>Fiber Sensing, Optical Compute, Fiber Telecommunication Optimization</t>
   </si>
   <si>
@@ -1593,9 +1563,6 @@
   </si>
   <si>
     <t>thin‑film lithium niobate (TFLN) and lithium tantalate (TFLT) photonics.</t>
-  </si>
-  <si>
-    <t>&lt; 10</t>
   </si>
   <si>
     <t>Mohammad Bereyhi, CEO &amp; Co‑Founder. Alberto Beccari, CTO, EPFL spinout</t>
@@ -2569,7 +2536,7 @@
         <v>7</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>148</v>
+        <v>139</v>
       </c>
     </row>
     <row r="3" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -2586,7 +2553,7 @@
         <v>6</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>149</v>
+        <v>140</v>
       </c>
     </row>
     <row r="4" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -2603,1520 +2570,1520 @@
         <v>9</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>137</v>
+        <v>128</v>
       </c>
     </row>
     <row r="5" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" s="3">
+        <v>200</v>
+      </c>
+      <c r="D5" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D5" s="1" t="s">
+      <c r="E5" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="1" t="s">
+      <c r="F5" s="1" t="s">
         <v>13</v>
-      </c>
-      <c r="F5" s="1" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="6" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C6" s="3">
         <v>280</v>
       </c>
       <c r="D6" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="E6" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="E6" s="1" t="s">
+      <c r="F6" s="1" t="s">
         <v>35</v>
-      </c>
-      <c r="F6" s="1" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="7" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B7" s="3" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C7" s="3">
         <v>50</v>
       </c>
       <c r="D7" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="E7" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="E7" s="1" t="s">
-        <v>38</v>
-      </c>
       <c r="F7" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="8" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B8" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C8" s="3">
         <v>100</v>
       </c>
       <c r="D8" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="E8" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="E8" s="1" t="s">
+      <c r="F8" s="1" t="s">
         <v>42</v>
-      </c>
-      <c r="F8" s="1" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="9" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B9" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C9" s="3">
         <v>20</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>615</v>
+        <v>604</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="10" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="C10" s="3">
+        <v>50</v>
+      </c>
+      <c r="D10" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="C10" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="D10" s="1" t="s">
+      <c r="E10" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="F10" s="1" t="s">
         <v>47</v>
-      </c>
-      <c r="E10" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="F10" s="1" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="11" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B11" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="C11" s="3">
+        <v>50</v>
+      </c>
+      <c r="D11" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="C11" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="D11" s="1" t="s">
-        <v>50</v>
-      </c>
       <c r="E11" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="12" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B12" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="C12" s="3" t="s">
-        <v>63</v>
+        <v>50</v>
+      </c>
+      <c r="C12" s="3">
+        <v>50</v>
       </c>
       <c r="D12" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="E12" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="E12" s="1" t="s">
+      <c r="F12" s="1" t="s">
         <v>54</v>
-      </c>
-      <c r="F12" s="1" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="13" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B13" s="3" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C13" s="3">
         <v>10</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>153</v>
+        <v>144</v>
       </c>
     </row>
     <row r="14" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B14" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="C14" s="3" t="s">
-        <v>63</v>
+        <v>26</v>
+      </c>
+      <c r="C14" s="3">
+        <v>50</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>154</v>
+        <v>145</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="15" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B15" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="C15" s="3" t="s">
-        <v>73</v>
+        <v>31</v>
+      </c>
+      <c r="C15" s="3">
+        <v>200</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
     </row>
     <row r="16" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B16" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="C16" s="3">
+        <v>50</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="E16" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="C16" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="D16" s="1" t="s">
-        <v>138</v>
-      </c>
-      <c r="E16" s="1" t="s">
-        <v>62</v>
-      </c>
       <c r="F16" s="1" t="s">
-        <v>176</v>
+        <v>166</v>
       </c>
     </row>
     <row r="17" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B17" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="C17" s="3">
+        <v>3</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="E17" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="C17" s="3" t="s">
+      <c r="F17" s="1" t="s">
         <v>65</v>
-      </c>
-      <c r="D17" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="E17" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="F17" s="1" t="s">
-        <v>68</v>
       </c>
     </row>
     <row r="18" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B18" s="3" t="s">
-        <v>80</v>
-      </c>
-      <c r="C18" s="3" t="s">
-        <v>81</v>
+        <v>76</v>
+      </c>
+      <c r="C18" s="3">
+        <v>50</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
     </row>
     <row r="19" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B19" s="3" t="s">
-        <v>82</v>
-      </c>
-      <c r="C19" s="3" t="s">
-        <v>85</v>
+        <v>77</v>
+      </c>
+      <c r="C19" s="3">
+        <v>30</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>176</v>
+        <v>166</v>
       </c>
     </row>
     <row r="20" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B20" s="3" t="s">
-        <v>86</v>
-      </c>
-      <c r="C20" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="C20" s="3">
+        <v>50</v>
+      </c>
+      <c r="D20" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="D20" s="1" t="s">
-        <v>87</v>
-      </c>
       <c r="E20" s="1" t="s">
-        <v>89</v>
+        <v>83</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>88</v>
+        <v>82</v>
       </c>
     </row>
     <row r="21" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B21" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="C21" s="3" t="s">
-        <v>81</v>
+        <v>84</v>
+      </c>
+      <c r="C21" s="3">
+        <v>50</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>91</v>
+        <v>85</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>93</v>
+        <v>87</v>
       </c>
     </row>
     <row r="22" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B22" s="3" t="s">
-        <v>96</v>
+        <v>90</v>
       </c>
       <c r="C22" s="3">
         <v>50</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>97</v>
+        <v>91</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>99</v>
+        <v>93</v>
       </c>
     </row>
     <row r="23" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B23" s="3" t="s">
-        <v>102</v>
-      </c>
-      <c r="C23" s="3" t="s">
-        <v>104</v>
+        <v>96</v>
+      </c>
+      <c r="C23" s="3">
+        <v>0</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>104</v>
+        <v>98</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>104</v>
+        <v>98</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
     </row>
     <row r="24" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B24" s="3" t="s">
-        <v>105</v>
-      </c>
-      <c r="C24" s="3" t="s">
-        <v>107</v>
+        <v>99</v>
+      </c>
+      <c r="C24" s="3">
+        <v>100</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>108</v>
+        <v>101</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>152</v>
+        <v>143</v>
       </c>
     </row>
     <row r="25" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B25" s="3" t="s">
-        <v>109</v>
-      </c>
-      <c r="C25" s="3" t="s">
-        <v>63</v>
+        <v>102</v>
+      </c>
+      <c r="C25" s="3">
+        <v>50</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>110</v>
+        <v>103</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>111</v>
+        <v>104</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>153</v>
+        <v>144</v>
       </c>
     </row>
     <row r="26" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B26" s="3" t="s">
-        <v>112</v>
-      </c>
-      <c r="C26" s="3" t="s">
-        <v>63</v>
+        <v>105</v>
+      </c>
+      <c r="C26" s="3">
+        <v>50</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>110</v>
+        <v>103</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>114</v>
+        <v>107</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>113</v>
+        <v>106</v>
       </c>
     </row>
     <row r="27" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B27" s="3" t="s">
-        <v>115</v>
-      </c>
-      <c r="C27" s="3" t="s">
-        <v>63</v>
+        <v>108</v>
+      </c>
+      <c r="C27" s="3">
+        <v>50</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>117</v>
+        <v>110</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>116</v>
+        <v>109</v>
       </c>
       <c r="F27" s="1" t="s">
-        <v>150</v>
+        <v>141</v>
       </c>
     </row>
     <row r="28" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B28" s="3" t="s">
-        <v>119</v>
-      </c>
-      <c r="C28" s="3" t="s">
-        <v>81</v>
+        <v>112</v>
+      </c>
+      <c r="C28" s="3">
+        <v>50</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>118</v>
+        <v>111</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>121</v>
+        <v>114</v>
       </c>
       <c r="F28" s="1" t="s">
-        <v>120</v>
+        <v>113</v>
       </c>
     </row>
     <row r="29" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B29" s="3" t="s">
-        <v>123</v>
-      </c>
-      <c r="C29" s="3" t="s">
-        <v>124</v>
+        <v>116</v>
+      </c>
+      <c r="C29" s="3">
+        <v>100</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>125</v>
+        <v>117</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="F29" s="1" t="s">
-        <v>126</v>
+        <v>118</v>
       </c>
     </row>
     <row r="30" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B30" s="3" t="s">
-        <v>130</v>
-      </c>
-      <c r="C30" s="3" t="s">
-        <v>81</v>
+        <v>122</v>
+      </c>
+      <c r="C30" s="3">
+        <v>50</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>131</v>
+        <v>123</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>132</v>
+        <v>124</v>
       </c>
       <c r="F30" s="1" t="s">
-        <v>224</v>
+        <v>214</v>
       </c>
     </row>
     <row r="31" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B31" s="3" t="s">
-        <v>133</v>
-      </c>
-      <c r="C31" s="3" t="s">
-        <v>134</v>
+        <v>125</v>
+      </c>
+      <c r="C31" s="3">
+        <v>20</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>135</v>
+        <v>126</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>155</v>
+        <v>146</v>
       </c>
       <c r="F31" s="1" t="s">
-        <v>151</v>
+        <v>142</v>
       </c>
     </row>
     <row r="32" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B32" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="C32" s="3">
+        <v>200</v>
+      </c>
+      <c r="D32" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="E32" s="1" t="s">
         <v>147</v>
       </c>
-      <c r="C32" s="3" t="s">
-        <v>73</v>
-      </c>
-      <c r="D32" s="1" t="s">
-        <v>157</v>
-      </c>
-      <c r="E32" s="1" t="s">
-        <v>156</v>
-      </c>
       <c r="F32" s="1" t="s">
-        <v>136</v>
+        <v>127</v>
       </c>
     </row>
     <row r="33" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B33" s="3" t="s">
-        <v>241</v>
+        <v>231</v>
       </c>
       <c r="C33" s="3">
         <v>10</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>242</v>
+        <v>232</v>
       </c>
       <c r="E33" s="1" t="s">
-        <v>244</v>
+        <v>234</v>
       </c>
       <c r="F33" s="1" t="s">
-        <v>243</v>
+        <v>233</v>
       </c>
     </row>
     <row r="34" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B34" s="3" t="s">
-        <v>288</v>
+        <v>278</v>
       </c>
       <c r="C34" s="3">
         <v>190</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>289</v>
+        <v>279</v>
       </c>
       <c r="E34" s="1" t="s">
-        <v>295</v>
+        <v>285</v>
       </c>
       <c r="F34" s="1" t="s">
-        <v>290</v>
+        <v>280</v>
       </c>
     </row>
     <row r="35" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B35" s="3" t="s">
-        <v>291</v>
+        <v>281</v>
       </c>
       <c r="C35" s="3">
         <v>30</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>292</v>
+        <v>282</v>
       </c>
       <c r="E35" s="1" t="s">
-        <v>293</v>
+        <v>283</v>
       </c>
       <c r="F35" s="1" t="s">
-        <v>294</v>
+        <v>284</v>
       </c>
     </row>
     <row r="36" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B36" s="3" t="s">
-        <v>296</v>
+        <v>286</v>
       </c>
       <c r="C36" s="3">
         <v>15</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>530</v>
+        <v>519</v>
       </c>
       <c r="E36" s="1" t="s">
-        <v>529</v>
+        <v>518</v>
       </c>
       <c r="F36" s="1" t="s">
-        <v>297</v>
+        <v>287</v>
       </c>
     </row>
     <row r="37" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B37" s="3" t="s">
-        <v>302</v>
+        <v>292</v>
       </c>
       <c r="C37" s="3">
         <v>40</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>305</v>
+        <v>295</v>
       </c>
       <c r="E37" s="1" t="s">
-        <v>304</v>
+        <v>294</v>
       </c>
       <c r="F37" s="1" t="s">
-        <v>303</v>
+        <v>293</v>
       </c>
     </row>
     <row r="38" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B38" s="3" t="s">
-        <v>310</v>
+        <v>300</v>
       </c>
       <c r="C38" s="3">
         <v>30</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>311</v>
+        <v>301</v>
       </c>
       <c r="E38" s="1" t="s">
-        <v>312</v>
+        <v>302</v>
       </c>
       <c r="F38" s="1" t="s">
-        <v>313</v>
+        <v>303</v>
       </c>
     </row>
     <row r="39" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B39" s="3" t="s">
-        <v>331</v>
+        <v>321</v>
       </c>
       <c r="C39" s="3">
         <v>50</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>329</v>
+        <v>319</v>
       </c>
       <c r="E39" s="1" t="s">
-        <v>330</v>
+        <v>320</v>
       </c>
       <c r="F39" s="1" t="s">
-        <v>333</v>
+        <v>323</v>
       </c>
     </row>
     <row r="40" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B40" s="3" t="s">
-        <v>342</v>
+        <v>332</v>
       </c>
       <c r="C40" s="3">
         <v>20</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>344</v>
+        <v>334</v>
       </c>
       <c r="E40" s="1" t="s">
-        <v>345</v>
+        <v>335</v>
       </c>
       <c r="F40" s="1" t="s">
-        <v>343</v>
+        <v>333</v>
       </c>
     </row>
     <row r="41" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B41" s="3" t="s">
-        <v>346</v>
+        <v>336</v>
       </c>
       <c r="C41" s="3">
         <v>81</v>
       </c>
       <c r="D41" s="1" t="s">
-        <v>347</v>
+        <v>337</v>
       </c>
       <c r="E41" s="1" t="s">
-        <v>349</v>
+        <v>339</v>
       </c>
       <c r="F41" s="1" t="s">
-        <v>348</v>
+        <v>338</v>
       </c>
     </row>
     <row r="42" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B42" s="3" t="s">
-        <v>350</v>
+        <v>340</v>
       </c>
       <c r="C42" s="3">
         <v>120</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>351</v>
+        <v>341</v>
       </c>
       <c r="E42" s="1" t="s">
-        <v>353</v>
+        <v>343</v>
       </c>
       <c r="F42" s="1" t="s">
-        <v>352</v>
+        <v>342</v>
       </c>
     </row>
     <row r="43" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B43" s="3" t="s">
-        <v>354</v>
+        <v>344</v>
       </c>
       <c r="C43" s="3">
         <v>20</v>
       </c>
       <c r="D43" s="1" t="s">
-        <v>355</v>
+        <v>345</v>
       </c>
       <c r="E43" s="1" t="s">
-        <v>356</v>
+        <v>346</v>
       </c>
       <c r="F43" s="1" t="s">
-        <v>357</v>
+        <v>347</v>
       </c>
     </row>
     <row r="44" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B44" s="3" t="s">
-        <v>358</v>
+        <v>348</v>
       </c>
       <c r="C44" s="3">
         <v>50</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>359</v>
+        <v>349</v>
       </c>
       <c r="E44" s="1" t="s">
-        <v>360</v>
+        <v>350</v>
       </c>
       <c r="F44" s="1" t="s">
-        <v>361</v>
+        <v>351</v>
       </c>
     </row>
     <row r="45" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B45" s="3" t="s">
-        <v>365</v>
+        <v>355</v>
       </c>
       <c r="C45" s="3">
         <v>20</v>
       </c>
       <c r="D45" s="1" t="s">
-        <v>367</v>
+        <v>357</v>
       </c>
       <c r="E45" s="1" t="s">
-        <v>366</v>
+        <v>356</v>
       </c>
       <c r="F45" s="1" t="s">
-        <v>368</v>
+        <v>358</v>
       </c>
     </row>
     <row r="46" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B46" s="3" t="s">
-        <v>369</v>
+        <v>359</v>
       </c>
       <c r="C46" s="3">
         <v>50</v>
       </c>
       <c r="D46" s="1" t="s">
-        <v>370</v>
+        <v>360</v>
       </c>
       <c r="E46" s="1" t="s">
-        <v>371</v>
+        <v>361</v>
       </c>
       <c r="F46" s="1" t="s">
-        <v>372</v>
+        <v>362</v>
       </c>
     </row>
     <row r="47" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B47" s="3" t="s">
-        <v>380</v>
+        <v>370</v>
       </c>
       <c r="C47" s="3">
         <v>150</v>
       </c>
       <c r="D47" s="1" t="s">
-        <v>379</v>
+        <v>369</v>
       </c>
       <c r="E47" s="1" t="s">
-        <v>378</v>
+        <v>368</v>
       </c>
       <c r="F47" s="1" t="s">
-        <v>377</v>
+        <v>367</v>
       </c>
     </row>
     <row r="48" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B48" s="3" t="s">
-        <v>385</v>
+        <v>375</v>
       </c>
       <c r="C48" s="3">
         <v>3</v>
       </c>
       <c r="D48" s="1" t="s">
-        <v>388</v>
+        <v>378</v>
       </c>
       <c r="E48" s="1" t="s">
-        <v>389</v>
+        <v>379</v>
       </c>
       <c r="F48" s="1" t="s">
-        <v>387</v>
+        <v>377</v>
       </c>
     </row>
     <row r="49" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B49" s="3" t="s">
-        <v>433</v>
+        <v>423</v>
       </c>
       <c r="C49" s="3">
         <v>104</v>
       </c>
       <c r="D49" s="1" t="s">
-        <v>434</v>
+        <v>424</v>
       </c>
       <c r="E49" s="1" t="s">
-        <v>435</v>
+        <v>425</v>
       </c>
       <c r="F49" s="1" t="s">
-        <v>432</v>
+        <v>422</v>
       </c>
     </row>
     <row r="50" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B50" s="3" t="s">
-        <v>439</v>
+        <v>429</v>
       </c>
       <c r="C50" s="3">
         <v>50</v>
       </c>
       <c r="D50" s="1" t="s">
-        <v>437</v>
+        <v>427</v>
       </c>
       <c r="E50" s="1" t="s">
-        <v>438</v>
+        <v>428</v>
       </c>
       <c r="F50" s="1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="51" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B51" s="3" t="s">
-        <v>446</v>
+        <v>436</v>
       </c>
       <c r="C51" s="3">
         <v>26</v>
       </c>
       <c r="D51" s="1" t="s">
-        <v>445</v>
+        <v>435</v>
       </c>
       <c r="E51" s="1" t="s">
-        <v>444</v>
+        <v>434</v>
       </c>
       <c r="F51" s="1" t="s">
-        <v>448</v>
+        <v>438</v>
       </c>
     </row>
     <row r="52" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B52" s="3" t="s">
-        <v>449</v>
+        <v>439</v>
       </c>
       <c r="C52" s="3">
         <v>21</v>
       </c>
       <c r="D52" s="1" t="s">
-        <v>450</v>
+        <v>440</v>
       </c>
       <c r="E52" s="1" t="s">
-        <v>451</v>
+        <v>441</v>
       </c>
       <c r="F52" s="1" t="s">
-        <v>447</v>
+        <v>437</v>
       </c>
     </row>
     <row r="53" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B53" s="3" t="s">
-        <v>452</v>
+        <v>442</v>
       </c>
       <c r="C53" s="3">
         <v>5</v>
       </c>
       <c r="D53" s="1" t="s">
-        <v>455</v>
+        <v>445</v>
       </c>
       <c r="E53" s="1" t="s">
-        <v>453</v>
+        <v>443</v>
       </c>
       <c r="F53" s="1" t="s">
-        <v>454</v>
+        <v>444</v>
       </c>
     </row>
     <row r="54" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B54" s="3" t="s">
-        <v>460</v>
+        <v>450</v>
       </c>
       <c r="C54" s="3">
         <v>207</v>
       </c>
       <c r="D54" s="1" t="s">
-        <v>461</v>
+        <v>451</v>
       </c>
       <c r="E54" s="1" t="s">
-        <v>462</v>
+        <v>452</v>
       </c>
       <c r="F54" s="1" t="s">
-        <v>482</v>
+        <v>472</v>
       </c>
     </row>
     <row r="55" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B55" s="3" t="s">
-        <v>465</v>
+        <v>455</v>
       </c>
       <c r="C55" s="3">
         <v>10</v>
       </c>
       <c r="D55" s="1" t="s">
-        <v>464</v>
+        <v>454</v>
       </c>
       <c r="E55" s="1" t="s">
-        <v>463</v>
+        <v>453</v>
       </c>
       <c r="F55" s="1" t="s">
-        <v>466</v>
+        <v>456</v>
       </c>
     </row>
     <row r="56" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B56" s="3" t="s">
-        <v>467</v>
+        <v>457</v>
       </c>
       <c r="C56" s="3">
         <v>13</v>
       </c>
       <c r="D56" s="1" t="s">
-        <v>468</v>
+        <v>458</v>
       </c>
       <c r="E56" s="1" t="s">
-        <v>470</v>
+        <v>460</v>
       </c>
       <c r="F56" s="1" t="s">
-        <v>469</v>
+        <v>459</v>
       </c>
     </row>
     <row r="57" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B57" s="3" t="s">
-        <v>471</v>
+        <v>461</v>
       </c>
       <c r="C57" s="3">
         <v>5</v>
       </c>
       <c r="D57" s="1" t="s">
-        <v>472</v>
+        <v>462</v>
       </c>
       <c r="E57" s="1" t="s">
-        <v>473</v>
+        <v>463</v>
       </c>
       <c r="F57" s="1" t="s">
-        <v>474</v>
+        <v>464</v>
       </c>
     </row>
     <row r="58" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B58" s="3" t="s">
-        <v>478</v>
+        <v>468</v>
       </c>
       <c r="C58" s="3">
         <v>50</v>
       </c>
       <c r="D58" s="1" t="s">
-        <v>479</v>
+        <v>469</v>
       </c>
       <c r="E58" s="1" t="s">
-        <v>480</v>
+        <v>470</v>
       </c>
       <c r="F58" s="1" t="s">
-        <v>481</v>
+        <v>471</v>
       </c>
     </row>
     <row r="59" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B59" s="3" t="s">
-        <v>483</v>
-      </c>
-      <c r="C59" s="3" t="s">
-        <v>63</v>
+        <v>473</v>
+      </c>
+      <c r="C59" s="3">
+        <v>50</v>
       </c>
       <c r="D59" s="1" t="s">
-        <v>484</v>
+        <v>474</v>
       </c>
       <c r="E59" s="1" t="s">
-        <v>485</v>
+        <v>475</v>
       </c>
       <c r="F59" s="1" t="s">
-        <v>486</v>
+        <v>476</v>
       </c>
     </row>
     <row r="60" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B60" s="3" t="s">
-        <v>490</v>
-      </c>
-      <c r="C60" s="3" t="s">
-        <v>81</v>
+        <v>480</v>
+      </c>
+      <c r="C60" s="3">
+        <v>50</v>
       </c>
       <c r="D60" s="1" t="s">
-        <v>487</v>
+        <v>477</v>
       </c>
       <c r="E60" s="1" t="s">
-        <v>488</v>
+        <v>478</v>
       </c>
       <c r="F60" s="1" t="s">
-        <v>489</v>
+        <v>479</v>
       </c>
     </row>
     <row r="61" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B61" s="3" t="s">
-        <v>491</v>
+        <v>481</v>
       </c>
       <c r="C61" s="3">
         <v>50</v>
       </c>
       <c r="D61" s="1" t="s">
-        <v>492</v>
+        <v>482</v>
       </c>
       <c r="E61" s="1" t="s">
-        <v>493</v>
+        <v>483</v>
       </c>
       <c r="F61" s="1" t="s">
-        <v>494</v>
+        <v>484</v>
       </c>
     </row>
     <row r="62" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B62" s="3" t="s">
-        <v>495</v>
-      </c>
-      <c r="C62" s="3" t="s">
-        <v>73</v>
+        <v>485</v>
+      </c>
+      <c r="C62" s="3">
+        <v>200</v>
       </c>
       <c r="D62" s="1" t="s">
-        <v>496</v>
+        <v>486</v>
       </c>
       <c r="E62" s="1" t="s">
-        <v>497</v>
+        <v>487</v>
       </c>
       <c r="F62" s="1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="63" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B63" s="3" t="s">
-        <v>500</v>
-      </c>
-      <c r="C63" s="3" t="s">
-        <v>63</v>
+        <v>490</v>
+      </c>
+      <c r="C63" s="3">
+        <v>50</v>
       </c>
       <c r="D63" s="1" t="s">
-        <v>498</v>
+        <v>488</v>
       </c>
       <c r="E63" s="1" t="s">
-        <v>499</v>
+        <v>489</v>
       </c>
       <c r="F63" s="1" t="s">
-        <v>248</v>
+        <v>238</v>
       </c>
     </row>
     <row r="64" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B64" s="3" t="s">
-        <v>511</v>
+        <v>501</v>
       </c>
       <c r="C64" s="3">
         <v>30</v>
       </c>
       <c r="D64" s="1" t="s">
-        <v>512</v>
+        <v>502</v>
       </c>
       <c r="E64" s="1" t="s">
-        <v>509</v>
+        <v>499</v>
       </c>
       <c r="F64" s="1" t="s">
-        <v>510</v>
+        <v>500</v>
       </c>
     </row>
     <row r="65" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B65" s="3" t="s">
-        <v>514</v>
-      </c>
-      <c r="C65" s="3" t="s">
-        <v>516</v>
+        <v>504</v>
+      </c>
+      <c r="C65" s="3">
+        <v>10</v>
       </c>
       <c r="D65" s="1" t="s">
-        <v>515</v>
+        <v>505</v>
       </c>
       <c r="E65" s="1" t="s">
-        <v>517</v>
+        <v>506</v>
       </c>
       <c r="F65" s="1" t="s">
-        <v>513</v>
+        <v>503</v>
       </c>
     </row>
     <row r="66" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B66" s="3" t="s">
-        <v>518</v>
-      </c>
-      <c r="C66" s="3" t="s">
-        <v>516</v>
+        <v>507</v>
+      </c>
+      <c r="C66" s="3">
+        <v>10</v>
       </c>
       <c r="D66" s="1" t="s">
-        <v>521</v>
+        <v>510</v>
       </c>
       <c r="E66" s="1" t="s">
-        <v>519</v>
+        <v>508</v>
       </c>
       <c r="F66" s="1" t="s">
-        <v>520</v>
+        <v>509</v>
       </c>
     </row>
     <row r="67" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B67" s="3" t="s">
-        <v>522</v>
-      </c>
-      <c r="C67" s="3" t="s">
-        <v>63</v>
+        <v>511</v>
+      </c>
+      <c r="C67" s="3">
+        <v>50</v>
       </c>
       <c r="D67" s="1" t="s">
-        <v>539</v>
+        <v>528</v>
       </c>
       <c r="E67" s="1" t="s">
-        <v>523</v>
+        <v>512</v>
       </c>
       <c r="F67" s="1" t="s">
-        <v>524</v>
+        <v>513</v>
       </c>
     </row>
     <row r="68" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B68" s="3" t="s">
-        <v>528</v>
+        <v>517</v>
       </c>
       <c r="C68" s="3">
         <v>18</v>
       </c>
       <c r="D68" s="1" t="s">
-        <v>527</v>
+        <v>516</v>
       </c>
       <c r="E68" s="1" t="s">
-        <v>526</v>
+        <v>515</v>
       </c>
       <c r="F68" s="1" t="s">
-        <v>525</v>
+        <v>514</v>
       </c>
     </row>
     <row r="69" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B69" s="3" t="s">
-        <v>534</v>
-      </c>
-      <c r="C69" s="3" t="s">
-        <v>85</v>
+        <v>523</v>
+      </c>
+      <c r="C69" s="3">
+        <v>30</v>
       </c>
       <c r="D69" s="1" t="s">
-        <v>533</v>
+        <v>522</v>
       </c>
       <c r="E69" s="1" t="s">
-        <v>531</v>
+        <v>520</v>
       </c>
       <c r="F69" s="1" t="s">
-        <v>532</v>
+        <v>521</v>
       </c>
     </row>
     <row r="70" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B70" s="3" t="s">
-        <v>535</v>
-      </c>
-      <c r="C70" s="3" t="s">
-        <v>143</v>
+        <v>524</v>
+      </c>
+      <c r="C70" s="3">
+        <v>100</v>
       </c>
       <c r="D70" s="1" t="s">
-        <v>538</v>
+        <v>527</v>
       </c>
       <c r="E70" s="1" t="s">
-        <v>536</v>
+        <v>525</v>
       </c>
       <c r="F70" s="1" t="s">
-        <v>537</v>
+        <v>526</v>
       </c>
     </row>
     <row r="71" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B71" s="3" t="s">
-        <v>540</v>
+        <v>529</v>
       </c>
       <c r="C71" s="3">
         <v>10</v>
       </c>
       <c r="D71" s="1" t="s">
-        <v>541</v>
+        <v>530</v>
       </c>
       <c r="E71" s="1" t="s">
-        <v>542</v>
+        <v>531</v>
       </c>
       <c r="F71" s="1" t="s">
-        <v>199</v>
+        <v>189</v>
       </c>
     </row>
     <row r="72" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B72" s="3" t="s">
-        <v>543</v>
+        <v>532</v>
       </c>
       <c r="C72" s="3">
         <v>20</v>
       </c>
       <c r="D72" s="1" t="s">
-        <v>544</v>
+        <v>533</v>
       </c>
       <c r="E72" s="1" t="s">
-        <v>546</v>
+        <v>535</v>
       </c>
       <c r="F72" s="1" t="s">
-        <v>545</v>
+        <v>534</v>
       </c>
     </row>
     <row r="73" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B73" s="3" t="s">
-        <v>547</v>
+        <v>536</v>
       </c>
       <c r="C73" s="3">
         <v>50</v>
       </c>
       <c r="D73" s="1" t="s">
-        <v>549</v>
+        <v>538</v>
       </c>
       <c r="E73" s="1" t="s">
-        <v>550</v>
+        <v>539</v>
       </c>
       <c r="F73" s="1" t="s">
-        <v>548</v>
+        <v>537</v>
       </c>
     </row>
     <row r="74" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B74" s="3" t="s">
-        <v>552</v>
+        <v>541</v>
       </c>
       <c r="C74" s="3">
         <v>22</v>
       </c>
       <c r="D74" s="1" t="s">
-        <v>620</v>
+        <v>609</v>
       </c>
       <c r="E74" s="1" t="s">
-        <v>553</v>
+        <v>542</v>
       </c>
       <c r="F74" s="1" t="s">
-        <v>551</v>
+        <v>540</v>
       </c>
     </row>
     <row r="75" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B75" s="3" t="s">
-        <v>555</v>
-      </c>
-      <c r="C75" s="1">
+        <v>544</v>
+      </c>
+      <c r="C75" s="3">
         <v>10</v>
       </c>
       <c r="D75" s="1" t="s">
-        <v>557</v>
+        <v>546</v>
       </c>
       <c r="E75" s="1" t="s">
-        <v>556</v>
+        <v>545</v>
       </c>
       <c r="F75" s="1" t="s">
-        <v>554</v>
+        <v>543</v>
       </c>
     </row>
     <row r="76" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B76" s="3" t="s">
-        <v>562</v>
-      </c>
-      <c r="C76" s="1">
+        <v>551</v>
+      </c>
+      <c r="C76" s="3">
         <v>10</v>
       </c>
       <c r="D76" s="1" t="s">
-        <v>565</v>
+        <v>554</v>
       </c>
       <c r="E76" s="1" t="s">
-        <v>563</v>
+        <v>552</v>
       </c>
       <c r="F76" s="1" t="s">
-        <v>564</v>
+        <v>553</v>
       </c>
     </row>
     <row r="77" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B77" s="3" t="s">
-        <v>566</v>
+        <v>555</v>
       </c>
       <c r="C77" s="3">
         <v>10</v>
       </c>
       <c r="D77" s="1" t="s">
-        <v>567</v>
+        <v>556</v>
       </c>
       <c r="E77" s="1" t="s">
-        <v>568</v>
+        <v>557</v>
       </c>
       <c r="F77" s="1" t="s">
-        <v>569</v>
+        <v>558</v>
       </c>
     </row>
     <row r="78" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B78" s="3" t="s">
-        <v>570</v>
+        <v>559</v>
       </c>
       <c r="C78" s="3">
         <v>15</v>
       </c>
       <c r="D78" s="1" t="s">
-        <v>571</v>
+        <v>560</v>
       </c>
       <c r="E78" s="1" t="s">
-        <v>572</v>
+        <v>561</v>
       </c>
       <c r="F78" s="1" t="s">
-        <v>573</v>
+        <v>562</v>
       </c>
     </row>
     <row r="79" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B79" s="3" t="s">
-        <v>574</v>
+        <v>563</v>
       </c>
       <c r="C79" s="3">
         <v>25</v>
       </c>
       <c r="D79" s="1" t="s">
-        <v>576</v>
+        <v>565</v>
       </c>
       <c r="E79" s="1" t="s">
-        <v>575</v>
+        <v>564</v>
       </c>
       <c r="F79" s="1" t="s">
-        <v>525</v>
+        <v>514</v>
       </c>
     </row>
     <row r="80" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B80" s="3" t="s">
-        <v>580</v>
+        <v>569</v>
       </c>
       <c r="C80" s="3">
         <v>10</v>
       </c>
       <c r="D80" s="1" t="s">
-        <v>581</v>
+        <v>570</v>
       </c>
       <c r="E80" s="1" t="s">
-        <v>582</v>
+        <v>571</v>
       </c>
       <c r="F80" s="1" t="s">
-        <v>583</v>
+        <v>572</v>
       </c>
     </row>
     <row r="81" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B81" s="3" t="s">
-        <v>588</v>
+        <v>577</v>
       </c>
       <c r="C81" s="3">
         <v>25</v>
       </c>
       <c r="D81" s="1" t="s">
-        <v>589</v>
+        <v>578</v>
       </c>
       <c r="E81" s="1" t="s">
-        <v>590</v>
+        <v>579</v>
       </c>
       <c r="F81" s="1" t="s">
-        <v>591</v>
+        <v>580</v>
       </c>
     </row>
     <row r="82" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B82" s="3" t="s">
-        <v>592</v>
+        <v>581</v>
       </c>
       <c r="C82" s="3">
         <v>30</v>
       </c>
       <c r="D82" s="1" t="s">
-        <v>593</v>
+        <v>582</v>
       </c>
       <c r="E82" s="1" t="s">
-        <v>594</v>
+        <v>583</v>
       </c>
       <c r="F82" s="1" t="s">
-        <v>595</v>
+        <v>584</v>
       </c>
     </row>
     <row r="83" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B83" s="3" t="s">
-        <v>596</v>
+        <v>585</v>
       </c>
       <c r="C83" s="3">
         <v>41</v>
       </c>
       <c r="D83" s="1" t="s">
-        <v>597</v>
+        <v>586</v>
       </c>
       <c r="E83" s="1" t="s">
-        <v>599</v>
+        <v>588</v>
       </c>
       <c r="F83" s="1" t="s">
-        <v>598</v>
+        <v>587</v>
       </c>
     </row>
     <row r="84" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B84" s="3" t="s">
-        <v>600</v>
+        <v>589</v>
       </c>
       <c r="C84" s="3">
         <v>100</v>
       </c>
       <c r="D84" s="1" t="s">
-        <v>601</v>
+        <v>590</v>
       </c>
       <c r="E84" s="1" t="s">
-        <v>602</v>
+        <v>591</v>
       </c>
       <c r="F84" s="1" t="s">
-        <v>603</v>
+        <v>592</v>
       </c>
     </row>
     <row r="85" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B85" s="3" t="s">
-        <v>604</v>
+        <v>593</v>
       </c>
       <c r="C85" s="3">
         <v>28</v>
       </c>
       <c r="D85" s="1" t="s">
-        <v>607</v>
+        <v>596</v>
       </c>
       <c r="E85" s="1" t="s">
-        <v>605</v>
+        <v>594</v>
       </c>
       <c r="F85" s="1" t="s">
-        <v>606</v>
+        <v>595</v>
       </c>
     </row>
     <row r="86" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B86" s="3" t="s">
-        <v>608</v>
+        <v>597</v>
       </c>
       <c r="C86" s="3">
         <v>25</v>
       </c>
       <c r="D86" s="1" t="s">
-        <v>609</v>
+        <v>598</v>
       </c>
       <c r="E86" s="1" t="s">
-        <v>610</v>
+        <v>599</v>
       </c>
       <c r="F86" s="1" t="s">
-        <v>573</v>
+        <v>562</v>
       </c>
     </row>
     <row r="87" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B87" s="3" t="s">
-        <v>611</v>
+        <v>600</v>
       </c>
       <c r="C87" s="3">
         <v>10</v>
       </c>
       <c r="D87" s="1" t="s">
-        <v>614</v>
+        <v>603</v>
       </c>
       <c r="E87" s="1" t="s">
-        <v>613</v>
+        <v>602</v>
       </c>
       <c r="F87" s="1" t="s">
-        <v>612</v>
+        <v>601</v>
       </c>
     </row>
     <row r="88" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B88" s="3" t="s">
-        <v>622</v>
+        <v>611</v>
       </c>
       <c r="C88" s="3">
         <v>20</v>
       </c>
       <c r="D88" s="1" t="s">
-        <v>623</v>
+        <v>612</v>
       </c>
       <c r="E88" s="1" t="s">
-        <v>624</v>
+        <v>613</v>
       </c>
       <c r="F88" s="1" t="s">
-        <v>625</v>
+        <v>614</v>
       </c>
     </row>
     <row r="89" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B89" s="3" t="s">
-        <v>626</v>
+        <v>615</v>
       </c>
       <c r="C89" s="3">
         <v>20</v>
       </c>
       <c r="D89" s="1" t="s">
-        <v>629</v>
+        <v>618</v>
       </c>
       <c r="E89" s="1" t="s">
-        <v>627</v>
+        <v>616</v>
       </c>
       <c r="F89" s="1" t="s">
-        <v>628</v>
+        <v>617</v>
       </c>
     </row>
     <row r="90" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B90" s="3" t="s">
-        <v>630</v>
+        <v>619</v>
       </c>
       <c r="C90" s="3">
         <v>20</v>
       </c>
       <c r="D90" s="1" t="s">
-        <v>631</v>
+        <v>620</v>
       </c>
       <c r="E90" s="1" t="s">
-        <v>632</v>
+        <v>621</v>
       </c>
       <c r="F90" s="1" t="s">
-        <v>633</v>
+        <v>622</v>
       </c>
     </row>
     <row r="91" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B91" s="3" t="s">
-        <v>634</v>
+        <v>623</v>
       </c>
       <c r="C91" s="3">
         <v>10</v>
       </c>
       <c r="D91" s="8" t="s">
-        <v>636</v>
+        <v>625</v>
       </c>
       <c r="E91" s="1" t="s">
-        <v>635</v>
+        <v>624</v>
       </c>
       <c r="F91" s="1" t="s">
-        <v>637</v>
+        <v>626</v>
       </c>
     </row>
     <row r="92" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B92" s="3" t="s">
-        <v>638</v>
+        <v>627</v>
       </c>
       <c r="C92" s="3">
         <v>10</v>
       </c>
       <c r="D92" s="1" t="s">
-        <v>640</v>
+        <v>629</v>
       </c>
       <c r="E92" s="1" t="s">
-        <v>639</v>
+        <v>628</v>
       </c>
       <c r="F92" s="1" t="s">
-        <v>595</v>
+        <v>584</v>
       </c>
     </row>
     <row r="93" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B93" s="3" t="s">
-        <v>650</v>
+        <v>639</v>
       </c>
       <c r="C93" s="3">
         <v>43</v>
       </c>
       <c r="D93" s="1" t="s">
-        <v>651</v>
+        <v>640</v>
       </c>
       <c r="E93" s="1" t="s">
-        <v>652</v>
+        <v>641</v>
       </c>
       <c r="F93" s="1" t="s">
-        <v>653</v>
+        <v>642</v>
       </c>
     </row>
     <row r="94" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -4160,534 +4127,534 @@
         <v>7</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>148</v>
+        <v>139</v>
       </c>
     </row>
     <row r="3" spans="2:6" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B3" s="3" t="s">
-        <v>160</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>11</v>
+        <v>151</v>
+      </c>
+      <c r="C3" s="3">
+        <v>200</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>158</v>
+        <v>149</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>159</v>
+        <v>150</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>161</v>
+        <v>152</v>
       </c>
     </row>
     <row r="4" spans="2:6" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>165</v>
+        <v>18</v>
+      </c>
+      <c r="C4" s="3">
+        <v>300</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>163</v>
+        <v>154</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>164</v>
+        <v>155</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>162</v>
+        <v>153</v>
       </c>
     </row>
     <row r="5" spans="2:6" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="3" t="s">
-        <v>253</v>
+        <v>243</v>
       </c>
       <c r="C5" s="3">
         <v>500</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>166</v>
+        <v>156</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>171</v>
+        <v>161</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>254</v>
+        <v>244</v>
       </c>
     </row>
     <row r="6" spans="2:6" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="3" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C6" s="3">
         <v>700</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>167</v>
+        <v>157</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>168</v>
+        <v>158</v>
       </c>
     </row>
     <row r="7" spans="2:6" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B7" s="3" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C7" s="3">
         <v>470</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>173</v>
+        <v>163</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>172</v>
+        <v>162</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>170</v>
+        <v>160</v>
       </c>
     </row>
     <row r="8" spans="2:6" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B8" s="3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C8" s="7">
         <v>1500</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>225</v>
+        <v>215</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>226</v>
+        <v>216</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>227</v>
+        <v>217</v>
       </c>
     </row>
     <row r="9" spans="2:6" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B9" s="3" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C9" s="7">
         <v>30000</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>230</v>
+        <v>220</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>229</v>
+        <v>219</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>228</v>
+        <v>218</v>
       </c>
     </row>
     <row r="10" spans="2:6" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="3" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C10" s="7">
         <v>5000</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>234</v>
+        <v>224</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>261</v>
+        <v>251</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>285</v>
+        <v>275</v>
       </c>
     </row>
     <row r="11" spans="2:6" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B11" s="3" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="C11" s="7">
         <v>8000</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>268</v>
+        <v>258</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>270</v>
+        <v>260</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>269</v>
+        <v>259</v>
       </c>
     </row>
     <row r="12" spans="2:6" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B12" s="3" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="C12" s="3">
         <v>150</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>273</v>
+        <v>263</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>271</v>
+        <v>261</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>272</v>
+        <v>262</v>
       </c>
     </row>
     <row r="13" spans="2:6" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B13" s="3" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="C13" s="7">
         <v>700</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>274</v>
+        <v>264</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>276</v>
+        <v>266</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>275</v>
+        <v>265</v>
       </c>
     </row>
     <row r="14" spans="2:6" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B14" s="3" t="s">
-        <v>277</v>
+        <v>267</v>
       </c>
       <c r="C14" s="3">
         <v>800</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>278</v>
+        <v>268</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>279</v>
+        <v>269</v>
       </c>
     </row>
     <row r="15" spans="2:6" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B15" s="3" t="s">
-        <v>282</v>
+        <v>272</v>
       </c>
       <c r="C15" s="7">
         <v>1400</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>283</v>
+        <v>273</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>281</v>
+        <v>271</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>284</v>
+        <v>274</v>
       </c>
     </row>
     <row r="16" spans="2:6" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B16" s="3" t="s">
-        <v>266</v>
+        <v>256</v>
       </c>
       <c r="C16" s="3">
         <v>500</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>264</v>
+        <v>254</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>267</v>
+        <v>257</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>265</v>
+        <v>255</v>
       </c>
     </row>
     <row r="17" spans="2:6" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B17" s="3" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="C17" s="3">
         <v>100</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>262</v>
+        <v>252</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>263</v>
+        <v>253</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>146</v>
+        <v>137</v>
       </c>
     </row>
     <row r="18" spans="2:6" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B18" s="3" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="C18" s="3">
         <v>30</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>259</v>
+        <v>249</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>258</v>
+        <v>248</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>260</v>
+        <v>250</v>
       </c>
     </row>
     <row r="19" spans="2:6" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B19" s="3" t="s">
-        <v>127</v>
+        <v>119</v>
       </c>
       <c r="C19" s="7">
         <v>15000</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>256</v>
+        <v>246</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>257</v>
+        <v>247</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>255</v>
+        <v>245</v>
       </c>
     </row>
     <row r="20" spans="2:6" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B20" s="3" t="s">
-        <v>129</v>
+        <v>121</v>
       </c>
       <c r="C20" s="3">
         <v>14000</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>250</v>
+        <v>240</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>252</v>
+        <v>242</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>251</v>
+        <v>241</v>
       </c>
     </row>
     <row r="21" spans="2:6" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B21" s="3" t="s">
-        <v>231</v>
+        <v>221</v>
       </c>
       <c r="C21" s="3">
         <v>300</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>233</v>
+        <v>223</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>645</v>
+        <v>634</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>232</v>
+        <v>222</v>
       </c>
     </row>
     <row r="22" spans="2:6" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B22" s="3" t="s">
-        <v>239</v>
+        <v>229</v>
       </c>
       <c r="C22" s="3">
         <v>500</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>240</v>
+        <v>230</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>318</v>
+        <v>308</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>249</v>
+        <v>239</v>
       </c>
     </row>
     <row r="23" spans="2:6" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B23" s="3" t="s">
-        <v>314</v>
+        <v>304</v>
       </c>
       <c r="C23" s="3">
         <v>100</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>315</v>
+        <v>305</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>316</v>
+        <v>306</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>317</v>
+        <v>307</v>
       </c>
     </row>
     <row r="24" spans="2:6" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B24" s="3" t="s">
-        <v>320</v>
+        <v>310</v>
       </c>
       <c r="C24" s="3">
         <v>500</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>319</v>
+        <v>309</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>325</v>
+        <v>315</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>176</v>
+        <v>166</v>
       </c>
     </row>
     <row r="25" spans="2:6" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B25" s="3" t="s">
-        <v>321</v>
+        <v>311</v>
       </c>
       <c r="C25" s="3">
         <v>200</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>322</v>
+        <v>312</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>323</v>
+        <v>313</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>324</v>
+        <v>314</v>
       </c>
     </row>
     <row r="26" spans="2:6" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B26" s="3" t="s">
-        <v>336</v>
+        <v>326</v>
       </c>
       <c r="C26" s="3">
         <v>400</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>335</v>
+        <v>325</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>337</v>
+        <v>327</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>334</v>
+        <v>324</v>
       </c>
     </row>
     <row r="27" spans="2:6" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B27" s="3" t="s">
-        <v>381</v>
+        <v>371</v>
       </c>
       <c r="C27" s="3">
         <v>500</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>383</v>
+        <v>373</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>384</v>
+        <v>374</v>
       </c>
       <c r="F27" s="1" t="s">
-        <v>382</v>
+        <v>372</v>
       </c>
     </row>
     <row r="28" spans="2:6" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B28" s="3" t="s">
-        <v>440</v>
+        <v>430</v>
       </c>
       <c r="C28" s="3">
         <v>2000</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>441</v>
+        <v>431</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>442</v>
+        <v>432</v>
       </c>
       <c r="F28" s="1" t="s">
-        <v>443</v>
+        <v>433</v>
       </c>
     </row>
     <row r="29" spans="2:6" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B29" s="3" t="s">
-        <v>456</v>
+        <v>446</v>
       </c>
       <c r="C29" s="3">
         <v>2300</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>457</v>
+        <v>447</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>458</v>
+        <v>448</v>
       </c>
       <c r="F29" s="1" t="s">
-        <v>459</v>
+        <v>449</v>
       </c>
     </row>
     <row r="30" spans="2:6" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B30" s="3" t="s">
-        <v>475</v>
+        <v>465</v>
       </c>
       <c r="C30" s="3">
         <v>5000</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>621</v>
+        <v>610</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>476</v>
+        <v>466</v>
       </c>
       <c r="F30" s="1" t="s">
-        <v>477</v>
+        <v>467</v>
       </c>
     </row>
     <row r="31" spans="2:6" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B31" s="3" t="s">
-        <v>501</v>
+        <v>491</v>
       </c>
       <c r="C31" s="7">
         <v>1294</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>502</v>
+        <v>492</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>503</v>
+        <v>493</v>
       </c>
       <c r="F31" s="1" t="s">
-        <v>504</v>
+        <v>494</v>
       </c>
     </row>
     <row r="32" spans="2:6" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B32" s="3" t="s">
-        <v>505</v>
+        <v>495</v>
       </c>
       <c r="C32" s="7">
         <v>1933</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>506</v>
+        <v>496</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>507</v>
+        <v>497</v>
       </c>
       <c r="F32" s="4" t="s">
-        <v>508</v>
+        <v>498</v>
       </c>
     </row>
     <row r="33" spans="2:6" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B33" s="3" t="s">
-        <v>646</v>
+        <v>635</v>
       </c>
       <c r="C33" s="3">
         <v>756</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>647</v>
+        <v>636</v>
       </c>
       <c r="E33" s="1" t="s">
-        <v>648</v>
+        <v>637</v>
       </c>
       <c r="F33" s="1" t="s">
-        <v>649</v>
+        <v>638</v>
       </c>
     </row>
     <row r="34" spans="2:6" ht="59.25" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -4734,585 +4701,585 @@
         <v>7</v>
       </c>
       <c r="F2" s="11" t="s">
-        <v>148</v>
+        <v>139</v>
       </c>
     </row>
     <row r="3" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B3" s="6" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C3" s="12">
         <v>13000</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>178</v>
+        <v>168</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>179</v>
+        <v>169</v>
       </c>
       <c r="F3" s="6" t="s">
-        <v>223</v>
+        <v>213</v>
       </c>
     </row>
     <row r="4" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B4" s="6" t="s">
-        <v>181</v>
+        <v>171</v>
       </c>
       <c r="C4" s="6">
         <v>500</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>182</v>
+        <v>172</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>186</v>
+        <v>176</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>180</v>
+        <v>170</v>
       </c>
     </row>
     <row r="5" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B5" s="6" t="s">
-        <v>184</v>
+        <v>174</v>
       </c>
       <c r="C5" s="6">
         <v>130</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>185</v>
+        <v>175</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>187</v>
+        <v>177</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>183</v>
+        <v>173</v>
       </c>
     </row>
     <row r="6" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B6" s="6" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>191</v>
+        <v>181</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>189</v>
+        <v>179</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>188</v>
+        <v>178</v>
       </c>
       <c r="F6" s="6" t="s">
-        <v>190</v>
+        <v>180</v>
       </c>
     </row>
     <row r="7" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B7" s="6" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>195</v>
+        <v>185</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>193</v>
+        <v>183</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>194</v>
+        <v>184</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>192</v>
+        <v>182</v>
       </c>
     </row>
     <row r="8" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B8" s="6" t="s">
-        <v>198</v>
+        <v>188</v>
       </c>
       <c r="C8" s="6">
         <v>70</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>196</v>
+        <v>186</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>197</v>
+        <v>187</v>
       </c>
       <c r="F8" s="6" t="s">
-        <v>199</v>
+        <v>189</v>
       </c>
     </row>
     <row r="9" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B9" s="6" t="s">
-        <v>200</v>
+        <v>190</v>
       </c>
       <c r="C9" s="12">
         <v>10000</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>201</v>
+        <v>191</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>202</v>
+        <v>192</v>
       </c>
       <c r="F9" s="6" t="s">
-        <v>222</v>
+        <v>212</v>
       </c>
     </row>
     <row r="10" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B10" s="6" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C10" s="6">
         <v>100</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>205</v>
+        <v>195</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="F10" s="6" t="s">
-        <v>94</v>
+        <v>88</v>
       </c>
     </row>
     <row r="11" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B11" s="6" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>207</v>
+        <v>197</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>208</v>
+        <v>198</v>
       </c>
       <c r="F11" s="6" t="s">
-        <v>209</v>
+        <v>199</v>
       </c>
     </row>
     <row r="12" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B12" s="6" t="s">
-        <v>122</v>
+        <v>115</v>
       </c>
       <c r="C12" s="12">
         <v>5500</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>211</v>
+        <v>201</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>212</v>
+        <v>202</v>
       </c>
       <c r="F12" s="6" t="s">
-        <v>287</v>
+        <v>277</v>
       </c>
     </row>
     <row r="13" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B13" s="6" t="s">
+        <v>193</v>
+      </c>
+      <c r="C13" s="6" t="s">
+        <v>205</v>
+      </c>
+      <c r="D13" s="6" t="s">
         <v>203</v>
       </c>
-      <c r="C13" s="6" t="s">
-        <v>215</v>
-      </c>
-      <c r="D13" s="6" t="s">
-        <v>213</v>
-      </c>
       <c r="E13" s="6" t="s">
-        <v>204</v>
+        <v>194</v>
       </c>
       <c r="F13" s="6" t="s">
-        <v>216</v>
+        <v>206</v>
       </c>
     </row>
     <row r="14" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B14" s="6" t="s">
-        <v>206</v>
+        <v>196</v>
       </c>
       <c r="C14" s="12">
         <v>4500</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>217</v>
+        <v>207</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>218</v>
+        <v>208</v>
       </c>
       <c r="F14" s="6" t="s">
-        <v>286</v>
+        <v>276</v>
       </c>
     </row>
     <row r="15" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B15" s="6" t="s">
-        <v>214</v>
+        <v>204</v>
       </c>
       <c r="C15" s="6">
         <v>20</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>219</v>
+        <v>209</v>
       </c>
       <c r="E15" s="6" t="s">
-        <v>220</v>
+        <v>210</v>
       </c>
       <c r="F15" s="6" t="s">
-        <v>221</v>
+        <v>211</v>
       </c>
     </row>
     <row r="16" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B16" s="6" t="s">
-        <v>237</v>
+        <v>227</v>
       </c>
       <c r="C16" s="6">
         <v>20</v>
       </c>
       <c r="D16" s="6" t="s">
-        <v>235</v>
+        <v>225</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>238</v>
+        <v>228</v>
       </c>
       <c r="F16" s="6" t="s">
-        <v>236</v>
+        <v>226</v>
       </c>
     </row>
     <row r="17" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B17" s="6" t="s">
-        <v>245</v>
+        <v>235</v>
       </c>
       <c r="C17" s="6">
         <v>150</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>246</v>
+        <v>236</v>
       </c>
       <c r="E17" s="6" t="s">
-        <v>247</v>
+        <v>237</v>
       </c>
       <c r="F17" s="6" t="s">
-        <v>248</v>
+        <v>238</v>
       </c>
     </row>
     <row r="18" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B18" s="6" t="s">
-        <v>306</v>
+        <v>296</v>
       </c>
       <c r="C18" s="6">
         <v>1000</v>
       </c>
       <c r="D18" s="6" t="s">
-        <v>308</v>
+        <v>298</v>
       </c>
       <c r="E18" s="6" t="s">
-        <v>307</v>
+        <v>297</v>
       </c>
       <c r="F18" s="9" t="s">
-        <v>309</v>
+        <v>299</v>
       </c>
     </row>
     <row r="19" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B19" s="6" t="s">
-        <v>326</v>
+        <v>316</v>
       </c>
       <c r="C19" s="6">
         <v>20</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>327</v>
+        <v>317</v>
       </c>
       <c r="E19" s="9" t="s">
-        <v>328</v>
+        <v>318</v>
       </c>
       <c r="F19" s="10" t="s">
-        <v>199</v>
+        <v>189</v>
       </c>
     </row>
     <row r="20" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B20" s="6" t="s">
-        <v>331</v>
+        <v>321</v>
       </c>
       <c r="C20" s="6">
         <v>50</v>
       </c>
       <c r="D20" s="6" t="s">
-        <v>329</v>
+        <v>319</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>330</v>
+        <v>320</v>
       </c>
       <c r="F20" s="6" t="s">
-        <v>332</v>
+        <v>322</v>
       </c>
     </row>
     <row r="21" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B21" s="6" t="s">
-        <v>391</v>
+        <v>381</v>
       </c>
       <c r="C21" s="6">
         <v>50</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>390</v>
+        <v>380</v>
       </c>
       <c r="E21" s="6" t="s">
-        <v>393</v>
+        <v>383</v>
       </c>
       <c r="F21" s="6" t="s">
-        <v>392</v>
+        <v>382</v>
       </c>
     </row>
     <row r="22" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B22" s="6" t="s">
-        <v>394</v>
+        <v>384</v>
       </c>
       <c r="C22" s="6" t="s">
+        <v>376</v>
+      </c>
+      <c r="D22" s="6" t="s">
+        <v>385</v>
+      </c>
+      <c r="E22" s="6" t="s">
         <v>386</v>
       </c>
-      <c r="D22" s="6" t="s">
-        <v>395</v>
-      </c>
-      <c r="E22" s="6" t="s">
-        <v>396</v>
-      </c>
       <c r="F22" s="6" t="s">
-        <v>151</v>
+        <v>142</v>
       </c>
     </row>
     <row r="23" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B23" s="6" t="s">
-        <v>398</v>
+        <v>388</v>
       </c>
       <c r="C23" s="6">
         <v>100</v>
       </c>
       <c r="D23" s="6" t="s">
-        <v>399</v>
+        <v>389</v>
       </c>
       <c r="E23" s="6" t="s">
-        <v>397</v>
+        <v>387</v>
       </c>
       <c r="F23" s="6" t="s">
-        <v>400</v>
+        <v>390</v>
       </c>
     </row>
     <row r="24" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B24" s="6" t="s">
-        <v>362</v>
+        <v>352</v>
       </c>
       <c r="C24" s="6">
         <v>10</v>
       </c>
       <c r="D24" s="6" t="s">
-        <v>363</v>
+        <v>353</v>
       </c>
       <c r="E24" s="6" t="s">
-        <v>364</v>
+        <v>354</v>
       </c>
       <c r="F24" s="6" t="s">
-        <v>120</v>
+        <v>113</v>
       </c>
     </row>
     <row r="25" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B25" s="6" t="s">
-        <v>401</v>
+        <v>391</v>
       </c>
       <c r="C25" s="6">
         <v>20</v>
       </c>
       <c r="D25" s="6" t="s">
-        <v>402</v>
+        <v>392</v>
       </c>
       <c r="E25" s="6" t="s">
-        <v>404</v>
+        <v>394</v>
       </c>
       <c r="F25" s="6" t="s">
-        <v>403</v>
+        <v>393</v>
       </c>
     </row>
     <row r="26" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B26" s="6" t="s">
-        <v>405</v>
+        <v>395</v>
       </c>
       <c r="C26" s="6">
         <v>1000</v>
       </c>
       <c r="D26" s="6" t="s">
-        <v>406</v>
+        <v>396</v>
       </c>
       <c r="E26" s="6" t="s">
-        <v>408</v>
+        <v>398</v>
       </c>
       <c r="F26" s="6" t="s">
-        <v>407</v>
+        <v>397</v>
       </c>
     </row>
     <row r="27" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B27" s="6" t="s">
-        <v>410</v>
+        <v>400</v>
       </c>
       <c r="C27" s="6">
         <v>200</v>
       </c>
       <c r="D27" s="6" t="s">
-        <v>409</v>
+        <v>399</v>
       </c>
       <c r="E27" s="6" t="s">
-        <v>411</v>
+        <v>401</v>
       </c>
       <c r="F27" s="6" t="s">
-        <v>413</v>
+        <v>403</v>
       </c>
     </row>
     <row r="28" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B28" s="6" t="s">
-        <v>412</v>
+        <v>402</v>
       </c>
       <c r="C28" s="6">
         <v>10</v>
       </c>
       <c r="D28" s="6" t="s">
-        <v>414</v>
+        <v>404</v>
       </c>
       <c r="E28" s="6" t="s">
-        <v>415</v>
+        <v>405</v>
       </c>
       <c r="F28" s="6" t="s">
-        <v>199</v>
+        <v>189</v>
       </c>
     </row>
     <row r="29" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B29" s="6" t="s">
-        <v>416</v>
+        <v>406</v>
       </c>
       <c r="C29" s="6">
         <v>35</v>
       </c>
       <c r="D29" s="6" t="s">
-        <v>419</v>
+        <v>409</v>
       </c>
       <c r="E29" s="6" t="s">
-        <v>421</v>
+        <v>411</v>
       </c>
       <c r="F29" s="6" t="s">
-        <v>420</v>
+        <v>410</v>
       </c>
     </row>
     <row r="30" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B30" s="6" t="s">
-        <v>425</v>
+        <v>415</v>
       </c>
       <c r="C30" s="6">
         <v>80</v>
       </c>
       <c r="D30" s="6" t="s">
-        <v>422</v>
+        <v>412</v>
       </c>
       <c r="E30" s="6" t="s">
-        <v>423</v>
+        <v>413</v>
       </c>
       <c r="F30" s="6" t="s">
-        <v>424</v>
+        <v>414</v>
       </c>
     </row>
     <row r="31" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B31" s="6" t="s">
-        <v>417</v>
+        <v>407</v>
       </c>
       <c r="C31" s="6">
         <v>20</v>
       </c>
       <c r="D31" s="6" t="s">
-        <v>426</v>
+        <v>416</v>
       </c>
       <c r="E31" s="6" t="s">
-        <v>427</v>
+        <v>417</v>
       </c>
       <c r="F31" s="6" t="s">
-        <v>428</v>
+        <v>418</v>
       </c>
     </row>
     <row r="32" spans="2:6" ht="58" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B32" s="6" t="s">
-        <v>418</v>
+        <v>408</v>
       </c>
       <c r="C32" s="6">
         <v>40</v>
       </c>
       <c r="D32" s="6" t="s">
-        <v>430</v>
+        <v>420</v>
       </c>
       <c r="E32" s="6" t="s">
-        <v>431</v>
+        <v>421</v>
       </c>
       <c r="F32" s="6" t="s">
-        <v>429</v>
+        <v>419</v>
       </c>
     </row>
     <row r="33" spans="2:7" ht="58" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B33" s="6" t="s">
-        <v>433</v>
+        <v>423</v>
       </c>
       <c r="C33" s="6">
         <v>104</v>
       </c>
       <c r="D33" s="6" t="s">
-        <v>436</v>
+        <v>426</v>
       </c>
       <c r="E33" s="6" t="s">
-        <v>435</v>
+        <v>425</v>
       </c>
       <c r="F33" s="6" t="s">
-        <v>432</v>
+        <v>422</v>
       </c>
     </row>
     <row r="34" spans="2:7" ht="58" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B34" s="6" t="s">
-        <v>559</v>
+        <v>548</v>
       </c>
       <c r="C34" s="6">
         <v>200</v>
       </c>
       <c r="D34" s="6" t="s">
-        <v>560</v>
+        <v>549</v>
       </c>
       <c r="E34" s="6" t="s">
-        <v>561</v>
+        <v>550</v>
       </c>
       <c r="F34" s="6" t="s">
-        <v>558</v>
+        <v>547</v>
       </c>
     </row>
     <row r="35" spans="2:7" ht="58" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B35" s="6" t="s">
-        <v>616</v>
+        <v>605</v>
       </c>
       <c r="C35" s="6">
         <v>50</v>
       </c>
       <c r="D35" s="6" t="s">
-        <v>619</v>
+        <v>608</v>
       </c>
       <c r="E35" s="6" t="s">
-        <v>617</v>
+        <v>606</v>
       </c>
       <c r="F35" s="6" t="s">
-        <v>618</v>
+        <v>607</v>
       </c>
     </row>
     <row r="36" spans="2:7" ht="58" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B36" s="14" t="s">
-        <v>641</v>
+        <v>630</v>
       </c>
       <c r="C36" s="6">
         <v>10</v>
       </c>
       <c r="D36" s="15" t="s">
-        <v>642</v>
+        <v>631</v>
       </c>
       <c r="E36" s="6" t="s">
-        <v>643</v>
+        <v>632</v>
       </c>
       <c r="F36" s="6" t="s">
-        <v>644</v>
+        <v>633</v>
       </c>
       <c r="G36" s="13"/>
     </row>
@@ -5356,143 +5323,143 @@
         <v>7</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>148</v>
+        <v>139</v>
       </c>
     </row>
     <row r="3" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B3" s="3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>143</v>
+        <v>134</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>139</v>
+        <v>130</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>177</v>
+        <v>167</v>
       </c>
     </row>
     <row r="4" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>143</v>
+        <v>134</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>144</v>
+        <v>135</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>140</v>
+        <v>131</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>174</v>
+        <v>164</v>
       </c>
     </row>
     <row r="5" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="3" t="s">
-        <v>142</v>
+        <v>133</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>143</v>
+        <v>134</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>145</v>
+        <v>136</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>141</v>
+        <v>132</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>175</v>
+        <v>165</v>
       </c>
     </row>
     <row r="6" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="3" t="s">
-        <v>298</v>
+        <v>288</v>
       </c>
       <c r="C6" s="3">
         <v>40</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>299</v>
+        <v>289</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>300</v>
+        <v>290</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>301</v>
+        <v>291</v>
       </c>
     </row>
     <row r="7" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B7" s="3" t="s">
-        <v>338</v>
+        <v>328</v>
       </c>
       <c r="C7" s="3">
         <v>50</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>339</v>
+        <v>329</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>341</v>
+        <v>331</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>340</v>
+        <v>330</v>
       </c>
     </row>
     <row r="8" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B8" s="3" t="s">
-        <v>373</v>
+        <v>363</v>
       </c>
       <c r="C8" s="3">
         <v>300</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>376</v>
+        <v>366</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>374</v>
+        <v>364</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>375</v>
+        <v>365</v>
       </c>
     </row>
     <row r="9" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B9" s="3" t="s">
-        <v>577</v>
+        <v>566</v>
       </c>
       <c r="C9" s="3">
         <v>5</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>578</v>
+        <v>567</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>579</v>
+        <v>568</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>199</v>
+        <v>189</v>
       </c>
     </row>
     <row r="10" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="3" t="s">
-        <v>584</v>
+        <v>573</v>
       </c>
       <c r="C10" s="3">
         <v>15</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>585</v>
+        <v>574</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>586</v>
+        <v>575</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>587</v>
+        <v>576</v>
       </c>
     </row>
     <row r="11" spans="2:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.25"/>

</xml_diff>